<commit_message>
Carga de la Mercería: lanas e hilos por ovillo y por gramo (existencia en gramos)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U9SAsfVct6L94yoocG63si
</commit_message>
<xml_diff>
--- a/herramientas/merceria-carga/plantilla_carga_merceria.xlsx
+++ b/herramientas/merceria-carga/plantilla_carga_merceria.xlsx
@@ -524,7 +524,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2. Para cada producto que vas a tener en la tienda, escribe la cantidad comprada y el costo de compra por unidad (lo que pagaste, con IVA).</t>
+          <t>2. Para cada producto que vas a tener en la tienda, escribe la cantidad comprada (ovillos o unidades) y el costo de compra de cada ovillo o unidad (lo que pagaste, con IVA).</t>
         </is>
       </c>
     </row>
@@ -569,21 +569,21 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>• Por unidad: el cliente compra el ovillo, paquete o pieza completa (lo normal en una mercería).</t>
+          <t>• Por ovillo y por gramo (lanas e hilos): en la caja se vende el ovillo completo o los gramos que pida el cliente. Escribe cuántos ovillos compraste y el costo de cada ovillo; el sistema guarda la existencia en gramos usando el peso del ovillo.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>• Por gramo: se pesa y se cobra por gramo (como se hace hoy en el Taller).</t>
+          <t>• Por unidad: agujas, herrajes, tijeras, paquetes de relleno, etc. Se vende la pieza completa.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Hoy el ERP tiene las lanas con precio por gramo y algunas marcadas por unidad: esta columna lo deja en orden.</t>
+          <t>Para las lanas y los hilos es obligatorio el peso por ovillo (columna "Peso por unidad (g)").</t>
         </is>
       </c>
     </row>
@@ -716,12 +716,12 @@
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
-          <t>Cantidad comprada</t>
+          <t>Cantidad comprada (ovillos o unidades)</t>
         </is>
       </c>
       <c r="L1" s="4" t="inlineStr">
         <is>
-          <t>Costo de compra por unidad (COP)</t>
+          <t>Costo de compra por ovillo o por unidad (COP)</t>
         </is>
       </c>
       <c r="M1" s="4" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J2" s="6" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>Por unidad</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>Por unidad</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>Por unidad</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
@@ -1240,7 +1240,7 @@
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
@@ -1303,7 +1303,7 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>Por unidad</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>Por unidad</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>Por unidad</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J15" s="6" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>Por unidad</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J20" s="6" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J21" s="6" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J24" s="6" t="inlineStr">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
@@ -2437,7 +2437,7 @@
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J33" s="6" t="inlineStr">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
@@ -2878,7 +2878,7 @@
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
@@ -3790,7 +3790,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Por unidad</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -3812,7 +3812,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por unidad</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>

<commit_message>
Carga de la Mercería: lanas e hilos por ovillo y por gramo (existencia en gramos) (#179)
Claude-Session: https://claude.ai/code/session_01U9SAsfVct6L94yoocG63si

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/herramientas/merceria-carga/plantilla_carga_merceria.xlsx
+++ b/herramientas/merceria-carga/plantilla_carga_merceria.xlsx
@@ -524,7 +524,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2. Para cada producto que vas a tener en la tienda, escribe la cantidad comprada y el costo de compra por unidad (lo que pagaste, con IVA).</t>
+          <t>2. Para cada producto que vas a tener en la tienda, escribe la cantidad comprada (ovillos o unidades) y el costo de compra de cada ovillo o unidad (lo que pagaste, con IVA).</t>
         </is>
       </c>
     </row>
@@ -569,21 +569,21 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>• Por unidad: el cliente compra el ovillo, paquete o pieza completa (lo normal en una mercería).</t>
+          <t>• Por ovillo y por gramo (lanas e hilos): en la caja se vende el ovillo completo o los gramos que pida el cliente. Escribe cuántos ovillos compraste y el costo de cada ovillo; el sistema guarda la existencia en gramos usando el peso del ovillo.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>• Por gramo: se pesa y se cobra por gramo (como se hace hoy en el Taller).</t>
+          <t>• Por unidad: agujas, herrajes, tijeras, paquetes de relleno, etc. Se vende la pieza completa.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Hoy el ERP tiene las lanas con precio por gramo y algunas marcadas por unidad: esta columna lo deja en orden.</t>
+          <t>Para las lanas y los hilos es obligatorio el peso por ovillo (columna "Peso por unidad (g)").</t>
         </is>
       </c>
     </row>
@@ -716,12 +716,12 @@
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
-          <t>Cantidad comprada</t>
+          <t>Cantidad comprada (ovillos o unidades)</t>
         </is>
       </c>
       <c r="L1" s="4" t="inlineStr">
         <is>
-          <t>Costo de compra por unidad (COP)</t>
+          <t>Costo de compra por ovillo o por unidad (COP)</t>
         </is>
       </c>
       <c r="M1" s="4" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J2" s="6" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>Por unidad</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>Por unidad</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>Por unidad</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
@@ -1240,7 +1240,7 @@
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
@@ -1303,7 +1303,7 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>Por unidad</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>Por unidad</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>Por unidad</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J15" s="6" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>Por unidad</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J20" s="6" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J21" s="6" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J24" s="6" t="inlineStr">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
@@ -2437,7 +2437,7 @@
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J33" s="6" t="inlineStr">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
@@ -2878,7 +2878,7 @@
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
@@ -3790,7 +3790,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Por unidad</t>
+          <t>Por ovillo y por gramo</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -3812,7 +3812,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Por gramo</t>
+          <t>Por unidad</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>

<commit_message>
Plantilla de carga de la Mercería: regla Taller/Tienda, hoja Resumen, revisión automática y más filas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U9SAsfVct6L94yoocG63si
</commit_message>
<xml_diff>
--- a/herramientas/merceria-carga/plantilla_carga_merceria.xlsx
+++ b/herramientas/merceria-carga/plantilla_carga_merceria.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Productos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Listas" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Productos'!$A$1:$S$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Productos'!$A$1:$S$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,10 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="165" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +58,17 @@
     <font>
       <color rgb="008A8A8F"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00B00020"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="5">
@@ -98,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -119,10 +132,44 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00B00020"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FDE2E2"/>
+          <bgColor rgb="00FDE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="002E7D32"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -484,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -504,127 +551,176 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>IMPORTANTE: esta plantilla es SOLO para lo que se VENDE en la Mercería (el inventario de la TIENDA). Lo que usas para tejer (lanas, relleno, ojos… del inventario del TALLER) NO va aquí.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Si dudas de un producto, pregúntate: ¿lo va a comprar una clienta en la tienda? Si sí, va aquí; si es para tejer, no.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Cómo llenarla</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>1. Hoja "Productos": las primeras 34 filas son los productos que ya existen en el ERP. No cambies la columna ID.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>2. Para cada producto que vas a tener en la tienda, escribe la cantidad comprada (ovillos o unidades) y el costo de compra de cada ovillo o unidad (lo que pagaste, con IVA).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>3. Si un producto ya no lo vas a vender, escribe "No" en la columna "¿Se vende en la tienda?".</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>4. Los productos nuevos (agujas, herrajes, accesorios, relleno, tijeras, etc.) van en las filas vacías de abajo, sin ID.</t>
+          <t>1. Hoja "Productos": las primeras 34 filas son los productos que ya existen en el ERP. No cambies la columna ID.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>5. Proveedor, factura y fecha de compra: llénalos si los tienes; sirven para el Kardex y para la contabilidad.</t>
+          <t>2. Para cada producto que vas a tener en la tienda, escribe la cantidad comprada (ovillos o unidades) y el costo de compra de cada ovillo o unidad (lo que pagaste, con IVA).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>6. Código de barras: si el producto lo trae, escríbelo (o escanéalo con un lector); así se encuentra rápido en el POS.</t>
+          <t>3. Si un producto ya no lo vas a vender, escribe "No" en la columna "¿Se vende en la tienda?".</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>4. Los productos nuevos (agujas, herrajes, accesorios, relleno, tijeras, etc.) van en las filas vacías de abajo, sin ID.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Columna "¿Cómo se vende?"</t>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>5. Proveedor, factura y fecha de compra: llénalos si los tienes; sirven para el Kardex y para la contabilidad.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>6. Código de barras: si el producto lo trae, escríbelo (o escanéalo con un lector); así se encuentra rápido en el POS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Columna "¿Cómo se vende?"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>• Por ovillo y por gramo (lanas e hilos): en la caja se vende el ovillo completo o los gramos que pida el cliente. Escribe cuántos ovillos compraste y el costo de cada ovillo; el sistema guarda la existencia en gramos usando el peso del ovillo.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>• Por unidad: agujas, herrajes, tijeras, paquetes de relleno, etc. Se vende la pieza completa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Para las lanas y los hilos es obligatorio el peso por ovillo (columna "Peso por unidad (g)").</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>El precio de venta no hace falta</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>Para las lanas y los hilos es obligatorio el peso por ovillo (columna "Peso por unidad (g)").</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>El precio de venta no hace falta</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>Claude lo calcula con la regla de la Mercería del ERP: costo × (1 + carga de costos fijos) ÷ (1 − 40 % de utilidad), redondeado a los $100.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>La columna "Precio de venta hoy" es solo de referencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Cuando termines</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>La columna "Precio de venta hoy" es solo de referencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Cuando termines</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t>Envía el archivo a Claude. Claude crea los productos nuevos, registra las entradas con su costo (como "Entrada de nueva mercancía" del ERP), calcula los precios y te muestra un resumen antes de dejarlo listo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>Para no equivocarte (ayudas nuevas, 22-oct-2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>• La columna T de "Productos" ("Revisión") te avisa en rojo si a una fila le falta el costo, el peso del ovillo o la categoría. Déjala vacía antes de enviar el archivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>• La hoja "Resumen" cuenta cuántos productos llevan cantidad, cuántos ovillos/unidades y cuánto vale la mercancía (cantidad × costo). Ese valor es el que necesita el contador para el saldo de apertura.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>• Ejemplo de una lana: Cantidad comprada = 10 (ovillos), Costo por ovillo = 7.500, Peso por unidad = 160. El sistema guarda 1.600 g a $46,88 el gramo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>• Ejemplo de una aguja: Cantidad = 24, Costo por unidad = 1.800, "¿Cómo se vende?" = Por unidad.</t>
         </is>
       </c>
     </row>
@@ -639,7 +735,105 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S75"/>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Resumen de la carga (se calcula solo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Productos con cantidad comprada</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>COUNTIFS(Productos!K2:K150,"&gt;0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ovillos o unidades compradas (suma)</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>SUM(Productos!K2:K150)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Valor de la mercancía a costo (COP)</t>
+        </is>
+      </c>
+      <c r="B5" s="16">
+        <f>SUMPRODUCT(Productos!K2:K150,Productos!L2:L150)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Productos nuevos (sin ID) por crear</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>COUNTIFS(Productos!A2:A150,"",Productos!C2:C150,"&lt;&gt;")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Filas con algo por corregir</t>
+        </is>
+      </c>
+      <c r="B7" s="17">
+        <f>COUNTIF(Productos!T2:T150,"Falta*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Productos marcados "No se vende"</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>COUNTIF(Productos!J2:J150,"No")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Si "Filas con algo por corregir" no es 0, revisa la columna T de la hoja Productos antes de enviar el archivo.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -661,6 +855,7 @@
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
     <col width="30" customWidth="1" min="19" max="19"/>
+    <col width="34" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1">
@@ -757,6 +952,11 @@
       <c r="S1" s="4" t="inlineStr">
         <is>
           <t>Notas</t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>Revisión (automática, no tocar)</t>
         </is>
       </c>
     </row>
@@ -822,6 +1022,10 @@
         </is>
       </c>
       <c r="S2" s="6" t="n"/>
+      <c r="T2">
+        <f>IF(C2="","",IF(AND(K2&lt;&gt;"",L2=""),"Falta el costo",IF(AND(LEFT(I2,6)="Por ov",K2&lt;&gt;"",G2=""),"Falta el peso del ovillo",IF(AND(A2="",B2=""),"Falta la categoría",IF(AND(A2="",I2=""),"Falta cómo se vende",IF(AND(K2&lt;&gt;"",N2="",M2=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -885,6 +1089,10 @@
         </is>
       </c>
       <c r="S3" s="6" t="n"/>
+      <c r="T3">
+        <f>IF(C3="","",IF(AND(K3&lt;&gt;"",L3=""),"Falta el costo",IF(AND(LEFT(I3,6)="Por ov",K3&lt;&gt;"",G3=""),"Falta el peso del ovillo",IF(AND(A3="",B3=""),"Falta la categoría",IF(AND(A3="",I3=""),"Falta cómo se vende",IF(AND(K3&lt;&gt;"",N3="",M3=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -948,6 +1156,10 @@
         </is>
       </c>
       <c r="S4" s="6" t="n"/>
+      <c r="T4">
+        <f>IF(C4="","",IF(AND(K4&lt;&gt;"",L4=""),"Falta el costo",IF(AND(LEFT(I4,6)="Por ov",K4&lt;&gt;"",G4=""),"Falta el peso del ovillo",IF(AND(A4="",B4=""),"Falta la categoría",IF(AND(A4="",I4=""),"Falta cómo se vende",IF(AND(K4&lt;&gt;"",N4="",M4=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -1011,6 +1223,10 @@
         </is>
       </c>
       <c r="S5" s="6" t="n"/>
+      <c r="T5">
+        <f>IF(C5="","",IF(AND(K5&lt;&gt;"",L5=""),"Falta el costo",IF(AND(LEFT(I5,6)="Por ov",K5&lt;&gt;"",G5=""),"Falta el peso del ovillo",IF(AND(A5="",B5=""),"Falta la categoría",IF(AND(A5="",I5=""),"Falta cómo se vende",IF(AND(K5&lt;&gt;"",N5="",M5=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1074,6 +1290,10 @@
         </is>
       </c>
       <c r="S6" s="6" t="n"/>
+      <c r="T6">
+        <f>IF(C6="","",IF(AND(K6&lt;&gt;"",L6=""),"Falta el costo",IF(AND(LEFT(I6,6)="Por ov",K6&lt;&gt;"",G6=""),"Falta el peso del ovillo",IF(AND(A6="",B6=""),"Falta la categoría",IF(AND(A6="",I6=""),"Falta cómo se vende",IF(AND(K6&lt;&gt;"",N6="",M6=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1137,6 +1357,10 @@
         </is>
       </c>
       <c r="S7" s="6" t="n"/>
+      <c r="T7">
+        <f>IF(C7="","",IF(AND(K7&lt;&gt;"",L7=""),"Falta el costo",IF(AND(LEFT(I7,6)="Por ov",K7&lt;&gt;"",G7=""),"Falta el peso del ovillo",IF(AND(A7="",B7=""),"Falta la categoría",IF(AND(A7="",I7=""),"Falta cómo se vende",IF(AND(K7&lt;&gt;"",N7="",M7=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1200,6 +1424,10 @@
         </is>
       </c>
       <c r="S8" s="6" t="n"/>
+      <c r="T8">
+        <f>IF(C8="","",IF(AND(K8&lt;&gt;"",L8=""),"Falta el costo",IF(AND(LEFT(I8,6)="Por ov",K8&lt;&gt;"",G8=""),"Falta el peso del ovillo",IF(AND(A8="",B8=""),"Falta la categoría",IF(AND(A8="",I8=""),"Falta cómo se vende",IF(AND(K8&lt;&gt;"",N8="",M8=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1263,6 +1491,10 @@
         </is>
       </c>
       <c r="S9" s="6" t="n"/>
+      <c r="T9">
+        <f>IF(C9="","",IF(AND(K9&lt;&gt;"",L9=""),"Falta el costo",IF(AND(LEFT(I9,6)="Por ov",K9&lt;&gt;"",G9=""),"Falta el peso del ovillo",IF(AND(A9="",B9=""),"Falta la categoría",IF(AND(A9="",I9=""),"Falta cómo se vende",IF(AND(K9&lt;&gt;"",N9="",M9=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1326,6 +1558,10 @@
         </is>
       </c>
       <c r="S10" s="6" t="n"/>
+      <c r="T10">
+        <f>IF(C10="","",IF(AND(K10&lt;&gt;"",L10=""),"Falta el costo",IF(AND(LEFT(I10,6)="Por ov",K10&lt;&gt;"",G10=""),"Falta el peso del ovillo",IF(AND(A10="",B10=""),"Falta la categoría",IF(AND(A10="",I10=""),"Falta cómo se vende",IF(AND(K10&lt;&gt;"",N10="",M10=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1389,6 +1625,10 @@
         </is>
       </c>
       <c r="S11" s="6" t="n"/>
+      <c r="T11">
+        <f>IF(C11="","",IF(AND(K11&lt;&gt;"",L11=""),"Falta el costo",IF(AND(LEFT(I11,6)="Por ov",K11&lt;&gt;"",G11=""),"Falta el peso del ovillo",IF(AND(A11="",B11=""),"Falta la categoría",IF(AND(A11="",I11=""),"Falta cómo se vende",IF(AND(K11&lt;&gt;"",N11="",M11=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1452,6 +1692,10 @@
         </is>
       </c>
       <c r="S12" s="6" t="n"/>
+      <c r="T12">
+        <f>IF(C12="","",IF(AND(K12&lt;&gt;"",L12=""),"Falta el costo",IF(AND(LEFT(I12,6)="Por ov",K12&lt;&gt;"",G12=""),"Falta el peso del ovillo",IF(AND(A12="",B12=""),"Falta la categoría",IF(AND(A12="",I12=""),"Falta cómo se vende",IF(AND(K12&lt;&gt;"",N12="",M12=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1515,6 +1759,10 @@
         </is>
       </c>
       <c r="S13" s="6" t="n"/>
+      <c r="T13">
+        <f>IF(C13="","",IF(AND(K13&lt;&gt;"",L13=""),"Falta el costo",IF(AND(LEFT(I13,6)="Por ov",K13&lt;&gt;"",G13=""),"Falta el peso del ovillo",IF(AND(A13="",B13=""),"Falta la categoría",IF(AND(A13="",I13=""),"Falta cómo se vende",IF(AND(K13&lt;&gt;"",N13="",M13=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1578,6 +1826,10 @@
         </is>
       </c>
       <c r="S14" s="6" t="n"/>
+      <c r="T14">
+        <f>IF(C14="","",IF(AND(K14&lt;&gt;"",L14=""),"Falta el costo",IF(AND(LEFT(I14,6)="Por ov",K14&lt;&gt;"",G14=""),"Falta el peso del ovillo",IF(AND(A14="",B14=""),"Falta la categoría",IF(AND(A14="",I14=""),"Falta cómo se vende",IF(AND(K14&lt;&gt;"",N14="",M14=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1641,6 +1893,10 @@
         </is>
       </c>
       <c r="S15" s="6" t="n"/>
+      <c r="T15">
+        <f>IF(C15="","",IF(AND(K15&lt;&gt;"",L15=""),"Falta el costo",IF(AND(LEFT(I15,6)="Por ov",K15&lt;&gt;"",G15=""),"Falta el peso del ovillo",IF(AND(A15="",B15=""),"Falta la categoría",IF(AND(A15="",I15=""),"Falta cómo se vende",IF(AND(K15&lt;&gt;"",N15="",M15=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1704,6 +1960,10 @@
         </is>
       </c>
       <c r="S16" s="6" t="n"/>
+      <c r="T16">
+        <f>IF(C16="","",IF(AND(K16&lt;&gt;"",L16=""),"Falta el costo",IF(AND(LEFT(I16,6)="Por ov",K16&lt;&gt;"",G16=""),"Falta el peso del ovillo",IF(AND(A16="",B16=""),"Falta la categoría",IF(AND(A16="",I16=""),"Falta cómo se vende",IF(AND(K16&lt;&gt;"",N16="",M16=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1767,6 +2027,10 @@
         </is>
       </c>
       <c r="S17" s="6" t="n"/>
+      <c r="T17">
+        <f>IF(C17="","",IF(AND(K17&lt;&gt;"",L17=""),"Falta el costo",IF(AND(LEFT(I17,6)="Por ov",K17&lt;&gt;"",G17=""),"Falta el peso del ovillo",IF(AND(A17="",B17=""),"Falta la categoría",IF(AND(A17="",I17=""),"Falta cómo se vende",IF(AND(K17&lt;&gt;"",N17="",M17=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1830,6 +2094,10 @@
         </is>
       </c>
       <c r="S18" s="6" t="n"/>
+      <c r="T18">
+        <f>IF(C18="","",IF(AND(K18&lt;&gt;"",L18=""),"Falta el costo",IF(AND(LEFT(I18,6)="Por ov",K18&lt;&gt;"",G18=""),"Falta el peso del ovillo",IF(AND(A18="",B18=""),"Falta la categoría",IF(AND(A18="",I18=""),"Falta cómo se vende",IF(AND(K18&lt;&gt;"",N18="",M18=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1893,6 +2161,10 @@
         </is>
       </c>
       <c r="S19" s="6" t="n"/>
+      <c r="T19">
+        <f>IF(C19="","",IF(AND(K19&lt;&gt;"",L19=""),"Falta el costo",IF(AND(LEFT(I19,6)="Por ov",K19&lt;&gt;"",G19=""),"Falta el peso del ovillo",IF(AND(A19="",B19=""),"Falta la categoría",IF(AND(A19="",I19=""),"Falta cómo se vende",IF(AND(K19&lt;&gt;"",N19="",M19=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1956,6 +2228,10 @@
         </is>
       </c>
       <c r="S20" s="6" t="n"/>
+      <c r="T20">
+        <f>IF(C20="","",IF(AND(K20&lt;&gt;"",L20=""),"Falta el costo",IF(AND(LEFT(I20,6)="Por ov",K20&lt;&gt;"",G20=""),"Falta el peso del ovillo",IF(AND(A20="",B20=""),"Falta la categoría",IF(AND(A20="",I20=""),"Falta cómo se vende",IF(AND(K20&lt;&gt;"",N20="",M20=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -2019,6 +2295,10 @@
         </is>
       </c>
       <c r="S21" s="6" t="n"/>
+      <c r="T21">
+        <f>IF(C21="","",IF(AND(K21&lt;&gt;"",L21=""),"Falta el costo",IF(AND(LEFT(I21,6)="Por ov",K21&lt;&gt;"",G21=""),"Falta el peso del ovillo",IF(AND(A21="",B21=""),"Falta la categoría",IF(AND(A21="",I21=""),"Falta cómo se vende",IF(AND(K21&lt;&gt;"",N21="",M21=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -2082,6 +2362,10 @@
         </is>
       </c>
       <c r="S22" s="6" t="n"/>
+      <c r="T22">
+        <f>IF(C22="","",IF(AND(K22&lt;&gt;"",L22=""),"Falta el costo",IF(AND(LEFT(I22,6)="Por ov",K22&lt;&gt;"",G22=""),"Falta el peso del ovillo",IF(AND(A22="",B22=""),"Falta la categoría",IF(AND(A22="",I22=""),"Falta cómo se vende",IF(AND(K22&lt;&gt;"",N22="",M22=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -2145,6 +2429,10 @@
         </is>
       </c>
       <c r="S23" s="6" t="n"/>
+      <c r="T23">
+        <f>IF(C23="","",IF(AND(K23&lt;&gt;"",L23=""),"Falta el costo",IF(AND(LEFT(I23,6)="Por ov",K23&lt;&gt;"",G23=""),"Falta el peso del ovillo",IF(AND(A23="",B23=""),"Falta la categoría",IF(AND(A23="",I23=""),"Falta cómo se vende",IF(AND(K23&lt;&gt;"",N23="",M23=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -2208,6 +2496,10 @@
         </is>
       </c>
       <c r="S24" s="6" t="n"/>
+      <c r="T24">
+        <f>IF(C24="","",IF(AND(K24&lt;&gt;"",L24=""),"Falta el costo",IF(AND(LEFT(I24,6)="Por ov",K24&lt;&gt;"",G24=""),"Falta el peso del ovillo",IF(AND(A24="",B24=""),"Falta la categoría",IF(AND(A24="",I24=""),"Falta cómo se vende",IF(AND(K24&lt;&gt;"",N24="",M24=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -2271,6 +2563,10 @@
         </is>
       </c>
       <c r="S25" s="6" t="n"/>
+      <c r="T25">
+        <f>IF(C25="","",IF(AND(K25&lt;&gt;"",L25=""),"Falta el costo",IF(AND(LEFT(I25,6)="Por ov",K25&lt;&gt;"",G25=""),"Falta el peso del ovillo",IF(AND(A25="",B25=""),"Falta la categoría",IF(AND(A25="",I25=""),"Falta cómo se vende",IF(AND(K25&lt;&gt;"",N25="",M25=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -2334,6 +2630,10 @@
         </is>
       </c>
       <c r="S26" s="6" t="n"/>
+      <c r="T26">
+        <f>IF(C26="","",IF(AND(K26&lt;&gt;"",L26=""),"Falta el costo",IF(AND(LEFT(I26,6)="Por ov",K26&lt;&gt;"",G26=""),"Falta el peso del ovillo",IF(AND(A26="",B26=""),"Falta la categoría",IF(AND(A26="",I26=""),"Falta cómo se vende",IF(AND(K26&lt;&gt;"",N26="",M26=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -2397,6 +2697,10 @@
         </is>
       </c>
       <c r="S27" s="6" t="n"/>
+      <c r="T27">
+        <f>IF(C27="","",IF(AND(K27&lt;&gt;"",L27=""),"Falta el costo",IF(AND(LEFT(I27,6)="Por ov",K27&lt;&gt;"",G27=""),"Falta el peso del ovillo",IF(AND(A27="",B27=""),"Falta la categoría",IF(AND(A27="",I27=""),"Falta cómo se vende",IF(AND(K27&lt;&gt;"",N27="",M27=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -2460,6 +2764,10 @@
         </is>
       </c>
       <c r="S28" s="6" t="n"/>
+      <c r="T28">
+        <f>IF(C28="","",IF(AND(K28&lt;&gt;"",L28=""),"Falta el costo",IF(AND(LEFT(I28,6)="Por ov",K28&lt;&gt;"",G28=""),"Falta el peso del ovillo",IF(AND(A28="",B28=""),"Falta la categoría",IF(AND(A28="",I28=""),"Falta cómo se vende",IF(AND(K28&lt;&gt;"",N28="",M28=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -2523,6 +2831,10 @@
         </is>
       </c>
       <c r="S29" s="6" t="n"/>
+      <c r="T29">
+        <f>IF(C29="","",IF(AND(K29&lt;&gt;"",L29=""),"Falta el costo",IF(AND(LEFT(I29,6)="Por ov",K29&lt;&gt;"",G29=""),"Falta el peso del ovillo",IF(AND(A29="",B29=""),"Falta la categoría",IF(AND(A29="",I29=""),"Falta cómo se vende",IF(AND(K29&lt;&gt;"",N29="",M29=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -2586,6 +2898,10 @@
         </is>
       </c>
       <c r="S30" s="6" t="n"/>
+      <c r="T30">
+        <f>IF(C30="","",IF(AND(K30&lt;&gt;"",L30=""),"Falta el costo",IF(AND(LEFT(I30,6)="Por ov",K30&lt;&gt;"",G30=""),"Falta el peso del ovillo",IF(AND(A30="",B30=""),"Falta la categoría",IF(AND(A30="",I30=""),"Falta cómo se vende",IF(AND(K30&lt;&gt;"",N30="",M30=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -2649,6 +2965,10 @@
         </is>
       </c>
       <c r="S31" s="6" t="n"/>
+      <c r="T31">
+        <f>IF(C31="","",IF(AND(K31&lt;&gt;"",L31=""),"Falta el costo",IF(AND(LEFT(I31,6)="Por ov",K31&lt;&gt;"",G31=""),"Falta el peso del ovillo",IF(AND(A31="",B31=""),"Falta la categoría",IF(AND(A31="",I31=""),"Falta cómo se vende",IF(AND(K31&lt;&gt;"",N31="",M31=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -2712,6 +3032,10 @@
         </is>
       </c>
       <c r="S32" s="6" t="n"/>
+      <c r="T32">
+        <f>IF(C32="","",IF(AND(K32&lt;&gt;"",L32=""),"Falta el costo",IF(AND(LEFT(I32,6)="Por ov",K32&lt;&gt;"",G32=""),"Falta el peso del ovillo",IF(AND(A32="",B32=""),"Falta la categoría",IF(AND(A32="",I32=""),"Falta cómo se vende",IF(AND(K32&lt;&gt;"",N32="",M32=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -2775,6 +3099,10 @@
         </is>
       </c>
       <c r="S33" s="6" t="n"/>
+      <c r="T33">
+        <f>IF(C33="","",IF(AND(K33&lt;&gt;"",L33=""),"Falta el costo",IF(AND(LEFT(I33,6)="Por ov",K33&lt;&gt;"",G33=""),"Falta el peso del ovillo",IF(AND(A33="",B33=""),"Falta la categoría",IF(AND(A33="",I33=""),"Falta cómo se vende",IF(AND(K33&lt;&gt;"",N33="",M33=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -2838,6 +3166,10 @@
         </is>
       </c>
       <c r="S34" s="6" t="n"/>
+      <c r="T34">
+        <f>IF(C34="","",IF(AND(K34&lt;&gt;"",L34=""),"Falta el costo",IF(AND(LEFT(I34,6)="Por ov",K34&lt;&gt;"",G34=""),"Falta el peso del ovillo",IF(AND(A34="",B34=""),"Falta la categoría",IF(AND(A34="",I34=""),"Falta cómo se vende",IF(AND(K34&lt;&gt;"",N34="",M34=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -2901,6 +3233,10 @@
         </is>
       </c>
       <c r="S35" s="6" t="n"/>
+      <c r="T35">
+        <f>IF(C35="","",IF(AND(K35&lt;&gt;"",L35=""),"Falta el costo",IF(AND(LEFT(I35,6)="Por ov",K35&lt;&gt;"",G35=""),"Falta el peso del ovillo",IF(AND(A35="",B35=""),"Falta la categoría",IF(AND(A35="",I35=""),"Falta cómo se vende",IF(AND(K35&lt;&gt;"",N35="",M35=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n"/>
@@ -2922,6 +3258,10 @@
       <c r="Q36" s="6" t="n"/>
       <c r="R36" s="6" t="n"/>
       <c r="S36" s="6" t="n"/>
+      <c r="T36">
+        <f>IF(C36="","",IF(AND(K36&lt;&gt;"",L36=""),"Falta el costo",IF(AND(LEFT(I36,6)="Por ov",K36&lt;&gt;"",G36=""),"Falta el peso del ovillo",IF(AND(A36="",B36=""),"Falta la categoría",IF(AND(A36="",I36=""),"Falta cómo se vende",IF(AND(K36&lt;&gt;"",N36="",M36=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n"/>
@@ -2943,6 +3283,10 @@
       <c r="Q37" s="6" t="n"/>
       <c r="R37" s="6" t="n"/>
       <c r="S37" s="6" t="n"/>
+      <c r="T37">
+        <f>IF(C37="","",IF(AND(K37&lt;&gt;"",L37=""),"Falta el costo",IF(AND(LEFT(I37,6)="Por ov",K37&lt;&gt;"",G37=""),"Falta el peso del ovillo",IF(AND(A37="",B37=""),"Falta la categoría",IF(AND(A37="",I37=""),"Falta cómo se vende",IF(AND(K37&lt;&gt;"",N37="",M37=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="n"/>
@@ -2964,6 +3308,10 @@
       <c r="Q38" s="6" t="n"/>
       <c r="R38" s="6" t="n"/>
       <c r="S38" s="6" t="n"/>
+      <c r="T38">
+        <f>IF(C38="","",IF(AND(K38&lt;&gt;"",L38=""),"Falta el costo",IF(AND(LEFT(I38,6)="Por ov",K38&lt;&gt;"",G38=""),"Falta el peso del ovillo",IF(AND(A38="",B38=""),"Falta la categoría",IF(AND(A38="",I38=""),"Falta cómo se vende",IF(AND(K38&lt;&gt;"",N38="",M38=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="11" t="n"/>
@@ -2985,6 +3333,10 @@
       <c r="Q39" s="6" t="n"/>
       <c r="R39" s="6" t="n"/>
       <c r="S39" s="6" t="n"/>
+      <c r="T39">
+        <f>IF(C39="","",IF(AND(K39&lt;&gt;"",L39=""),"Falta el costo",IF(AND(LEFT(I39,6)="Por ov",K39&lt;&gt;"",G39=""),"Falta el peso del ovillo",IF(AND(A39="",B39=""),"Falta la categoría",IF(AND(A39="",I39=""),"Falta cómo se vende",IF(AND(K39&lt;&gt;"",N39="",M39=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="11" t="n"/>
@@ -3006,6 +3358,10 @@
       <c r="Q40" s="6" t="n"/>
       <c r="R40" s="6" t="n"/>
       <c r="S40" s="6" t="n"/>
+      <c r="T40">
+        <f>IF(C40="","",IF(AND(K40&lt;&gt;"",L40=""),"Falta el costo",IF(AND(LEFT(I40,6)="Por ov",K40&lt;&gt;"",G40=""),"Falta el peso del ovillo",IF(AND(A40="",B40=""),"Falta la categoría",IF(AND(A40="",I40=""),"Falta cómo se vende",IF(AND(K40&lt;&gt;"",N40="",M40=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="11" t="n"/>
@@ -3027,6 +3383,10 @@
       <c r="Q41" s="6" t="n"/>
       <c r="R41" s="6" t="n"/>
       <c r="S41" s="6" t="n"/>
+      <c r="T41">
+        <f>IF(C41="","",IF(AND(K41&lt;&gt;"",L41=""),"Falta el costo",IF(AND(LEFT(I41,6)="Por ov",K41&lt;&gt;"",G41=""),"Falta el peso del ovillo",IF(AND(A41="",B41=""),"Falta la categoría",IF(AND(A41="",I41=""),"Falta cómo se vende",IF(AND(K41&lt;&gt;"",N41="",M41=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="11" t="n"/>
@@ -3048,6 +3408,10 @@
       <c r="Q42" s="6" t="n"/>
       <c r="R42" s="6" t="n"/>
       <c r="S42" s="6" t="n"/>
+      <c r="T42">
+        <f>IF(C42="","",IF(AND(K42&lt;&gt;"",L42=""),"Falta el costo",IF(AND(LEFT(I42,6)="Por ov",K42&lt;&gt;"",G42=""),"Falta el peso del ovillo",IF(AND(A42="",B42=""),"Falta la categoría",IF(AND(A42="",I42=""),"Falta cómo se vende",IF(AND(K42&lt;&gt;"",N42="",M42=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="11" t="n"/>
@@ -3069,6 +3433,10 @@
       <c r="Q43" s="6" t="n"/>
       <c r="R43" s="6" t="n"/>
       <c r="S43" s="6" t="n"/>
+      <c r="T43">
+        <f>IF(C43="","",IF(AND(K43&lt;&gt;"",L43=""),"Falta el costo",IF(AND(LEFT(I43,6)="Por ov",K43&lt;&gt;"",G43=""),"Falta el peso del ovillo",IF(AND(A43="",B43=""),"Falta la categoría",IF(AND(A43="",I43=""),"Falta cómo se vende",IF(AND(K43&lt;&gt;"",N43="",M43=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="11" t="n"/>
@@ -3090,6 +3458,10 @@
       <c r="Q44" s="6" t="n"/>
       <c r="R44" s="6" t="n"/>
       <c r="S44" s="6" t="n"/>
+      <c r="T44">
+        <f>IF(C44="","",IF(AND(K44&lt;&gt;"",L44=""),"Falta el costo",IF(AND(LEFT(I44,6)="Por ov",K44&lt;&gt;"",G44=""),"Falta el peso del ovillo",IF(AND(A44="",B44=""),"Falta la categoría",IF(AND(A44="",I44=""),"Falta cómo se vende",IF(AND(K44&lt;&gt;"",N44="",M44=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="11" t="n"/>
@@ -3111,6 +3483,10 @@
       <c r="Q45" s="6" t="n"/>
       <c r="R45" s="6" t="n"/>
       <c r="S45" s="6" t="n"/>
+      <c r="T45">
+        <f>IF(C45="","",IF(AND(K45&lt;&gt;"",L45=""),"Falta el costo",IF(AND(LEFT(I45,6)="Por ov",K45&lt;&gt;"",G45=""),"Falta el peso del ovillo",IF(AND(A45="",B45=""),"Falta la categoría",IF(AND(A45="",I45=""),"Falta cómo se vende",IF(AND(K45&lt;&gt;"",N45="",M45=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="11" t="n"/>
@@ -3132,6 +3508,10 @@
       <c r="Q46" s="6" t="n"/>
       <c r="R46" s="6" t="n"/>
       <c r="S46" s="6" t="n"/>
+      <c r="T46">
+        <f>IF(C46="","",IF(AND(K46&lt;&gt;"",L46=""),"Falta el costo",IF(AND(LEFT(I46,6)="Por ov",K46&lt;&gt;"",G46=""),"Falta el peso del ovillo",IF(AND(A46="",B46=""),"Falta la categoría",IF(AND(A46="",I46=""),"Falta cómo se vende",IF(AND(K46&lt;&gt;"",N46="",M46=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="11" t="n"/>
@@ -3153,6 +3533,10 @@
       <c r="Q47" s="6" t="n"/>
       <c r="R47" s="6" t="n"/>
       <c r="S47" s="6" t="n"/>
+      <c r="T47">
+        <f>IF(C47="","",IF(AND(K47&lt;&gt;"",L47=""),"Falta el costo",IF(AND(LEFT(I47,6)="Por ov",K47&lt;&gt;"",G47=""),"Falta el peso del ovillo",IF(AND(A47="",B47=""),"Falta la categoría",IF(AND(A47="",I47=""),"Falta cómo se vende",IF(AND(K47&lt;&gt;"",N47="",M47=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="11" t="n"/>
@@ -3174,6 +3558,10 @@
       <c r="Q48" s="6" t="n"/>
       <c r="R48" s="6" t="n"/>
       <c r="S48" s="6" t="n"/>
+      <c r="T48">
+        <f>IF(C48="","",IF(AND(K48&lt;&gt;"",L48=""),"Falta el costo",IF(AND(LEFT(I48,6)="Por ov",K48&lt;&gt;"",G48=""),"Falta el peso del ovillo",IF(AND(A48="",B48=""),"Falta la categoría",IF(AND(A48="",I48=""),"Falta cómo se vende",IF(AND(K48&lt;&gt;"",N48="",M48=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="11" t="n"/>
@@ -3195,6 +3583,10 @@
       <c r="Q49" s="6" t="n"/>
       <c r="R49" s="6" t="n"/>
       <c r="S49" s="6" t="n"/>
+      <c r="T49">
+        <f>IF(C49="","",IF(AND(K49&lt;&gt;"",L49=""),"Falta el costo",IF(AND(LEFT(I49,6)="Por ov",K49&lt;&gt;"",G49=""),"Falta el peso del ovillo",IF(AND(A49="",B49=""),"Falta la categoría",IF(AND(A49="",I49=""),"Falta cómo se vende",IF(AND(K49&lt;&gt;"",N49="",M49=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="11" t="n"/>
@@ -3216,6 +3608,10 @@
       <c r="Q50" s="6" t="n"/>
       <c r="R50" s="6" t="n"/>
       <c r="S50" s="6" t="n"/>
+      <c r="T50">
+        <f>IF(C50="","",IF(AND(K50&lt;&gt;"",L50=""),"Falta el costo",IF(AND(LEFT(I50,6)="Por ov",K50&lt;&gt;"",G50=""),"Falta el peso del ovillo",IF(AND(A50="",B50=""),"Falta la categoría",IF(AND(A50="",I50=""),"Falta cómo se vende",IF(AND(K50&lt;&gt;"",N50="",M50=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="11" t="n"/>
@@ -3237,6 +3633,10 @@
       <c r="Q51" s="6" t="n"/>
       <c r="R51" s="6" t="n"/>
       <c r="S51" s="6" t="n"/>
+      <c r="T51">
+        <f>IF(C51="","",IF(AND(K51&lt;&gt;"",L51=""),"Falta el costo",IF(AND(LEFT(I51,6)="Por ov",K51&lt;&gt;"",G51=""),"Falta el peso del ovillo",IF(AND(A51="",B51=""),"Falta la categoría",IF(AND(A51="",I51=""),"Falta cómo se vende",IF(AND(K51&lt;&gt;"",N51="",M51=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="11" t="n"/>
@@ -3258,6 +3658,10 @@
       <c r="Q52" s="6" t="n"/>
       <c r="R52" s="6" t="n"/>
       <c r="S52" s="6" t="n"/>
+      <c r="T52">
+        <f>IF(C52="","",IF(AND(K52&lt;&gt;"",L52=""),"Falta el costo",IF(AND(LEFT(I52,6)="Por ov",K52&lt;&gt;"",G52=""),"Falta el peso del ovillo",IF(AND(A52="",B52=""),"Falta la categoría",IF(AND(A52="",I52=""),"Falta cómo se vende",IF(AND(K52&lt;&gt;"",N52="",M52=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n"/>
@@ -3279,6 +3683,10 @@
       <c r="Q53" s="6" t="n"/>
       <c r="R53" s="6" t="n"/>
       <c r="S53" s="6" t="n"/>
+      <c r="T53">
+        <f>IF(C53="","",IF(AND(K53&lt;&gt;"",L53=""),"Falta el costo",IF(AND(LEFT(I53,6)="Por ov",K53&lt;&gt;"",G53=""),"Falta el peso del ovillo",IF(AND(A53="",B53=""),"Falta la categoría",IF(AND(A53="",I53=""),"Falta cómo se vende",IF(AND(K53&lt;&gt;"",N53="",M53=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="11" t="n"/>
@@ -3300,6 +3708,10 @@
       <c r="Q54" s="6" t="n"/>
       <c r="R54" s="6" t="n"/>
       <c r="S54" s="6" t="n"/>
+      <c r="T54">
+        <f>IF(C54="","",IF(AND(K54&lt;&gt;"",L54=""),"Falta el costo",IF(AND(LEFT(I54,6)="Por ov",K54&lt;&gt;"",G54=""),"Falta el peso del ovillo",IF(AND(A54="",B54=""),"Falta la categoría",IF(AND(A54="",I54=""),"Falta cómo se vende",IF(AND(K54&lt;&gt;"",N54="",M54=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n"/>
@@ -3321,6 +3733,10 @@
       <c r="Q55" s="6" t="n"/>
       <c r="R55" s="6" t="n"/>
       <c r="S55" s="6" t="n"/>
+      <c r="T55">
+        <f>IF(C55="","",IF(AND(K55&lt;&gt;"",L55=""),"Falta el costo",IF(AND(LEFT(I55,6)="Por ov",K55&lt;&gt;"",G55=""),"Falta el peso del ovillo",IF(AND(A55="",B55=""),"Falta la categoría",IF(AND(A55="",I55=""),"Falta cómo se vende",IF(AND(K55&lt;&gt;"",N55="",M55=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n"/>
@@ -3342,6 +3758,10 @@
       <c r="Q56" s="6" t="n"/>
       <c r="R56" s="6" t="n"/>
       <c r="S56" s="6" t="n"/>
+      <c r="T56">
+        <f>IF(C56="","",IF(AND(K56&lt;&gt;"",L56=""),"Falta el costo",IF(AND(LEFT(I56,6)="Por ov",K56&lt;&gt;"",G56=""),"Falta el peso del ovillo",IF(AND(A56="",B56=""),"Falta la categoría",IF(AND(A56="",I56=""),"Falta cómo se vende",IF(AND(K56&lt;&gt;"",N56="",M56=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n"/>
@@ -3363,6 +3783,10 @@
       <c r="Q57" s="6" t="n"/>
       <c r="R57" s="6" t="n"/>
       <c r="S57" s="6" t="n"/>
+      <c r="T57">
+        <f>IF(C57="","",IF(AND(K57&lt;&gt;"",L57=""),"Falta el costo",IF(AND(LEFT(I57,6)="Por ov",K57&lt;&gt;"",G57=""),"Falta el peso del ovillo",IF(AND(A57="",B57=""),"Falta la categoría",IF(AND(A57="",I57=""),"Falta cómo se vende",IF(AND(K57&lt;&gt;"",N57="",M57=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n"/>
@@ -3384,6 +3808,10 @@
       <c r="Q58" s="6" t="n"/>
       <c r="R58" s="6" t="n"/>
       <c r="S58" s="6" t="n"/>
+      <c r="T58">
+        <f>IF(C58="","",IF(AND(K58&lt;&gt;"",L58=""),"Falta el costo",IF(AND(LEFT(I58,6)="Por ov",K58&lt;&gt;"",G58=""),"Falta el peso del ovillo",IF(AND(A58="",B58=""),"Falta la categoría",IF(AND(A58="",I58=""),"Falta cómo se vende",IF(AND(K58&lt;&gt;"",N58="",M58=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="11" t="n"/>
@@ -3405,6 +3833,10 @@
       <c r="Q59" s="6" t="n"/>
       <c r="R59" s="6" t="n"/>
       <c r="S59" s="6" t="n"/>
+      <c r="T59">
+        <f>IF(C59="","",IF(AND(K59&lt;&gt;"",L59=""),"Falta el costo",IF(AND(LEFT(I59,6)="Por ov",K59&lt;&gt;"",G59=""),"Falta el peso del ovillo",IF(AND(A59="",B59=""),"Falta la categoría",IF(AND(A59="",I59=""),"Falta cómo se vende",IF(AND(K59&lt;&gt;"",N59="",M59=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n"/>
@@ -3426,6 +3858,10 @@
       <c r="Q60" s="6" t="n"/>
       <c r="R60" s="6" t="n"/>
       <c r="S60" s="6" t="n"/>
+      <c r="T60">
+        <f>IF(C60="","",IF(AND(K60&lt;&gt;"",L60=""),"Falta el costo",IF(AND(LEFT(I60,6)="Por ov",K60&lt;&gt;"",G60=""),"Falta el peso del ovillo",IF(AND(A60="",B60=""),"Falta la categoría",IF(AND(A60="",I60=""),"Falta cómo se vende",IF(AND(K60&lt;&gt;"",N60="",M60=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n"/>
@@ -3447,6 +3883,10 @@
       <c r="Q61" s="6" t="n"/>
       <c r="R61" s="6" t="n"/>
       <c r="S61" s="6" t="n"/>
+      <c r="T61">
+        <f>IF(C61="","",IF(AND(K61&lt;&gt;"",L61=""),"Falta el costo",IF(AND(LEFT(I61,6)="Por ov",K61&lt;&gt;"",G61=""),"Falta el peso del ovillo",IF(AND(A61="",B61=""),"Falta la categoría",IF(AND(A61="",I61=""),"Falta cómo se vende",IF(AND(K61&lt;&gt;"",N61="",M61=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n"/>
@@ -3468,6 +3908,10 @@
       <c r="Q62" s="6" t="n"/>
       <c r="R62" s="6" t="n"/>
       <c r="S62" s="6" t="n"/>
+      <c r="T62">
+        <f>IF(C62="","",IF(AND(K62&lt;&gt;"",L62=""),"Falta el costo",IF(AND(LEFT(I62,6)="Por ov",K62&lt;&gt;"",G62=""),"Falta el peso del ovillo",IF(AND(A62="",B62=""),"Falta la categoría",IF(AND(A62="",I62=""),"Falta cómo se vende",IF(AND(K62&lt;&gt;"",N62="",M62=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n"/>
@@ -3489,6 +3933,10 @@
       <c r="Q63" s="6" t="n"/>
       <c r="R63" s="6" t="n"/>
       <c r="S63" s="6" t="n"/>
+      <c r="T63">
+        <f>IF(C63="","",IF(AND(K63&lt;&gt;"",L63=""),"Falta el costo",IF(AND(LEFT(I63,6)="Por ov",K63&lt;&gt;"",G63=""),"Falta el peso del ovillo",IF(AND(A63="",B63=""),"Falta la categoría",IF(AND(A63="",I63=""),"Falta cómo se vende",IF(AND(K63&lt;&gt;"",N63="",M63=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="11" t="n"/>
@@ -3510,6 +3958,10 @@
       <c r="Q64" s="6" t="n"/>
       <c r="R64" s="6" t="n"/>
       <c r="S64" s="6" t="n"/>
+      <c r="T64">
+        <f>IF(C64="","",IF(AND(K64&lt;&gt;"",L64=""),"Falta el costo",IF(AND(LEFT(I64,6)="Por ov",K64&lt;&gt;"",G64=""),"Falta el peso del ovillo",IF(AND(A64="",B64=""),"Falta la categoría",IF(AND(A64="",I64=""),"Falta cómo se vende",IF(AND(K64&lt;&gt;"",N64="",M64=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="11" t="n"/>
@@ -3531,6 +3983,10 @@
       <c r="Q65" s="6" t="n"/>
       <c r="R65" s="6" t="n"/>
       <c r="S65" s="6" t="n"/>
+      <c r="T65">
+        <f>IF(C65="","",IF(AND(K65&lt;&gt;"",L65=""),"Falta el costo",IF(AND(LEFT(I65,6)="Por ov",K65&lt;&gt;"",G65=""),"Falta el peso del ovillo",IF(AND(A65="",B65=""),"Falta la categoría",IF(AND(A65="",I65=""),"Falta cómo se vende",IF(AND(K65&lt;&gt;"",N65="",M65=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="11" t="n"/>
@@ -3552,6 +4008,10 @@
       <c r="Q66" s="6" t="n"/>
       <c r="R66" s="6" t="n"/>
       <c r="S66" s="6" t="n"/>
+      <c r="T66">
+        <f>IF(C66="","",IF(AND(K66&lt;&gt;"",L66=""),"Falta el costo",IF(AND(LEFT(I66,6)="Por ov",K66&lt;&gt;"",G66=""),"Falta el peso del ovillo",IF(AND(A66="",B66=""),"Falta la categoría",IF(AND(A66="",I66=""),"Falta cómo se vende",IF(AND(K66&lt;&gt;"",N66="",M66=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="11" t="n"/>
@@ -3573,6 +4033,10 @@
       <c r="Q67" s="6" t="n"/>
       <c r="R67" s="6" t="n"/>
       <c r="S67" s="6" t="n"/>
+      <c r="T67">
+        <f>IF(C67="","",IF(AND(K67&lt;&gt;"",L67=""),"Falta el costo",IF(AND(LEFT(I67,6)="Por ov",K67&lt;&gt;"",G67=""),"Falta el peso del ovillo",IF(AND(A67="",B67=""),"Falta la categoría",IF(AND(A67="",I67=""),"Falta cómo se vende",IF(AND(K67&lt;&gt;"",N67="",M67=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="11" t="n"/>
@@ -3594,6 +4058,10 @@
       <c r="Q68" s="6" t="n"/>
       <c r="R68" s="6" t="n"/>
       <c r="S68" s="6" t="n"/>
+      <c r="T68">
+        <f>IF(C68="","",IF(AND(K68&lt;&gt;"",L68=""),"Falta el costo",IF(AND(LEFT(I68,6)="Por ov",K68&lt;&gt;"",G68=""),"Falta el peso del ovillo",IF(AND(A68="",B68=""),"Falta la categoría",IF(AND(A68="",I68=""),"Falta cómo se vende",IF(AND(K68&lt;&gt;"",N68="",M68=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="11" t="n"/>
@@ -3615,6 +4083,10 @@
       <c r="Q69" s="6" t="n"/>
       <c r="R69" s="6" t="n"/>
       <c r="S69" s="6" t="n"/>
+      <c r="T69">
+        <f>IF(C69="","",IF(AND(K69&lt;&gt;"",L69=""),"Falta el costo",IF(AND(LEFT(I69,6)="Por ov",K69&lt;&gt;"",G69=""),"Falta el peso del ovillo",IF(AND(A69="",B69=""),"Falta la categoría",IF(AND(A69="",I69=""),"Falta cómo se vende",IF(AND(K69&lt;&gt;"",N69="",M69=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="11" t="n"/>
@@ -3636,6 +4108,10 @@
       <c r="Q70" s="6" t="n"/>
       <c r="R70" s="6" t="n"/>
       <c r="S70" s="6" t="n"/>
+      <c r="T70">
+        <f>IF(C70="","",IF(AND(K70&lt;&gt;"",L70=""),"Falta el costo",IF(AND(LEFT(I70,6)="Por ov",K70&lt;&gt;"",G70=""),"Falta el peso del ovillo",IF(AND(A70="",B70=""),"Falta la categoría",IF(AND(A70="",I70=""),"Falta cómo se vende",IF(AND(K70&lt;&gt;"",N70="",M70=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="11" t="n"/>
@@ -3657,6 +4133,10 @@
       <c r="Q71" s="6" t="n"/>
       <c r="R71" s="6" t="n"/>
       <c r="S71" s="6" t="n"/>
+      <c r="T71">
+        <f>IF(C71="","",IF(AND(K71&lt;&gt;"",L71=""),"Falta el costo",IF(AND(LEFT(I71,6)="Por ov",K71&lt;&gt;"",G71=""),"Falta el peso del ovillo",IF(AND(A71="",B71=""),"Falta la categoría",IF(AND(A71="",I71=""),"Falta cómo se vende",IF(AND(K71&lt;&gt;"",N71="",M71=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="11" t="n"/>
@@ -3678,6 +4158,10 @@
       <c r="Q72" s="6" t="n"/>
       <c r="R72" s="6" t="n"/>
       <c r="S72" s="6" t="n"/>
+      <c r="T72">
+        <f>IF(C72="","",IF(AND(K72&lt;&gt;"",L72=""),"Falta el costo",IF(AND(LEFT(I72,6)="Por ov",K72&lt;&gt;"",G72=""),"Falta el peso del ovillo",IF(AND(A72="",B72=""),"Falta la categoría",IF(AND(A72="",I72=""),"Falta cómo se vende",IF(AND(K72&lt;&gt;"",N72="",M72=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="11" t="n"/>
@@ -3699,6 +4183,10 @@
       <c r="Q73" s="6" t="n"/>
       <c r="R73" s="6" t="n"/>
       <c r="S73" s="6" t="n"/>
+      <c r="T73">
+        <f>IF(C73="","",IF(AND(K73&lt;&gt;"",L73=""),"Falta el costo",IF(AND(LEFT(I73,6)="Por ov",K73&lt;&gt;"",G73=""),"Falta el peso del ovillo",IF(AND(A73="",B73=""),"Falta la categoría",IF(AND(A73="",I73=""),"Falta cómo se vende",IF(AND(K73&lt;&gt;"",N73="",M73=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="11" t="n"/>
@@ -3720,6 +4208,10 @@
       <c r="Q74" s="6" t="n"/>
       <c r="R74" s="6" t="n"/>
       <c r="S74" s="6" t="n"/>
+      <c r="T74">
+        <f>IF(C74="","",IF(AND(K74&lt;&gt;"",L74=""),"Falta el costo",IF(AND(LEFT(I74,6)="Por ov",K74&lt;&gt;"",G74=""),"Falta el peso del ovillo",IF(AND(A74="",B74=""),"Falta la categoría",IF(AND(A74="",I74=""),"Falta cómo se vende",IF(AND(K74&lt;&gt;"",N74="",M74=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="11" t="n"/>
@@ -3741,26 +4233,1913 @@
       <c r="Q75" s="6" t="n"/>
       <c r="R75" s="6" t="n"/>
       <c r="S75" s="6" t="n"/>
+      <c r="T75">
+        <f>IF(C75="","",IF(AND(K75&lt;&gt;"",L75=""),"Falta el costo",IF(AND(LEFT(I75,6)="Por ov",K75&lt;&gt;"",G75=""),"Falta el peso del ovillo",IF(AND(A75="",B75=""),"Falta la categoría",IF(AND(A75="",I75=""),"Falta cómo se vende",IF(AND(K75&lt;&gt;"",N75="",M75=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="n"/>
+      <c r="B76" s="6" t="n"/>
+      <c r="C76" s="6" t="n"/>
+      <c r="D76" s="6" t="n"/>
+      <c r="E76" s="6" t="n"/>
+      <c r="F76" s="6" t="n"/>
+      <c r="G76" s="6" t="n"/>
+      <c r="H76" s="6" t="n"/>
+      <c r="I76" s="6" t="n"/>
+      <c r="J76" s="6" t="n"/>
+      <c r="K76" s="7" t="n"/>
+      <c r="L76" s="8" t="n"/>
+      <c r="M76" s="6" t="n"/>
+      <c r="N76" s="6" t="n"/>
+      <c r="O76" s="9" t="n"/>
+      <c r="P76" s="6" t="n"/>
+      <c r="Q76" s="6" t="n"/>
+      <c r="R76" s="6" t="n"/>
+      <c r="S76" s="6" t="n"/>
+      <c r="T76">
+        <f>IF(C76="","",IF(AND(K76&lt;&gt;"",L76=""),"Falta el costo",IF(AND(LEFT(I76,6)="Por ov",K76&lt;&gt;"",G76=""),"Falta el peso del ovillo",IF(AND(A76="",B76=""),"Falta la categoría",IF(AND(A76="",I76=""),"Falta cómo se vende",IF(AND(K76&lt;&gt;"",N76="",M76=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="11" t="n"/>
+      <c r="B77" s="6" t="n"/>
+      <c r="C77" s="6" t="n"/>
+      <c r="D77" s="6" t="n"/>
+      <c r="E77" s="6" t="n"/>
+      <c r="F77" s="6" t="n"/>
+      <c r="G77" s="6" t="n"/>
+      <c r="H77" s="6" t="n"/>
+      <c r="I77" s="6" t="n"/>
+      <c r="J77" s="6" t="n"/>
+      <c r="K77" s="7" t="n"/>
+      <c r="L77" s="8" t="n"/>
+      <c r="M77" s="6" t="n"/>
+      <c r="N77" s="6" t="n"/>
+      <c r="O77" s="9" t="n"/>
+      <c r="P77" s="6" t="n"/>
+      <c r="Q77" s="6" t="n"/>
+      <c r="R77" s="6" t="n"/>
+      <c r="S77" s="6" t="n"/>
+      <c r="T77">
+        <f>IF(C77="","",IF(AND(K77&lt;&gt;"",L77=""),"Falta el costo",IF(AND(LEFT(I77,6)="Por ov",K77&lt;&gt;"",G77=""),"Falta el peso del ovillo",IF(AND(A77="",B77=""),"Falta la categoría",IF(AND(A77="",I77=""),"Falta cómo se vende",IF(AND(K77&lt;&gt;"",N77="",M77=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="n"/>
+      <c r="B78" s="6" t="n"/>
+      <c r="C78" s="6" t="n"/>
+      <c r="D78" s="6" t="n"/>
+      <c r="E78" s="6" t="n"/>
+      <c r="F78" s="6" t="n"/>
+      <c r="G78" s="6" t="n"/>
+      <c r="H78" s="6" t="n"/>
+      <c r="I78" s="6" t="n"/>
+      <c r="J78" s="6" t="n"/>
+      <c r="K78" s="7" t="n"/>
+      <c r="L78" s="8" t="n"/>
+      <c r="M78" s="6" t="n"/>
+      <c r="N78" s="6" t="n"/>
+      <c r="O78" s="9" t="n"/>
+      <c r="P78" s="6" t="n"/>
+      <c r="Q78" s="6" t="n"/>
+      <c r="R78" s="6" t="n"/>
+      <c r="S78" s="6" t="n"/>
+      <c r="T78">
+        <f>IF(C78="","",IF(AND(K78&lt;&gt;"",L78=""),"Falta el costo",IF(AND(LEFT(I78,6)="Por ov",K78&lt;&gt;"",G78=""),"Falta el peso del ovillo",IF(AND(A78="",B78=""),"Falta la categoría",IF(AND(A78="",I78=""),"Falta cómo se vende",IF(AND(K78&lt;&gt;"",N78="",M78=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="11" t="n"/>
+      <c r="B79" s="6" t="n"/>
+      <c r="C79" s="6" t="n"/>
+      <c r="D79" s="6" t="n"/>
+      <c r="E79" s="6" t="n"/>
+      <c r="F79" s="6" t="n"/>
+      <c r="G79" s="6" t="n"/>
+      <c r="H79" s="6" t="n"/>
+      <c r="I79" s="6" t="n"/>
+      <c r="J79" s="6" t="n"/>
+      <c r="K79" s="7" t="n"/>
+      <c r="L79" s="8" t="n"/>
+      <c r="M79" s="6" t="n"/>
+      <c r="N79" s="6" t="n"/>
+      <c r="O79" s="9" t="n"/>
+      <c r="P79" s="6" t="n"/>
+      <c r="Q79" s="6" t="n"/>
+      <c r="R79" s="6" t="n"/>
+      <c r="S79" s="6" t="n"/>
+      <c r="T79">
+        <f>IF(C79="","",IF(AND(K79&lt;&gt;"",L79=""),"Falta el costo",IF(AND(LEFT(I79,6)="Por ov",K79&lt;&gt;"",G79=""),"Falta el peso del ovillo",IF(AND(A79="",B79=""),"Falta la categoría",IF(AND(A79="",I79=""),"Falta cómo se vende",IF(AND(K79&lt;&gt;"",N79="",M79=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="n"/>
+      <c r="B80" s="6" t="n"/>
+      <c r="C80" s="6" t="n"/>
+      <c r="D80" s="6" t="n"/>
+      <c r="E80" s="6" t="n"/>
+      <c r="F80" s="6" t="n"/>
+      <c r="G80" s="6" t="n"/>
+      <c r="H80" s="6" t="n"/>
+      <c r="I80" s="6" t="n"/>
+      <c r="J80" s="6" t="n"/>
+      <c r="K80" s="7" t="n"/>
+      <c r="L80" s="8" t="n"/>
+      <c r="M80" s="6" t="n"/>
+      <c r="N80" s="6" t="n"/>
+      <c r="O80" s="9" t="n"/>
+      <c r="P80" s="6" t="n"/>
+      <c r="Q80" s="6" t="n"/>
+      <c r="R80" s="6" t="n"/>
+      <c r="S80" s="6" t="n"/>
+      <c r="T80">
+        <f>IF(C80="","",IF(AND(K80&lt;&gt;"",L80=""),"Falta el costo",IF(AND(LEFT(I80,6)="Por ov",K80&lt;&gt;"",G80=""),"Falta el peso del ovillo",IF(AND(A80="",B80=""),"Falta la categoría",IF(AND(A80="",I80=""),"Falta cómo se vende",IF(AND(K80&lt;&gt;"",N80="",M80=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="11" t="n"/>
+      <c r="B81" s="6" t="n"/>
+      <c r="C81" s="6" t="n"/>
+      <c r="D81" s="6" t="n"/>
+      <c r="E81" s="6" t="n"/>
+      <c r="F81" s="6" t="n"/>
+      <c r="G81" s="6" t="n"/>
+      <c r="H81" s="6" t="n"/>
+      <c r="I81" s="6" t="n"/>
+      <c r="J81" s="6" t="n"/>
+      <c r="K81" s="7" t="n"/>
+      <c r="L81" s="8" t="n"/>
+      <c r="M81" s="6" t="n"/>
+      <c r="N81" s="6" t="n"/>
+      <c r="O81" s="9" t="n"/>
+      <c r="P81" s="6" t="n"/>
+      <c r="Q81" s="6" t="n"/>
+      <c r="R81" s="6" t="n"/>
+      <c r="S81" s="6" t="n"/>
+      <c r="T81">
+        <f>IF(C81="","",IF(AND(K81&lt;&gt;"",L81=""),"Falta el costo",IF(AND(LEFT(I81,6)="Por ov",K81&lt;&gt;"",G81=""),"Falta el peso del ovillo",IF(AND(A81="",B81=""),"Falta la categoría",IF(AND(A81="",I81=""),"Falta cómo se vende",IF(AND(K81&lt;&gt;"",N81="",M81=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="n"/>
+      <c r="B82" s="6" t="n"/>
+      <c r="C82" s="6" t="n"/>
+      <c r="D82" s="6" t="n"/>
+      <c r="E82" s="6" t="n"/>
+      <c r="F82" s="6" t="n"/>
+      <c r="G82" s="6" t="n"/>
+      <c r="H82" s="6" t="n"/>
+      <c r="I82" s="6" t="n"/>
+      <c r="J82" s="6" t="n"/>
+      <c r="K82" s="7" t="n"/>
+      <c r="L82" s="8" t="n"/>
+      <c r="M82" s="6" t="n"/>
+      <c r="N82" s="6" t="n"/>
+      <c r="O82" s="9" t="n"/>
+      <c r="P82" s="6" t="n"/>
+      <c r="Q82" s="6" t="n"/>
+      <c r="R82" s="6" t="n"/>
+      <c r="S82" s="6" t="n"/>
+      <c r="T82">
+        <f>IF(C82="","",IF(AND(K82&lt;&gt;"",L82=""),"Falta el costo",IF(AND(LEFT(I82,6)="Por ov",K82&lt;&gt;"",G82=""),"Falta el peso del ovillo",IF(AND(A82="",B82=""),"Falta la categoría",IF(AND(A82="",I82=""),"Falta cómo se vende",IF(AND(K82&lt;&gt;"",N82="",M82=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="11" t="n"/>
+      <c r="B83" s="6" t="n"/>
+      <c r="C83" s="6" t="n"/>
+      <c r="D83" s="6" t="n"/>
+      <c r="E83" s="6" t="n"/>
+      <c r="F83" s="6" t="n"/>
+      <c r="G83" s="6" t="n"/>
+      <c r="H83" s="6" t="n"/>
+      <c r="I83" s="6" t="n"/>
+      <c r="J83" s="6" t="n"/>
+      <c r="K83" s="7" t="n"/>
+      <c r="L83" s="8" t="n"/>
+      <c r="M83" s="6" t="n"/>
+      <c r="N83" s="6" t="n"/>
+      <c r="O83" s="9" t="n"/>
+      <c r="P83" s="6" t="n"/>
+      <c r="Q83" s="6" t="n"/>
+      <c r="R83" s="6" t="n"/>
+      <c r="S83" s="6" t="n"/>
+      <c r="T83">
+        <f>IF(C83="","",IF(AND(K83&lt;&gt;"",L83=""),"Falta el costo",IF(AND(LEFT(I83,6)="Por ov",K83&lt;&gt;"",G83=""),"Falta el peso del ovillo",IF(AND(A83="",B83=""),"Falta la categoría",IF(AND(A83="",I83=""),"Falta cómo se vende",IF(AND(K83&lt;&gt;"",N83="",M83=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="n"/>
+      <c r="B84" s="6" t="n"/>
+      <c r="C84" s="6" t="n"/>
+      <c r="D84" s="6" t="n"/>
+      <c r="E84" s="6" t="n"/>
+      <c r="F84" s="6" t="n"/>
+      <c r="G84" s="6" t="n"/>
+      <c r="H84" s="6" t="n"/>
+      <c r="I84" s="6" t="n"/>
+      <c r="J84" s="6" t="n"/>
+      <c r="K84" s="7" t="n"/>
+      <c r="L84" s="8" t="n"/>
+      <c r="M84" s="6" t="n"/>
+      <c r="N84" s="6" t="n"/>
+      <c r="O84" s="9" t="n"/>
+      <c r="P84" s="6" t="n"/>
+      <c r="Q84" s="6" t="n"/>
+      <c r="R84" s="6" t="n"/>
+      <c r="S84" s="6" t="n"/>
+      <c r="T84">
+        <f>IF(C84="","",IF(AND(K84&lt;&gt;"",L84=""),"Falta el costo",IF(AND(LEFT(I84,6)="Por ov",K84&lt;&gt;"",G84=""),"Falta el peso del ovillo",IF(AND(A84="",B84=""),"Falta la categoría",IF(AND(A84="",I84=""),"Falta cómo se vende",IF(AND(K84&lt;&gt;"",N84="",M84=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="11" t="n"/>
+      <c r="B85" s="6" t="n"/>
+      <c r="C85" s="6" t="n"/>
+      <c r="D85" s="6" t="n"/>
+      <c r="E85" s="6" t="n"/>
+      <c r="F85" s="6" t="n"/>
+      <c r="G85" s="6" t="n"/>
+      <c r="H85" s="6" t="n"/>
+      <c r="I85" s="6" t="n"/>
+      <c r="J85" s="6" t="n"/>
+      <c r="K85" s="7" t="n"/>
+      <c r="L85" s="8" t="n"/>
+      <c r="M85" s="6" t="n"/>
+      <c r="N85" s="6" t="n"/>
+      <c r="O85" s="9" t="n"/>
+      <c r="P85" s="6" t="n"/>
+      <c r="Q85" s="6" t="n"/>
+      <c r="R85" s="6" t="n"/>
+      <c r="S85" s="6" t="n"/>
+      <c r="T85">
+        <f>IF(C85="","",IF(AND(K85&lt;&gt;"",L85=""),"Falta el costo",IF(AND(LEFT(I85,6)="Por ov",K85&lt;&gt;"",G85=""),"Falta el peso del ovillo",IF(AND(A85="",B85=""),"Falta la categoría",IF(AND(A85="",I85=""),"Falta cómo se vende",IF(AND(K85&lt;&gt;"",N85="",M85=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="11" t="n"/>
+      <c r="B86" s="6" t="n"/>
+      <c r="C86" s="6" t="n"/>
+      <c r="D86" s="6" t="n"/>
+      <c r="E86" s="6" t="n"/>
+      <c r="F86" s="6" t="n"/>
+      <c r="G86" s="6" t="n"/>
+      <c r="H86" s="6" t="n"/>
+      <c r="I86" s="6" t="n"/>
+      <c r="J86" s="6" t="n"/>
+      <c r="K86" s="7" t="n"/>
+      <c r="L86" s="8" t="n"/>
+      <c r="M86" s="6" t="n"/>
+      <c r="N86" s="6" t="n"/>
+      <c r="O86" s="9" t="n"/>
+      <c r="P86" s="6" t="n"/>
+      <c r="Q86" s="6" t="n"/>
+      <c r="R86" s="6" t="n"/>
+      <c r="S86" s="6" t="n"/>
+      <c r="T86">
+        <f>IF(C86="","",IF(AND(K86&lt;&gt;"",L86=""),"Falta el costo",IF(AND(LEFT(I86,6)="Por ov",K86&lt;&gt;"",G86=""),"Falta el peso del ovillo",IF(AND(A86="",B86=""),"Falta la categoría",IF(AND(A86="",I86=""),"Falta cómo se vende",IF(AND(K86&lt;&gt;"",N86="",M86=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="11" t="n"/>
+      <c r="B87" s="6" t="n"/>
+      <c r="C87" s="6" t="n"/>
+      <c r="D87" s="6" t="n"/>
+      <c r="E87" s="6" t="n"/>
+      <c r="F87" s="6" t="n"/>
+      <c r="G87" s="6" t="n"/>
+      <c r="H87" s="6" t="n"/>
+      <c r="I87" s="6" t="n"/>
+      <c r="J87" s="6" t="n"/>
+      <c r="K87" s="7" t="n"/>
+      <c r="L87" s="8" t="n"/>
+      <c r="M87" s="6" t="n"/>
+      <c r="N87" s="6" t="n"/>
+      <c r="O87" s="9" t="n"/>
+      <c r="P87" s="6" t="n"/>
+      <c r="Q87" s="6" t="n"/>
+      <c r="R87" s="6" t="n"/>
+      <c r="S87" s="6" t="n"/>
+      <c r="T87">
+        <f>IF(C87="","",IF(AND(K87&lt;&gt;"",L87=""),"Falta el costo",IF(AND(LEFT(I87,6)="Por ov",K87&lt;&gt;"",G87=""),"Falta el peso del ovillo",IF(AND(A87="",B87=""),"Falta la categoría",IF(AND(A87="",I87=""),"Falta cómo se vende",IF(AND(K87&lt;&gt;"",N87="",M87=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="11" t="n"/>
+      <c r="B88" s="6" t="n"/>
+      <c r="C88" s="6" t="n"/>
+      <c r="D88" s="6" t="n"/>
+      <c r="E88" s="6" t="n"/>
+      <c r="F88" s="6" t="n"/>
+      <c r="G88" s="6" t="n"/>
+      <c r="H88" s="6" t="n"/>
+      <c r="I88" s="6" t="n"/>
+      <c r="J88" s="6" t="n"/>
+      <c r="K88" s="7" t="n"/>
+      <c r="L88" s="8" t="n"/>
+      <c r="M88" s="6" t="n"/>
+      <c r="N88" s="6" t="n"/>
+      <c r="O88" s="9" t="n"/>
+      <c r="P88" s="6" t="n"/>
+      <c r="Q88" s="6" t="n"/>
+      <c r="R88" s="6" t="n"/>
+      <c r="S88" s="6" t="n"/>
+      <c r="T88">
+        <f>IF(C88="","",IF(AND(K88&lt;&gt;"",L88=""),"Falta el costo",IF(AND(LEFT(I88,6)="Por ov",K88&lt;&gt;"",G88=""),"Falta el peso del ovillo",IF(AND(A88="",B88=""),"Falta la categoría",IF(AND(A88="",I88=""),"Falta cómo se vende",IF(AND(K88&lt;&gt;"",N88="",M88=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="11" t="n"/>
+      <c r="B89" s="6" t="n"/>
+      <c r="C89" s="6" t="n"/>
+      <c r="D89" s="6" t="n"/>
+      <c r="E89" s="6" t="n"/>
+      <c r="F89" s="6" t="n"/>
+      <c r="G89" s="6" t="n"/>
+      <c r="H89" s="6" t="n"/>
+      <c r="I89" s="6" t="n"/>
+      <c r="J89" s="6" t="n"/>
+      <c r="K89" s="7" t="n"/>
+      <c r="L89" s="8" t="n"/>
+      <c r="M89" s="6" t="n"/>
+      <c r="N89" s="6" t="n"/>
+      <c r="O89" s="9" t="n"/>
+      <c r="P89" s="6" t="n"/>
+      <c r="Q89" s="6" t="n"/>
+      <c r="R89" s="6" t="n"/>
+      <c r="S89" s="6" t="n"/>
+      <c r="T89">
+        <f>IF(C89="","",IF(AND(K89&lt;&gt;"",L89=""),"Falta el costo",IF(AND(LEFT(I89,6)="Por ov",K89&lt;&gt;"",G89=""),"Falta el peso del ovillo",IF(AND(A89="",B89=""),"Falta la categoría",IF(AND(A89="",I89=""),"Falta cómo se vende",IF(AND(K89&lt;&gt;"",N89="",M89=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="11" t="n"/>
+      <c r="B90" s="6" t="n"/>
+      <c r="C90" s="6" t="n"/>
+      <c r="D90" s="6" t="n"/>
+      <c r="E90" s="6" t="n"/>
+      <c r="F90" s="6" t="n"/>
+      <c r="G90" s="6" t="n"/>
+      <c r="H90" s="6" t="n"/>
+      <c r="I90" s="6" t="n"/>
+      <c r="J90" s="6" t="n"/>
+      <c r="K90" s="7" t="n"/>
+      <c r="L90" s="8" t="n"/>
+      <c r="M90" s="6" t="n"/>
+      <c r="N90" s="6" t="n"/>
+      <c r="O90" s="9" t="n"/>
+      <c r="P90" s="6" t="n"/>
+      <c r="Q90" s="6" t="n"/>
+      <c r="R90" s="6" t="n"/>
+      <c r="S90" s="6" t="n"/>
+      <c r="T90">
+        <f>IF(C90="","",IF(AND(K90&lt;&gt;"",L90=""),"Falta el costo",IF(AND(LEFT(I90,6)="Por ov",K90&lt;&gt;"",G90=""),"Falta el peso del ovillo",IF(AND(A90="",B90=""),"Falta la categoría",IF(AND(A90="",I90=""),"Falta cómo se vende",IF(AND(K90&lt;&gt;"",N90="",M90=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="11" t="n"/>
+      <c r="B91" s="6" t="n"/>
+      <c r="C91" s="6" t="n"/>
+      <c r="D91" s="6" t="n"/>
+      <c r="E91" s="6" t="n"/>
+      <c r="F91" s="6" t="n"/>
+      <c r="G91" s="6" t="n"/>
+      <c r="H91" s="6" t="n"/>
+      <c r="I91" s="6" t="n"/>
+      <c r="J91" s="6" t="n"/>
+      <c r="K91" s="7" t="n"/>
+      <c r="L91" s="8" t="n"/>
+      <c r="M91" s="6" t="n"/>
+      <c r="N91" s="6" t="n"/>
+      <c r="O91" s="9" t="n"/>
+      <c r="P91" s="6" t="n"/>
+      <c r="Q91" s="6" t="n"/>
+      <c r="R91" s="6" t="n"/>
+      <c r="S91" s="6" t="n"/>
+      <c r="T91">
+        <f>IF(C91="","",IF(AND(K91&lt;&gt;"",L91=""),"Falta el costo",IF(AND(LEFT(I91,6)="Por ov",K91&lt;&gt;"",G91=""),"Falta el peso del ovillo",IF(AND(A91="",B91=""),"Falta la categoría",IF(AND(A91="",I91=""),"Falta cómo se vende",IF(AND(K91&lt;&gt;"",N91="",M91=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="11" t="n"/>
+      <c r="B92" s="6" t="n"/>
+      <c r="C92" s="6" t="n"/>
+      <c r="D92" s="6" t="n"/>
+      <c r="E92" s="6" t="n"/>
+      <c r="F92" s="6" t="n"/>
+      <c r="G92" s="6" t="n"/>
+      <c r="H92" s="6" t="n"/>
+      <c r="I92" s="6" t="n"/>
+      <c r="J92" s="6" t="n"/>
+      <c r="K92" s="7" t="n"/>
+      <c r="L92" s="8" t="n"/>
+      <c r="M92" s="6" t="n"/>
+      <c r="N92" s="6" t="n"/>
+      <c r="O92" s="9" t="n"/>
+      <c r="P92" s="6" t="n"/>
+      <c r="Q92" s="6" t="n"/>
+      <c r="R92" s="6" t="n"/>
+      <c r="S92" s="6" t="n"/>
+      <c r="T92">
+        <f>IF(C92="","",IF(AND(K92&lt;&gt;"",L92=""),"Falta el costo",IF(AND(LEFT(I92,6)="Por ov",K92&lt;&gt;"",G92=""),"Falta el peso del ovillo",IF(AND(A92="",B92=""),"Falta la categoría",IF(AND(A92="",I92=""),"Falta cómo se vende",IF(AND(K92&lt;&gt;"",N92="",M92=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="11" t="n"/>
+      <c r="B93" s="6" t="n"/>
+      <c r="C93" s="6" t="n"/>
+      <c r="D93" s="6" t="n"/>
+      <c r="E93" s="6" t="n"/>
+      <c r="F93" s="6" t="n"/>
+      <c r="G93" s="6" t="n"/>
+      <c r="H93" s="6" t="n"/>
+      <c r="I93" s="6" t="n"/>
+      <c r="J93" s="6" t="n"/>
+      <c r="K93" s="7" t="n"/>
+      <c r="L93" s="8" t="n"/>
+      <c r="M93" s="6" t="n"/>
+      <c r="N93" s="6" t="n"/>
+      <c r="O93" s="9" t="n"/>
+      <c r="P93" s="6" t="n"/>
+      <c r="Q93" s="6" t="n"/>
+      <c r="R93" s="6" t="n"/>
+      <c r="S93" s="6" t="n"/>
+      <c r="T93">
+        <f>IF(C93="","",IF(AND(K93&lt;&gt;"",L93=""),"Falta el costo",IF(AND(LEFT(I93,6)="Por ov",K93&lt;&gt;"",G93=""),"Falta el peso del ovillo",IF(AND(A93="",B93=""),"Falta la categoría",IF(AND(A93="",I93=""),"Falta cómo se vende",IF(AND(K93&lt;&gt;"",N93="",M93=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="11" t="n"/>
+      <c r="B94" s="6" t="n"/>
+      <c r="C94" s="6" t="n"/>
+      <c r="D94" s="6" t="n"/>
+      <c r="E94" s="6" t="n"/>
+      <c r="F94" s="6" t="n"/>
+      <c r="G94" s="6" t="n"/>
+      <c r="H94" s="6" t="n"/>
+      <c r="I94" s="6" t="n"/>
+      <c r="J94" s="6" t="n"/>
+      <c r="K94" s="7" t="n"/>
+      <c r="L94" s="8" t="n"/>
+      <c r="M94" s="6" t="n"/>
+      <c r="N94" s="6" t="n"/>
+      <c r="O94" s="9" t="n"/>
+      <c r="P94" s="6" t="n"/>
+      <c r="Q94" s="6" t="n"/>
+      <c r="R94" s="6" t="n"/>
+      <c r="S94" s="6" t="n"/>
+      <c r="T94">
+        <f>IF(C94="","",IF(AND(K94&lt;&gt;"",L94=""),"Falta el costo",IF(AND(LEFT(I94,6)="Por ov",K94&lt;&gt;"",G94=""),"Falta el peso del ovillo",IF(AND(A94="",B94=""),"Falta la categoría",IF(AND(A94="",I94=""),"Falta cómo se vende",IF(AND(K94&lt;&gt;"",N94="",M94=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="11" t="n"/>
+      <c r="B95" s="6" t="n"/>
+      <c r="C95" s="6" t="n"/>
+      <c r="D95" s="6" t="n"/>
+      <c r="E95" s="6" t="n"/>
+      <c r="F95" s="6" t="n"/>
+      <c r="G95" s="6" t="n"/>
+      <c r="H95" s="6" t="n"/>
+      <c r="I95" s="6" t="n"/>
+      <c r="J95" s="6" t="n"/>
+      <c r="K95" s="7" t="n"/>
+      <c r="L95" s="8" t="n"/>
+      <c r="M95" s="6" t="n"/>
+      <c r="N95" s="6" t="n"/>
+      <c r="O95" s="9" t="n"/>
+      <c r="P95" s="6" t="n"/>
+      <c r="Q95" s="6" t="n"/>
+      <c r="R95" s="6" t="n"/>
+      <c r="S95" s="6" t="n"/>
+      <c r="T95">
+        <f>IF(C95="","",IF(AND(K95&lt;&gt;"",L95=""),"Falta el costo",IF(AND(LEFT(I95,6)="Por ov",K95&lt;&gt;"",G95=""),"Falta el peso del ovillo",IF(AND(A95="",B95=""),"Falta la categoría",IF(AND(A95="",I95=""),"Falta cómo se vende",IF(AND(K95&lt;&gt;"",N95="",M95=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="11" t="n"/>
+      <c r="B96" s="6" t="n"/>
+      <c r="C96" s="6" t="n"/>
+      <c r="D96" s="6" t="n"/>
+      <c r="E96" s="6" t="n"/>
+      <c r="F96" s="6" t="n"/>
+      <c r="G96" s="6" t="n"/>
+      <c r="H96" s="6" t="n"/>
+      <c r="I96" s="6" t="n"/>
+      <c r="J96" s="6" t="n"/>
+      <c r="K96" s="7" t="n"/>
+      <c r="L96" s="8" t="n"/>
+      <c r="M96" s="6" t="n"/>
+      <c r="N96" s="6" t="n"/>
+      <c r="O96" s="9" t="n"/>
+      <c r="P96" s="6" t="n"/>
+      <c r="Q96" s="6" t="n"/>
+      <c r="R96" s="6" t="n"/>
+      <c r="S96" s="6" t="n"/>
+      <c r="T96">
+        <f>IF(C96="","",IF(AND(K96&lt;&gt;"",L96=""),"Falta el costo",IF(AND(LEFT(I96,6)="Por ov",K96&lt;&gt;"",G96=""),"Falta el peso del ovillo",IF(AND(A96="",B96=""),"Falta la categoría",IF(AND(A96="",I96=""),"Falta cómo se vende",IF(AND(K96&lt;&gt;"",N96="",M96=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="11" t="n"/>
+      <c r="B97" s="6" t="n"/>
+      <c r="C97" s="6" t="n"/>
+      <c r="D97" s="6" t="n"/>
+      <c r="E97" s="6" t="n"/>
+      <c r="F97" s="6" t="n"/>
+      <c r="G97" s="6" t="n"/>
+      <c r="H97" s="6" t="n"/>
+      <c r="I97" s="6" t="n"/>
+      <c r="J97" s="6" t="n"/>
+      <c r="K97" s="7" t="n"/>
+      <c r="L97" s="8" t="n"/>
+      <c r="M97" s="6" t="n"/>
+      <c r="N97" s="6" t="n"/>
+      <c r="O97" s="9" t="n"/>
+      <c r="P97" s="6" t="n"/>
+      <c r="Q97" s="6" t="n"/>
+      <c r="R97" s="6" t="n"/>
+      <c r="S97" s="6" t="n"/>
+      <c r="T97">
+        <f>IF(C97="","",IF(AND(K97&lt;&gt;"",L97=""),"Falta el costo",IF(AND(LEFT(I97,6)="Por ov",K97&lt;&gt;"",G97=""),"Falta el peso del ovillo",IF(AND(A97="",B97=""),"Falta la categoría",IF(AND(A97="",I97=""),"Falta cómo se vende",IF(AND(K97&lt;&gt;"",N97="",M97=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="11" t="n"/>
+      <c r="B98" s="6" t="n"/>
+      <c r="C98" s="6" t="n"/>
+      <c r="D98" s="6" t="n"/>
+      <c r="E98" s="6" t="n"/>
+      <c r="F98" s="6" t="n"/>
+      <c r="G98" s="6" t="n"/>
+      <c r="H98" s="6" t="n"/>
+      <c r="I98" s="6" t="n"/>
+      <c r="J98" s="6" t="n"/>
+      <c r="K98" s="7" t="n"/>
+      <c r="L98" s="8" t="n"/>
+      <c r="M98" s="6" t="n"/>
+      <c r="N98" s="6" t="n"/>
+      <c r="O98" s="9" t="n"/>
+      <c r="P98" s="6" t="n"/>
+      <c r="Q98" s="6" t="n"/>
+      <c r="R98" s="6" t="n"/>
+      <c r="S98" s="6" t="n"/>
+      <c r="T98">
+        <f>IF(C98="","",IF(AND(K98&lt;&gt;"",L98=""),"Falta el costo",IF(AND(LEFT(I98,6)="Por ov",K98&lt;&gt;"",G98=""),"Falta el peso del ovillo",IF(AND(A98="",B98=""),"Falta la categoría",IF(AND(A98="",I98=""),"Falta cómo se vende",IF(AND(K98&lt;&gt;"",N98="",M98=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="11" t="n"/>
+      <c r="B99" s="6" t="n"/>
+      <c r="C99" s="6" t="n"/>
+      <c r="D99" s="6" t="n"/>
+      <c r="E99" s="6" t="n"/>
+      <c r="F99" s="6" t="n"/>
+      <c r="G99" s="6" t="n"/>
+      <c r="H99" s="6" t="n"/>
+      <c r="I99" s="6" t="n"/>
+      <c r="J99" s="6" t="n"/>
+      <c r="K99" s="7" t="n"/>
+      <c r="L99" s="8" t="n"/>
+      <c r="M99" s="6" t="n"/>
+      <c r="N99" s="6" t="n"/>
+      <c r="O99" s="9" t="n"/>
+      <c r="P99" s="6" t="n"/>
+      <c r="Q99" s="6" t="n"/>
+      <c r="R99" s="6" t="n"/>
+      <c r="S99" s="6" t="n"/>
+      <c r="T99">
+        <f>IF(C99="","",IF(AND(K99&lt;&gt;"",L99=""),"Falta el costo",IF(AND(LEFT(I99,6)="Por ov",K99&lt;&gt;"",G99=""),"Falta el peso del ovillo",IF(AND(A99="",B99=""),"Falta la categoría",IF(AND(A99="",I99=""),"Falta cómo se vende",IF(AND(K99&lt;&gt;"",N99="",M99=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="11" t="n"/>
+      <c r="B100" s="6" t="n"/>
+      <c r="C100" s="6" t="n"/>
+      <c r="D100" s="6" t="n"/>
+      <c r="E100" s="6" t="n"/>
+      <c r="F100" s="6" t="n"/>
+      <c r="G100" s="6" t="n"/>
+      <c r="H100" s="6" t="n"/>
+      <c r="I100" s="6" t="n"/>
+      <c r="J100" s="6" t="n"/>
+      <c r="K100" s="7" t="n"/>
+      <c r="L100" s="8" t="n"/>
+      <c r="M100" s="6" t="n"/>
+      <c r="N100" s="6" t="n"/>
+      <c r="O100" s="9" t="n"/>
+      <c r="P100" s="6" t="n"/>
+      <c r="Q100" s="6" t="n"/>
+      <c r="R100" s="6" t="n"/>
+      <c r="S100" s="6" t="n"/>
+      <c r="T100">
+        <f>IF(C100="","",IF(AND(K100&lt;&gt;"",L100=""),"Falta el costo",IF(AND(LEFT(I100,6)="Por ov",K100&lt;&gt;"",G100=""),"Falta el peso del ovillo",IF(AND(A100="",B100=""),"Falta la categoría",IF(AND(A100="",I100=""),"Falta cómo se vende",IF(AND(K100&lt;&gt;"",N100="",M100=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="11" t="n"/>
+      <c r="B101" s="6" t="n"/>
+      <c r="C101" s="6" t="n"/>
+      <c r="D101" s="6" t="n"/>
+      <c r="E101" s="6" t="n"/>
+      <c r="F101" s="6" t="n"/>
+      <c r="G101" s="6" t="n"/>
+      <c r="H101" s="6" t="n"/>
+      <c r="I101" s="6" t="n"/>
+      <c r="J101" s="6" t="n"/>
+      <c r="K101" s="7" t="n"/>
+      <c r="L101" s="8" t="n"/>
+      <c r="M101" s="6" t="n"/>
+      <c r="N101" s="6" t="n"/>
+      <c r="O101" s="9" t="n"/>
+      <c r="P101" s="6" t="n"/>
+      <c r="Q101" s="6" t="n"/>
+      <c r="R101" s="6" t="n"/>
+      <c r="S101" s="6" t="n"/>
+      <c r="T101">
+        <f>IF(C101="","",IF(AND(K101&lt;&gt;"",L101=""),"Falta el costo",IF(AND(LEFT(I101,6)="Por ov",K101&lt;&gt;"",G101=""),"Falta el peso del ovillo",IF(AND(A101="",B101=""),"Falta la categoría",IF(AND(A101="",I101=""),"Falta cómo se vende",IF(AND(K101&lt;&gt;"",N101="",M101=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="11" t="n"/>
+      <c r="B102" s="6" t="n"/>
+      <c r="C102" s="6" t="n"/>
+      <c r="D102" s="6" t="n"/>
+      <c r="E102" s="6" t="n"/>
+      <c r="F102" s="6" t="n"/>
+      <c r="G102" s="6" t="n"/>
+      <c r="H102" s="6" t="n"/>
+      <c r="I102" s="6" t="n"/>
+      <c r="J102" s="6" t="n"/>
+      <c r="K102" s="7" t="n"/>
+      <c r="L102" s="8" t="n"/>
+      <c r="M102" s="6" t="n"/>
+      <c r="N102" s="6" t="n"/>
+      <c r="O102" s="9" t="n"/>
+      <c r="P102" s="6" t="n"/>
+      <c r="Q102" s="6" t="n"/>
+      <c r="R102" s="6" t="n"/>
+      <c r="S102" s="6" t="n"/>
+      <c r="T102">
+        <f>IF(C102="","",IF(AND(K102&lt;&gt;"",L102=""),"Falta el costo",IF(AND(LEFT(I102,6)="Por ov",K102&lt;&gt;"",G102=""),"Falta el peso del ovillo",IF(AND(A102="",B102=""),"Falta la categoría",IF(AND(A102="",I102=""),"Falta cómo se vende",IF(AND(K102&lt;&gt;"",N102="",M102=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="11" t="n"/>
+      <c r="B103" s="6" t="n"/>
+      <c r="C103" s="6" t="n"/>
+      <c r="D103" s="6" t="n"/>
+      <c r="E103" s="6" t="n"/>
+      <c r="F103" s="6" t="n"/>
+      <c r="G103" s="6" t="n"/>
+      <c r="H103" s="6" t="n"/>
+      <c r="I103" s="6" t="n"/>
+      <c r="J103" s="6" t="n"/>
+      <c r="K103" s="7" t="n"/>
+      <c r="L103" s="8" t="n"/>
+      <c r="M103" s="6" t="n"/>
+      <c r="N103" s="6" t="n"/>
+      <c r="O103" s="9" t="n"/>
+      <c r="P103" s="6" t="n"/>
+      <c r="Q103" s="6" t="n"/>
+      <c r="R103" s="6" t="n"/>
+      <c r="S103" s="6" t="n"/>
+      <c r="T103">
+        <f>IF(C103="","",IF(AND(K103&lt;&gt;"",L103=""),"Falta el costo",IF(AND(LEFT(I103,6)="Por ov",K103&lt;&gt;"",G103=""),"Falta el peso del ovillo",IF(AND(A103="",B103=""),"Falta la categoría",IF(AND(A103="",I103=""),"Falta cómo se vende",IF(AND(K103&lt;&gt;"",N103="",M103=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="11" t="n"/>
+      <c r="B104" s="6" t="n"/>
+      <c r="C104" s="6" t="n"/>
+      <c r="D104" s="6" t="n"/>
+      <c r="E104" s="6" t="n"/>
+      <c r="F104" s="6" t="n"/>
+      <c r="G104" s="6" t="n"/>
+      <c r="H104" s="6" t="n"/>
+      <c r="I104" s="6" t="n"/>
+      <c r="J104" s="6" t="n"/>
+      <c r="K104" s="7" t="n"/>
+      <c r="L104" s="8" t="n"/>
+      <c r="M104" s="6" t="n"/>
+      <c r="N104" s="6" t="n"/>
+      <c r="O104" s="9" t="n"/>
+      <c r="P104" s="6" t="n"/>
+      <c r="Q104" s="6" t="n"/>
+      <c r="R104" s="6" t="n"/>
+      <c r="S104" s="6" t="n"/>
+      <c r="T104">
+        <f>IF(C104="","",IF(AND(K104&lt;&gt;"",L104=""),"Falta el costo",IF(AND(LEFT(I104,6)="Por ov",K104&lt;&gt;"",G104=""),"Falta el peso del ovillo",IF(AND(A104="",B104=""),"Falta la categoría",IF(AND(A104="",I104=""),"Falta cómo se vende",IF(AND(K104&lt;&gt;"",N104="",M104=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="11" t="n"/>
+      <c r="B105" s="6" t="n"/>
+      <c r="C105" s="6" t="n"/>
+      <c r="D105" s="6" t="n"/>
+      <c r="E105" s="6" t="n"/>
+      <c r="F105" s="6" t="n"/>
+      <c r="G105" s="6" t="n"/>
+      <c r="H105" s="6" t="n"/>
+      <c r="I105" s="6" t="n"/>
+      <c r="J105" s="6" t="n"/>
+      <c r="K105" s="7" t="n"/>
+      <c r="L105" s="8" t="n"/>
+      <c r="M105" s="6" t="n"/>
+      <c r="N105" s="6" t="n"/>
+      <c r="O105" s="9" t="n"/>
+      <c r="P105" s="6" t="n"/>
+      <c r="Q105" s="6" t="n"/>
+      <c r="R105" s="6" t="n"/>
+      <c r="S105" s="6" t="n"/>
+      <c r="T105">
+        <f>IF(C105="","",IF(AND(K105&lt;&gt;"",L105=""),"Falta el costo",IF(AND(LEFT(I105,6)="Por ov",K105&lt;&gt;"",G105=""),"Falta el peso del ovillo",IF(AND(A105="",B105=""),"Falta la categoría",IF(AND(A105="",I105=""),"Falta cómo se vende",IF(AND(K105&lt;&gt;"",N105="",M105=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="11" t="n"/>
+      <c r="B106" s="6" t="n"/>
+      <c r="C106" s="6" t="n"/>
+      <c r="D106" s="6" t="n"/>
+      <c r="E106" s="6" t="n"/>
+      <c r="F106" s="6" t="n"/>
+      <c r="G106" s="6" t="n"/>
+      <c r="H106" s="6" t="n"/>
+      <c r="I106" s="6" t="n"/>
+      <c r="J106" s="6" t="n"/>
+      <c r="K106" s="7" t="n"/>
+      <c r="L106" s="8" t="n"/>
+      <c r="M106" s="6" t="n"/>
+      <c r="N106" s="6" t="n"/>
+      <c r="O106" s="9" t="n"/>
+      <c r="P106" s="6" t="n"/>
+      <c r="Q106" s="6" t="n"/>
+      <c r="R106" s="6" t="n"/>
+      <c r="S106" s="6" t="n"/>
+      <c r="T106">
+        <f>IF(C106="","",IF(AND(K106&lt;&gt;"",L106=""),"Falta el costo",IF(AND(LEFT(I106,6)="Por ov",K106&lt;&gt;"",G106=""),"Falta el peso del ovillo",IF(AND(A106="",B106=""),"Falta la categoría",IF(AND(A106="",I106=""),"Falta cómo se vende",IF(AND(K106&lt;&gt;"",N106="",M106=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="11" t="n"/>
+      <c r="B107" s="6" t="n"/>
+      <c r="C107" s="6" t="n"/>
+      <c r="D107" s="6" t="n"/>
+      <c r="E107" s="6" t="n"/>
+      <c r="F107" s="6" t="n"/>
+      <c r="G107" s="6" t="n"/>
+      <c r="H107" s="6" t="n"/>
+      <c r="I107" s="6" t="n"/>
+      <c r="J107" s="6" t="n"/>
+      <c r="K107" s="7" t="n"/>
+      <c r="L107" s="8" t="n"/>
+      <c r="M107" s="6" t="n"/>
+      <c r="N107" s="6" t="n"/>
+      <c r="O107" s="9" t="n"/>
+      <c r="P107" s="6" t="n"/>
+      <c r="Q107" s="6" t="n"/>
+      <c r="R107" s="6" t="n"/>
+      <c r="S107" s="6" t="n"/>
+      <c r="T107">
+        <f>IF(C107="","",IF(AND(K107&lt;&gt;"",L107=""),"Falta el costo",IF(AND(LEFT(I107,6)="Por ov",K107&lt;&gt;"",G107=""),"Falta el peso del ovillo",IF(AND(A107="",B107=""),"Falta la categoría",IF(AND(A107="",I107=""),"Falta cómo se vende",IF(AND(K107&lt;&gt;"",N107="",M107=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="11" t="n"/>
+      <c r="B108" s="6" t="n"/>
+      <c r="C108" s="6" t="n"/>
+      <c r="D108" s="6" t="n"/>
+      <c r="E108" s="6" t="n"/>
+      <c r="F108" s="6" t="n"/>
+      <c r="G108" s="6" t="n"/>
+      <c r="H108" s="6" t="n"/>
+      <c r="I108" s="6" t="n"/>
+      <c r="J108" s="6" t="n"/>
+      <c r="K108" s="7" t="n"/>
+      <c r="L108" s="8" t="n"/>
+      <c r="M108" s="6" t="n"/>
+      <c r="N108" s="6" t="n"/>
+      <c r="O108" s="9" t="n"/>
+      <c r="P108" s="6" t="n"/>
+      <c r="Q108" s="6" t="n"/>
+      <c r="R108" s="6" t="n"/>
+      <c r="S108" s="6" t="n"/>
+      <c r="T108">
+        <f>IF(C108="","",IF(AND(K108&lt;&gt;"",L108=""),"Falta el costo",IF(AND(LEFT(I108,6)="Por ov",K108&lt;&gt;"",G108=""),"Falta el peso del ovillo",IF(AND(A108="",B108=""),"Falta la categoría",IF(AND(A108="",I108=""),"Falta cómo se vende",IF(AND(K108&lt;&gt;"",N108="",M108=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="11" t="n"/>
+      <c r="B109" s="6" t="n"/>
+      <c r="C109" s="6" t="n"/>
+      <c r="D109" s="6" t="n"/>
+      <c r="E109" s="6" t="n"/>
+      <c r="F109" s="6" t="n"/>
+      <c r="G109" s="6" t="n"/>
+      <c r="H109" s="6" t="n"/>
+      <c r="I109" s="6" t="n"/>
+      <c r="J109" s="6" t="n"/>
+      <c r="K109" s="7" t="n"/>
+      <c r="L109" s="8" t="n"/>
+      <c r="M109" s="6" t="n"/>
+      <c r="N109" s="6" t="n"/>
+      <c r="O109" s="9" t="n"/>
+      <c r="P109" s="6" t="n"/>
+      <c r="Q109" s="6" t="n"/>
+      <c r="R109" s="6" t="n"/>
+      <c r="S109" s="6" t="n"/>
+      <c r="T109">
+        <f>IF(C109="","",IF(AND(K109&lt;&gt;"",L109=""),"Falta el costo",IF(AND(LEFT(I109,6)="Por ov",K109&lt;&gt;"",G109=""),"Falta el peso del ovillo",IF(AND(A109="",B109=""),"Falta la categoría",IF(AND(A109="",I109=""),"Falta cómo se vende",IF(AND(K109&lt;&gt;"",N109="",M109=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="11" t="n"/>
+      <c r="B110" s="6" t="n"/>
+      <c r="C110" s="6" t="n"/>
+      <c r="D110" s="6" t="n"/>
+      <c r="E110" s="6" t="n"/>
+      <c r="F110" s="6" t="n"/>
+      <c r="G110" s="6" t="n"/>
+      <c r="H110" s="6" t="n"/>
+      <c r="I110" s="6" t="n"/>
+      <c r="J110" s="6" t="n"/>
+      <c r="K110" s="7" t="n"/>
+      <c r="L110" s="8" t="n"/>
+      <c r="M110" s="6" t="n"/>
+      <c r="N110" s="6" t="n"/>
+      <c r="O110" s="9" t="n"/>
+      <c r="P110" s="6" t="n"/>
+      <c r="Q110" s="6" t="n"/>
+      <c r="R110" s="6" t="n"/>
+      <c r="S110" s="6" t="n"/>
+      <c r="T110">
+        <f>IF(C110="","",IF(AND(K110&lt;&gt;"",L110=""),"Falta el costo",IF(AND(LEFT(I110,6)="Por ov",K110&lt;&gt;"",G110=""),"Falta el peso del ovillo",IF(AND(A110="",B110=""),"Falta la categoría",IF(AND(A110="",I110=""),"Falta cómo se vende",IF(AND(K110&lt;&gt;"",N110="",M110=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="11" t="n"/>
+      <c r="B111" s="6" t="n"/>
+      <c r="C111" s="6" t="n"/>
+      <c r="D111" s="6" t="n"/>
+      <c r="E111" s="6" t="n"/>
+      <c r="F111" s="6" t="n"/>
+      <c r="G111" s="6" t="n"/>
+      <c r="H111" s="6" t="n"/>
+      <c r="I111" s="6" t="n"/>
+      <c r="J111" s="6" t="n"/>
+      <c r="K111" s="7" t="n"/>
+      <c r="L111" s="8" t="n"/>
+      <c r="M111" s="6" t="n"/>
+      <c r="N111" s="6" t="n"/>
+      <c r="O111" s="9" t="n"/>
+      <c r="P111" s="6" t="n"/>
+      <c r="Q111" s="6" t="n"/>
+      <c r="R111" s="6" t="n"/>
+      <c r="S111" s="6" t="n"/>
+      <c r="T111">
+        <f>IF(C111="","",IF(AND(K111&lt;&gt;"",L111=""),"Falta el costo",IF(AND(LEFT(I111,6)="Por ov",K111&lt;&gt;"",G111=""),"Falta el peso del ovillo",IF(AND(A111="",B111=""),"Falta la categoría",IF(AND(A111="",I111=""),"Falta cómo se vende",IF(AND(K111&lt;&gt;"",N111="",M111=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="11" t="n"/>
+      <c r="B112" s="6" t="n"/>
+      <c r="C112" s="6" t="n"/>
+      <c r="D112" s="6" t="n"/>
+      <c r="E112" s="6" t="n"/>
+      <c r="F112" s="6" t="n"/>
+      <c r="G112" s="6" t="n"/>
+      <c r="H112" s="6" t="n"/>
+      <c r="I112" s="6" t="n"/>
+      <c r="J112" s="6" t="n"/>
+      <c r="K112" s="7" t="n"/>
+      <c r="L112" s="8" t="n"/>
+      <c r="M112" s="6" t="n"/>
+      <c r="N112" s="6" t="n"/>
+      <c r="O112" s="9" t="n"/>
+      <c r="P112" s="6" t="n"/>
+      <c r="Q112" s="6" t="n"/>
+      <c r="R112" s="6" t="n"/>
+      <c r="S112" s="6" t="n"/>
+      <c r="T112">
+        <f>IF(C112="","",IF(AND(K112&lt;&gt;"",L112=""),"Falta el costo",IF(AND(LEFT(I112,6)="Por ov",K112&lt;&gt;"",G112=""),"Falta el peso del ovillo",IF(AND(A112="",B112=""),"Falta la categoría",IF(AND(A112="",I112=""),"Falta cómo se vende",IF(AND(K112&lt;&gt;"",N112="",M112=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="11" t="n"/>
+      <c r="B113" s="6" t="n"/>
+      <c r="C113" s="6" t="n"/>
+      <c r="D113" s="6" t="n"/>
+      <c r="E113" s="6" t="n"/>
+      <c r="F113" s="6" t="n"/>
+      <c r="G113" s="6" t="n"/>
+      <c r="H113" s="6" t="n"/>
+      <c r="I113" s="6" t="n"/>
+      <c r="J113" s="6" t="n"/>
+      <c r="K113" s="7" t="n"/>
+      <c r="L113" s="8" t="n"/>
+      <c r="M113" s="6" t="n"/>
+      <c r="N113" s="6" t="n"/>
+      <c r="O113" s="9" t="n"/>
+      <c r="P113" s="6" t="n"/>
+      <c r="Q113" s="6" t="n"/>
+      <c r="R113" s="6" t="n"/>
+      <c r="S113" s="6" t="n"/>
+      <c r="T113">
+        <f>IF(C113="","",IF(AND(K113&lt;&gt;"",L113=""),"Falta el costo",IF(AND(LEFT(I113,6)="Por ov",K113&lt;&gt;"",G113=""),"Falta el peso del ovillo",IF(AND(A113="",B113=""),"Falta la categoría",IF(AND(A113="",I113=""),"Falta cómo se vende",IF(AND(K113&lt;&gt;"",N113="",M113=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="11" t="n"/>
+      <c r="B114" s="6" t="n"/>
+      <c r="C114" s="6" t="n"/>
+      <c r="D114" s="6" t="n"/>
+      <c r="E114" s="6" t="n"/>
+      <c r="F114" s="6" t="n"/>
+      <c r="G114" s="6" t="n"/>
+      <c r="H114" s="6" t="n"/>
+      <c r="I114" s="6" t="n"/>
+      <c r="J114" s="6" t="n"/>
+      <c r="K114" s="7" t="n"/>
+      <c r="L114" s="8" t="n"/>
+      <c r="M114" s="6" t="n"/>
+      <c r="N114" s="6" t="n"/>
+      <c r="O114" s="9" t="n"/>
+      <c r="P114" s="6" t="n"/>
+      <c r="Q114" s="6" t="n"/>
+      <c r="R114" s="6" t="n"/>
+      <c r="S114" s="6" t="n"/>
+      <c r="T114">
+        <f>IF(C114="","",IF(AND(K114&lt;&gt;"",L114=""),"Falta el costo",IF(AND(LEFT(I114,6)="Por ov",K114&lt;&gt;"",G114=""),"Falta el peso del ovillo",IF(AND(A114="",B114=""),"Falta la categoría",IF(AND(A114="",I114=""),"Falta cómo se vende",IF(AND(K114&lt;&gt;"",N114="",M114=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="11" t="n"/>
+      <c r="B115" s="6" t="n"/>
+      <c r="C115" s="6" t="n"/>
+      <c r="D115" s="6" t="n"/>
+      <c r="E115" s="6" t="n"/>
+      <c r="F115" s="6" t="n"/>
+      <c r="G115" s="6" t="n"/>
+      <c r="H115" s="6" t="n"/>
+      <c r="I115" s="6" t="n"/>
+      <c r="J115" s="6" t="n"/>
+      <c r="K115" s="7" t="n"/>
+      <c r="L115" s="8" t="n"/>
+      <c r="M115" s="6" t="n"/>
+      <c r="N115" s="6" t="n"/>
+      <c r="O115" s="9" t="n"/>
+      <c r="P115" s="6" t="n"/>
+      <c r="Q115" s="6" t="n"/>
+      <c r="R115" s="6" t="n"/>
+      <c r="S115" s="6" t="n"/>
+      <c r="T115">
+        <f>IF(C115="","",IF(AND(K115&lt;&gt;"",L115=""),"Falta el costo",IF(AND(LEFT(I115,6)="Por ov",K115&lt;&gt;"",G115=""),"Falta el peso del ovillo",IF(AND(A115="",B115=""),"Falta la categoría",IF(AND(A115="",I115=""),"Falta cómo se vende",IF(AND(K115&lt;&gt;"",N115="",M115=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="11" t="n"/>
+      <c r="B116" s="6" t="n"/>
+      <c r="C116" s="6" t="n"/>
+      <c r="D116" s="6" t="n"/>
+      <c r="E116" s="6" t="n"/>
+      <c r="F116" s="6" t="n"/>
+      <c r="G116" s="6" t="n"/>
+      <c r="H116" s="6" t="n"/>
+      <c r="I116" s="6" t="n"/>
+      <c r="J116" s="6" t="n"/>
+      <c r="K116" s="7" t="n"/>
+      <c r="L116" s="8" t="n"/>
+      <c r="M116" s="6" t="n"/>
+      <c r="N116" s="6" t="n"/>
+      <c r="O116" s="9" t="n"/>
+      <c r="P116" s="6" t="n"/>
+      <c r="Q116" s="6" t="n"/>
+      <c r="R116" s="6" t="n"/>
+      <c r="S116" s="6" t="n"/>
+      <c r="T116">
+        <f>IF(C116="","",IF(AND(K116&lt;&gt;"",L116=""),"Falta el costo",IF(AND(LEFT(I116,6)="Por ov",K116&lt;&gt;"",G116=""),"Falta el peso del ovillo",IF(AND(A116="",B116=""),"Falta la categoría",IF(AND(A116="",I116=""),"Falta cómo se vende",IF(AND(K116&lt;&gt;"",N116="",M116=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="11" t="n"/>
+      <c r="B117" s="6" t="n"/>
+      <c r="C117" s="6" t="n"/>
+      <c r="D117" s="6" t="n"/>
+      <c r="E117" s="6" t="n"/>
+      <c r="F117" s="6" t="n"/>
+      <c r="G117" s="6" t="n"/>
+      <c r="H117" s="6" t="n"/>
+      <c r="I117" s="6" t="n"/>
+      <c r="J117" s="6" t="n"/>
+      <c r="K117" s="7" t="n"/>
+      <c r="L117" s="8" t="n"/>
+      <c r="M117" s="6" t="n"/>
+      <c r="N117" s="6" t="n"/>
+      <c r="O117" s="9" t="n"/>
+      <c r="P117" s="6" t="n"/>
+      <c r="Q117" s="6" t="n"/>
+      <c r="R117" s="6" t="n"/>
+      <c r="S117" s="6" t="n"/>
+      <c r="T117">
+        <f>IF(C117="","",IF(AND(K117&lt;&gt;"",L117=""),"Falta el costo",IF(AND(LEFT(I117,6)="Por ov",K117&lt;&gt;"",G117=""),"Falta el peso del ovillo",IF(AND(A117="",B117=""),"Falta la categoría",IF(AND(A117="",I117=""),"Falta cómo se vende",IF(AND(K117&lt;&gt;"",N117="",M117=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="11" t="n"/>
+      <c r="B118" s="6" t="n"/>
+      <c r="C118" s="6" t="n"/>
+      <c r="D118" s="6" t="n"/>
+      <c r="E118" s="6" t="n"/>
+      <c r="F118" s="6" t="n"/>
+      <c r="G118" s="6" t="n"/>
+      <c r="H118" s="6" t="n"/>
+      <c r="I118" s="6" t="n"/>
+      <c r="J118" s="6" t="n"/>
+      <c r="K118" s="7" t="n"/>
+      <c r="L118" s="8" t="n"/>
+      <c r="M118" s="6" t="n"/>
+      <c r="N118" s="6" t="n"/>
+      <c r="O118" s="9" t="n"/>
+      <c r="P118" s="6" t="n"/>
+      <c r="Q118" s="6" t="n"/>
+      <c r="R118" s="6" t="n"/>
+      <c r="S118" s="6" t="n"/>
+      <c r="T118">
+        <f>IF(C118="","",IF(AND(K118&lt;&gt;"",L118=""),"Falta el costo",IF(AND(LEFT(I118,6)="Por ov",K118&lt;&gt;"",G118=""),"Falta el peso del ovillo",IF(AND(A118="",B118=""),"Falta la categoría",IF(AND(A118="",I118=""),"Falta cómo se vende",IF(AND(K118&lt;&gt;"",N118="",M118=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="11" t="n"/>
+      <c r="B119" s="6" t="n"/>
+      <c r="C119" s="6" t="n"/>
+      <c r="D119" s="6" t="n"/>
+      <c r="E119" s="6" t="n"/>
+      <c r="F119" s="6" t="n"/>
+      <c r="G119" s="6" t="n"/>
+      <c r="H119" s="6" t="n"/>
+      <c r="I119" s="6" t="n"/>
+      <c r="J119" s="6" t="n"/>
+      <c r="K119" s="7" t="n"/>
+      <c r="L119" s="8" t="n"/>
+      <c r="M119" s="6" t="n"/>
+      <c r="N119" s="6" t="n"/>
+      <c r="O119" s="9" t="n"/>
+      <c r="P119" s="6" t="n"/>
+      <c r="Q119" s="6" t="n"/>
+      <c r="R119" s="6" t="n"/>
+      <c r="S119" s="6" t="n"/>
+      <c r="T119">
+        <f>IF(C119="","",IF(AND(K119&lt;&gt;"",L119=""),"Falta el costo",IF(AND(LEFT(I119,6)="Por ov",K119&lt;&gt;"",G119=""),"Falta el peso del ovillo",IF(AND(A119="",B119=""),"Falta la categoría",IF(AND(A119="",I119=""),"Falta cómo se vende",IF(AND(K119&lt;&gt;"",N119="",M119=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="11" t="n"/>
+      <c r="B120" s="6" t="n"/>
+      <c r="C120" s="6" t="n"/>
+      <c r="D120" s="6" t="n"/>
+      <c r="E120" s="6" t="n"/>
+      <c r="F120" s="6" t="n"/>
+      <c r="G120" s="6" t="n"/>
+      <c r="H120" s="6" t="n"/>
+      <c r="I120" s="6" t="n"/>
+      <c r="J120" s="6" t="n"/>
+      <c r="K120" s="7" t="n"/>
+      <c r="L120" s="8" t="n"/>
+      <c r="M120" s="6" t="n"/>
+      <c r="N120" s="6" t="n"/>
+      <c r="O120" s="9" t="n"/>
+      <c r="P120" s="6" t="n"/>
+      <c r="Q120" s="6" t="n"/>
+      <c r="R120" s="6" t="n"/>
+      <c r="S120" s="6" t="n"/>
+      <c r="T120">
+        <f>IF(C120="","",IF(AND(K120&lt;&gt;"",L120=""),"Falta el costo",IF(AND(LEFT(I120,6)="Por ov",K120&lt;&gt;"",G120=""),"Falta el peso del ovillo",IF(AND(A120="",B120=""),"Falta la categoría",IF(AND(A120="",I120=""),"Falta cómo se vende",IF(AND(K120&lt;&gt;"",N120="",M120=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="11" t="n"/>
+      <c r="B121" s="6" t="n"/>
+      <c r="C121" s="6" t="n"/>
+      <c r="D121" s="6" t="n"/>
+      <c r="E121" s="6" t="n"/>
+      <c r="F121" s="6" t="n"/>
+      <c r="G121" s="6" t="n"/>
+      <c r="H121" s="6" t="n"/>
+      <c r="I121" s="6" t="n"/>
+      <c r="J121" s="6" t="n"/>
+      <c r="K121" s="7" t="n"/>
+      <c r="L121" s="8" t="n"/>
+      <c r="M121" s="6" t="n"/>
+      <c r="N121" s="6" t="n"/>
+      <c r="O121" s="9" t="n"/>
+      <c r="P121" s="6" t="n"/>
+      <c r="Q121" s="6" t="n"/>
+      <c r="R121" s="6" t="n"/>
+      <c r="S121" s="6" t="n"/>
+      <c r="T121">
+        <f>IF(C121="","",IF(AND(K121&lt;&gt;"",L121=""),"Falta el costo",IF(AND(LEFT(I121,6)="Por ov",K121&lt;&gt;"",G121=""),"Falta el peso del ovillo",IF(AND(A121="",B121=""),"Falta la categoría",IF(AND(A121="",I121=""),"Falta cómo se vende",IF(AND(K121&lt;&gt;"",N121="",M121=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="11" t="n"/>
+      <c r="B122" s="6" t="n"/>
+      <c r="C122" s="6" t="n"/>
+      <c r="D122" s="6" t="n"/>
+      <c r="E122" s="6" t="n"/>
+      <c r="F122" s="6" t="n"/>
+      <c r="G122" s="6" t="n"/>
+      <c r="H122" s="6" t="n"/>
+      <c r="I122" s="6" t="n"/>
+      <c r="J122" s="6" t="n"/>
+      <c r="K122" s="7" t="n"/>
+      <c r="L122" s="8" t="n"/>
+      <c r="M122" s="6" t="n"/>
+      <c r="N122" s="6" t="n"/>
+      <c r="O122" s="9" t="n"/>
+      <c r="P122" s="6" t="n"/>
+      <c r="Q122" s="6" t="n"/>
+      <c r="R122" s="6" t="n"/>
+      <c r="S122" s="6" t="n"/>
+      <c r="T122">
+        <f>IF(C122="","",IF(AND(K122&lt;&gt;"",L122=""),"Falta el costo",IF(AND(LEFT(I122,6)="Por ov",K122&lt;&gt;"",G122=""),"Falta el peso del ovillo",IF(AND(A122="",B122=""),"Falta la categoría",IF(AND(A122="",I122=""),"Falta cómo se vende",IF(AND(K122&lt;&gt;"",N122="",M122=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="11" t="n"/>
+      <c r="B123" s="6" t="n"/>
+      <c r="C123" s="6" t="n"/>
+      <c r="D123" s="6" t="n"/>
+      <c r="E123" s="6" t="n"/>
+      <c r="F123" s="6" t="n"/>
+      <c r="G123" s="6" t="n"/>
+      <c r="H123" s="6" t="n"/>
+      <c r="I123" s="6" t="n"/>
+      <c r="J123" s="6" t="n"/>
+      <c r="K123" s="7" t="n"/>
+      <c r="L123" s="8" t="n"/>
+      <c r="M123" s="6" t="n"/>
+      <c r="N123" s="6" t="n"/>
+      <c r="O123" s="9" t="n"/>
+      <c r="P123" s="6" t="n"/>
+      <c r="Q123" s="6" t="n"/>
+      <c r="R123" s="6" t="n"/>
+      <c r="S123" s="6" t="n"/>
+      <c r="T123">
+        <f>IF(C123="","",IF(AND(K123&lt;&gt;"",L123=""),"Falta el costo",IF(AND(LEFT(I123,6)="Por ov",K123&lt;&gt;"",G123=""),"Falta el peso del ovillo",IF(AND(A123="",B123=""),"Falta la categoría",IF(AND(A123="",I123=""),"Falta cómo se vende",IF(AND(K123&lt;&gt;"",N123="",M123=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="11" t="n"/>
+      <c r="B124" s="6" t="n"/>
+      <c r="C124" s="6" t="n"/>
+      <c r="D124" s="6" t="n"/>
+      <c r="E124" s="6" t="n"/>
+      <c r="F124" s="6" t="n"/>
+      <c r="G124" s="6" t="n"/>
+      <c r="H124" s="6" t="n"/>
+      <c r="I124" s="6" t="n"/>
+      <c r="J124" s="6" t="n"/>
+      <c r="K124" s="7" t="n"/>
+      <c r="L124" s="8" t="n"/>
+      <c r="M124" s="6" t="n"/>
+      <c r="N124" s="6" t="n"/>
+      <c r="O124" s="9" t="n"/>
+      <c r="P124" s="6" t="n"/>
+      <c r="Q124" s="6" t="n"/>
+      <c r="R124" s="6" t="n"/>
+      <c r="S124" s="6" t="n"/>
+      <c r="T124">
+        <f>IF(C124="","",IF(AND(K124&lt;&gt;"",L124=""),"Falta el costo",IF(AND(LEFT(I124,6)="Por ov",K124&lt;&gt;"",G124=""),"Falta el peso del ovillo",IF(AND(A124="",B124=""),"Falta la categoría",IF(AND(A124="",I124=""),"Falta cómo se vende",IF(AND(K124&lt;&gt;"",N124="",M124=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="11" t="n"/>
+      <c r="B125" s="6" t="n"/>
+      <c r="C125" s="6" t="n"/>
+      <c r="D125" s="6" t="n"/>
+      <c r="E125" s="6" t="n"/>
+      <c r="F125" s="6" t="n"/>
+      <c r="G125" s="6" t="n"/>
+      <c r="H125" s="6" t="n"/>
+      <c r="I125" s="6" t="n"/>
+      <c r="J125" s="6" t="n"/>
+      <c r="K125" s="7" t="n"/>
+      <c r="L125" s="8" t="n"/>
+      <c r="M125" s="6" t="n"/>
+      <c r="N125" s="6" t="n"/>
+      <c r="O125" s="9" t="n"/>
+      <c r="P125" s="6" t="n"/>
+      <c r="Q125" s="6" t="n"/>
+      <c r="R125" s="6" t="n"/>
+      <c r="S125" s="6" t="n"/>
+      <c r="T125">
+        <f>IF(C125="","",IF(AND(K125&lt;&gt;"",L125=""),"Falta el costo",IF(AND(LEFT(I125,6)="Por ov",K125&lt;&gt;"",G125=""),"Falta el peso del ovillo",IF(AND(A125="",B125=""),"Falta la categoría",IF(AND(A125="",I125=""),"Falta cómo se vende",IF(AND(K125&lt;&gt;"",N125="",M125=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="11" t="n"/>
+      <c r="B126" s="6" t="n"/>
+      <c r="C126" s="6" t="n"/>
+      <c r="D126" s="6" t="n"/>
+      <c r="E126" s="6" t="n"/>
+      <c r="F126" s="6" t="n"/>
+      <c r="G126" s="6" t="n"/>
+      <c r="H126" s="6" t="n"/>
+      <c r="I126" s="6" t="n"/>
+      <c r="J126" s="6" t="n"/>
+      <c r="K126" s="7" t="n"/>
+      <c r="L126" s="8" t="n"/>
+      <c r="M126" s="6" t="n"/>
+      <c r="N126" s="6" t="n"/>
+      <c r="O126" s="9" t="n"/>
+      <c r="P126" s="6" t="n"/>
+      <c r="Q126" s="6" t="n"/>
+      <c r="R126" s="6" t="n"/>
+      <c r="S126" s="6" t="n"/>
+      <c r="T126">
+        <f>IF(C126="","",IF(AND(K126&lt;&gt;"",L126=""),"Falta el costo",IF(AND(LEFT(I126,6)="Por ov",K126&lt;&gt;"",G126=""),"Falta el peso del ovillo",IF(AND(A126="",B126=""),"Falta la categoría",IF(AND(A126="",I126=""),"Falta cómo se vende",IF(AND(K126&lt;&gt;"",N126="",M126=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="11" t="n"/>
+      <c r="B127" s="6" t="n"/>
+      <c r="C127" s="6" t="n"/>
+      <c r="D127" s="6" t="n"/>
+      <c r="E127" s="6" t="n"/>
+      <c r="F127" s="6" t="n"/>
+      <c r="G127" s="6" t="n"/>
+      <c r="H127" s="6" t="n"/>
+      <c r="I127" s="6" t="n"/>
+      <c r="J127" s="6" t="n"/>
+      <c r="K127" s="7" t="n"/>
+      <c r="L127" s="8" t="n"/>
+      <c r="M127" s="6" t="n"/>
+      <c r="N127" s="6" t="n"/>
+      <c r="O127" s="9" t="n"/>
+      <c r="P127" s="6" t="n"/>
+      <c r="Q127" s="6" t="n"/>
+      <c r="R127" s="6" t="n"/>
+      <c r="S127" s="6" t="n"/>
+      <c r="T127">
+        <f>IF(C127="","",IF(AND(K127&lt;&gt;"",L127=""),"Falta el costo",IF(AND(LEFT(I127,6)="Por ov",K127&lt;&gt;"",G127=""),"Falta el peso del ovillo",IF(AND(A127="",B127=""),"Falta la categoría",IF(AND(A127="",I127=""),"Falta cómo se vende",IF(AND(K127&lt;&gt;"",N127="",M127=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="11" t="n"/>
+      <c r="B128" s="6" t="n"/>
+      <c r="C128" s="6" t="n"/>
+      <c r="D128" s="6" t="n"/>
+      <c r="E128" s="6" t="n"/>
+      <c r="F128" s="6" t="n"/>
+      <c r="G128" s="6" t="n"/>
+      <c r="H128" s="6" t="n"/>
+      <c r="I128" s="6" t="n"/>
+      <c r="J128" s="6" t="n"/>
+      <c r="K128" s="7" t="n"/>
+      <c r="L128" s="8" t="n"/>
+      <c r="M128" s="6" t="n"/>
+      <c r="N128" s="6" t="n"/>
+      <c r="O128" s="9" t="n"/>
+      <c r="P128" s="6" t="n"/>
+      <c r="Q128" s="6" t="n"/>
+      <c r="R128" s="6" t="n"/>
+      <c r="S128" s="6" t="n"/>
+      <c r="T128">
+        <f>IF(C128="","",IF(AND(K128&lt;&gt;"",L128=""),"Falta el costo",IF(AND(LEFT(I128,6)="Por ov",K128&lt;&gt;"",G128=""),"Falta el peso del ovillo",IF(AND(A128="",B128=""),"Falta la categoría",IF(AND(A128="",I128=""),"Falta cómo se vende",IF(AND(K128&lt;&gt;"",N128="",M128=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="11" t="n"/>
+      <c r="B129" s="6" t="n"/>
+      <c r="C129" s="6" t="n"/>
+      <c r="D129" s="6" t="n"/>
+      <c r="E129" s="6" t="n"/>
+      <c r="F129" s="6" t="n"/>
+      <c r="G129" s="6" t="n"/>
+      <c r="H129" s="6" t="n"/>
+      <c r="I129" s="6" t="n"/>
+      <c r="J129" s="6" t="n"/>
+      <c r="K129" s="7" t="n"/>
+      <c r="L129" s="8" t="n"/>
+      <c r="M129" s="6" t="n"/>
+      <c r="N129" s="6" t="n"/>
+      <c r="O129" s="9" t="n"/>
+      <c r="P129" s="6" t="n"/>
+      <c r="Q129" s="6" t="n"/>
+      <c r="R129" s="6" t="n"/>
+      <c r="S129" s="6" t="n"/>
+      <c r="T129">
+        <f>IF(C129="","",IF(AND(K129&lt;&gt;"",L129=""),"Falta el costo",IF(AND(LEFT(I129,6)="Por ov",K129&lt;&gt;"",G129=""),"Falta el peso del ovillo",IF(AND(A129="",B129=""),"Falta la categoría",IF(AND(A129="",I129=""),"Falta cómo se vende",IF(AND(K129&lt;&gt;"",N129="",M129=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="11" t="n"/>
+      <c r="B130" s="6" t="n"/>
+      <c r="C130" s="6" t="n"/>
+      <c r="D130" s="6" t="n"/>
+      <c r="E130" s="6" t="n"/>
+      <c r="F130" s="6" t="n"/>
+      <c r="G130" s="6" t="n"/>
+      <c r="H130" s="6" t="n"/>
+      <c r="I130" s="6" t="n"/>
+      <c r="J130" s="6" t="n"/>
+      <c r="K130" s="7" t="n"/>
+      <c r="L130" s="8" t="n"/>
+      <c r="M130" s="6" t="n"/>
+      <c r="N130" s="6" t="n"/>
+      <c r="O130" s="9" t="n"/>
+      <c r="P130" s="6" t="n"/>
+      <c r="Q130" s="6" t="n"/>
+      <c r="R130" s="6" t="n"/>
+      <c r="S130" s="6" t="n"/>
+      <c r="T130">
+        <f>IF(C130="","",IF(AND(K130&lt;&gt;"",L130=""),"Falta el costo",IF(AND(LEFT(I130,6)="Por ov",K130&lt;&gt;"",G130=""),"Falta el peso del ovillo",IF(AND(A130="",B130=""),"Falta la categoría",IF(AND(A130="",I130=""),"Falta cómo se vende",IF(AND(K130&lt;&gt;"",N130="",M130=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="11" t="n"/>
+      <c r="B131" s="6" t="n"/>
+      <c r="C131" s="6" t="n"/>
+      <c r="D131" s="6" t="n"/>
+      <c r="E131" s="6" t="n"/>
+      <c r="F131" s="6" t="n"/>
+      <c r="G131" s="6" t="n"/>
+      <c r="H131" s="6" t="n"/>
+      <c r="I131" s="6" t="n"/>
+      <c r="J131" s="6" t="n"/>
+      <c r="K131" s="7" t="n"/>
+      <c r="L131" s="8" t="n"/>
+      <c r="M131" s="6" t="n"/>
+      <c r="N131" s="6" t="n"/>
+      <c r="O131" s="9" t="n"/>
+      <c r="P131" s="6" t="n"/>
+      <c r="Q131" s="6" t="n"/>
+      <c r="R131" s="6" t="n"/>
+      <c r="S131" s="6" t="n"/>
+      <c r="T131">
+        <f>IF(C131="","",IF(AND(K131&lt;&gt;"",L131=""),"Falta el costo",IF(AND(LEFT(I131,6)="Por ov",K131&lt;&gt;"",G131=""),"Falta el peso del ovillo",IF(AND(A131="",B131=""),"Falta la categoría",IF(AND(A131="",I131=""),"Falta cómo se vende",IF(AND(K131&lt;&gt;"",N131="",M131=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="11" t="n"/>
+      <c r="B132" s="6" t="n"/>
+      <c r="C132" s="6" t="n"/>
+      <c r="D132" s="6" t="n"/>
+      <c r="E132" s="6" t="n"/>
+      <c r="F132" s="6" t="n"/>
+      <c r="G132" s="6" t="n"/>
+      <c r="H132" s="6" t="n"/>
+      <c r="I132" s="6" t="n"/>
+      <c r="J132" s="6" t="n"/>
+      <c r="K132" s="7" t="n"/>
+      <c r="L132" s="8" t="n"/>
+      <c r="M132" s="6" t="n"/>
+      <c r="N132" s="6" t="n"/>
+      <c r="O132" s="9" t="n"/>
+      <c r="P132" s="6" t="n"/>
+      <c r="Q132" s="6" t="n"/>
+      <c r="R132" s="6" t="n"/>
+      <c r="S132" s="6" t="n"/>
+      <c r="T132">
+        <f>IF(C132="","",IF(AND(K132&lt;&gt;"",L132=""),"Falta el costo",IF(AND(LEFT(I132,6)="Por ov",K132&lt;&gt;"",G132=""),"Falta el peso del ovillo",IF(AND(A132="",B132=""),"Falta la categoría",IF(AND(A132="",I132=""),"Falta cómo se vende",IF(AND(K132&lt;&gt;"",N132="",M132=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="11" t="n"/>
+      <c r="B133" s="6" t="n"/>
+      <c r="C133" s="6" t="n"/>
+      <c r="D133" s="6" t="n"/>
+      <c r="E133" s="6" t="n"/>
+      <c r="F133" s="6" t="n"/>
+      <c r="G133" s="6" t="n"/>
+      <c r="H133" s="6" t="n"/>
+      <c r="I133" s="6" t="n"/>
+      <c r="J133" s="6" t="n"/>
+      <c r="K133" s="7" t="n"/>
+      <c r="L133" s="8" t="n"/>
+      <c r="M133" s="6" t="n"/>
+      <c r="N133" s="6" t="n"/>
+      <c r="O133" s="9" t="n"/>
+      <c r="P133" s="6" t="n"/>
+      <c r="Q133" s="6" t="n"/>
+      <c r="R133" s="6" t="n"/>
+      <c r="S133" s="6" t="n"/>
+      <c r="T133">
+        <f>IF(C133="","",IF(AND(K133&lt;&gt;"",L133=""),"Falta el costo",IF(AND(LEFT(I133,6)="Por ov",K133&lt;&gt;"",G133=""),"Falta el peso del ovillo",IF(AND(A133="",B133=""),"Falta la categoría",IF(AND(A133="",I133=""),"Falta cómo se vende",IF(AND(K133&lt;&gt;"",N133="",M133=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="11" t="n"/>
+      <c r="B134" s="6" t="n"/>
+      <c r="C134" s="6" t="n"/>
+      <c r="D134" s="6" t="n"/>
+      <c r="E134" s="6" t="n"/>
+      <c r="F134" s="6" t="n"/>
+      <c r="G134" s="6" t="n"/>
+      <c r="H134" s="6" t="n"/>
+      <c r="I134" s="6" t="n"/>
+      <c r="J134" s="6" t="n"/>
+      <c r="K134" s="7" t="n"/>
+      <c r="L134" s="8" t="n"/>
+      <c r="M134" s="6" t="n"/>
+      <c r="N134" s="6" t="n"/>
+      <c r="O134" s="9" t="n"/>
+      <c r="P134" s="6" t="n"/>
+      <c r="Q134" s="6" t="n"/>
+      <c r="R134" s="6" t="n"/>
+      <c r="S134" s="6" t="n"/>
+      <c r="T134">
+        <f>IF(C134="","",IF(AND(K134&lt;&gt;"",L134=""),"Falta el costo",IF(AND(LEFT(I134,6)="Por ov",K134&lt;&gt;"",G134=""),"Falta el peso del ovillo",IF(AND(A134="",B134=""),"Falta la categoría",IF(AND(A134="",I134=""),"Falta cómo se vende",IF(AND(K134&lt;&gt;"",N134="",M134=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="11" t="n"/>
+      <c r="B135" s="6" t="n"/>
+      <c r="C135" s="6" t="n"/>
+      <c r="D135" s="6" t="n"/>
+      <c r="E135" s="6" t="n"/>
+      <c r="F135" s="6" t="n"/>
+      <c r="G135" s="6" t="n"/>
+      <c r="H135" s="6" t="n"/>
+      <c r="I135" s="6" t="n"/>
+      <c r="J135" s="6" t="n"/>
+      <c r="K135" s="7" t="n"/>
+      <c r="L135" s="8" t="n"/>
+      <c r="M135" s="6" t="n"/>
+      <c r="N135" s="6" t="n"/>
+      <c r="O135" s="9" t="n"/>
+      <c r="P135" s="6" t="n"/>
+      <c r="Q135" s="6" t="n"/>
+      <c r="R135" s="6" t="n"/>
+      <c r="S135" s="6" t="n"/>
+      <c r="T135">
+        <f>IF(C135="","",IF(AND(K135&lt;&gt;"",L135=""),"Falta el costo",IF(AND(LEFT(I135,6)="Por ov",K135&lt;&gt;"",G135=""),"Falta el peso del ovillo",IF(AND(A135="",B135=""),"Falta la categoría",IF(AND(A135="",I135=""),"Falta cómo se vende",IF(AND(K135&lt;&gt;"",N135="",M135=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="11" t="n"/>
+      <c r="B136" s="6" t="n"/>
+      <c r="C136" s="6" t="n"/>
+      <c r="D136" s="6" t="n"/>
+      <c r="E136" s="6" t="n"/>
+      <c r="F136" s="6" t="n"/>
+      <c r="G136" s="6" t="n"/>
+      <c r="H136" s="6" t="n"/>
+      <c r="I136" s="6" t="n"/>
+      <c r="J136" s="6" t="n"/>
+      <c r="K136" s="7" t="n"/>
+      <c r="L136" s="8" t="n"/>
+      <c r="M136" s="6" t="n"/>
+      <c r="N136" s="6" t="n"/>
+      <c r="O136" s="9" t="n"/>
+      <c r="P136" s="6" t="n"/>
+      <c r="Q136" s="6" t="n"/>
+      <c r="R136" s="6" t="n"/>
+      <c r="S136" s="6" t="n"/>
+      <c r="T136">
+        <f>IF(C136="","",IF(AND(K136&lt;&gt;"",L136=""),"Falta el costo",IF(AND(LEFT(I136,6)="Por ov",K136&lt;&gt;"",G136=""),"Falta el peso del ovillo",IF(AND(A136="",B136=""),"Falta la categoría",IF(AND(A136="",I136=""),"Falta cómo se vende",IF(AND(K136&lt;&gt;"",N136="",M136=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="11" t="n"/>
+      <c r="B137" s="6" t="n"/>
+      <c r="C137" s="6" t="n"/>
+      <c r="D137" s="6" t="n"/>
+      <c r="E137" s="6" t="n"/>
+      <c r="F137" s="6" t="n"/>
+      <c r="G137" s="6" t="n"/>
+      <c r="H137" s="6" t="n"/>
+      <c r="I137" s="6" t="n"/>
+      <c r="J137" s="6" t="n"/>
+      <c r="K137" s="7" t="n"/>
+      <c r="L137" s="8" t="n"/>
+      <c r="M137" s="6" t="n"/>
+      <c r="N137" s="6" t="n"/>
+      <c r="O137" s="9" t="n"/>
+      <c r="P137" s="6" t="n"/>
+      <c r="Q137" s="6" t="n"/>
+      <c r="R137" s="6" t="n"/>
+      <c r="S137" s="6" t="n"/>
+      <c r="T137">
+        <f>IF(C137="","",IF(AND(K137&lt;&gt;"",L137=""),"Falta el costo",IF(AND(LEFT(I137,6)="Por ov",K137&lt;&gt;"",G137=""),"Falta el peso del ovillo",IF(AND(A137="",B137=""),"Falta la categoría",IF(AND(A137="",I137=""),"Falta cómo se vende",IF(AND(K137&lt;&gt;"",N137="",M137=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="11" t="n"/>
+      <c r="B138" s="6" t="n"/>
+      <c r="C138" s="6" t="n"/>
+      <c r="D138" s="6" t="n"/>
+      <c r="E138" s="6" t="n"/>
+      <c r="F138" s="6" t="n"/>
+      <c r="G138" s="6" t="n"/>
+      <c r="H138" s="6" t="n"/>
+      <c r="I138" s="6" t="n"/>
+      <c r="J138" s="6" t="n"/>
+      <c r="K138" s="7" t="n"/>
+      <c r="L138" s="8" t="n"/>
+      <c r="M138" s="6" t="n"/>
+      <c r="N138" s="6" t="n"/>
+      <c r="O138" s="9" t="n"/>
+      <c r="P138" s="6" t="n"/>
+      <c r="Q138" s="6" t="n"/>
+      <c r="R138" s="6" t="n"/>
+      <c r="S138" s="6" t="n"/>
+      <c r="T138">
+        <f>IF(C138="","",IF(AND(K138&lt;&gt;"",L138=""),"Falta el costo",IF(AND(LEFT(I138,6)="Por ov",K138&lt;&gt;"",G138=""),"Falta el peso del ovillo",IF(AND(A138="",B138=""),"Falta la categoría",IF(AND(A138="",I138=""),"Falta cómo se vende",IF(AND(K138&lt;&gt;"",N138="",M138=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="11" t="n"/>
+      <c r="B139" s="6" t="n"/>
+      <c r="C139" s="6" t="n"/>
+      <c r="D139" s="6" t="n"/>
+      <c r="E139" s="6" t="n"/>
+      <c r="F139" s="6" t="n"/>
+      <c r="G139" s="6" t="n"/>
+      <c r="H139" s="6" t="n"/>
+      <c r="I139" s="6" t="n"/>
+      <c r="J139" s="6" t="n"/>
+      <c r="K139" s="7" t="n"/>
+      <c r="L139" s="8" t="n"/>
+      <c r="M139" s="6" t="n"/>
+      <c r="N139" s="6" t="n"/>
+      <c r="O139" s="9" t="n"/>
+      <c r="P139" s="6" t="n"/>
+      <c r="Q139" s="6" t="n"/>
+      <c r="R139" s="6" t="n"/>
+      <c r="S139" s="6" t="n"/>
+      <c r="T139">
+        <f>IF(C139="","",IF(AND(K139&lt;&gt;"",L139=""),"Falta el costo",IF(AND(LEFT(I139,6)="Por ov",K139&lt;&gt;"",G139=""),"Falta el peso del ovillo",IF(AND(A139="",B139=""),"Falta la categoría",IF(AND(A139="",I139=""),"Falta cómo se vende",IF(AND(K139&lt;&gt;"",N139="",M139=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="11" t="n"/>
+      <c r="B140" s="6" t="n"/>
+      <c r="C140" s="6" t="n"/>
+      <c r="D140" s="6" t="n"/>
+      <c r="E140" s="6" t="n"/>
+      <c r="F140" s="6" t="n"/>
+      <c r="G140" s="6" t="n"/>
+      <c r="H140" s="6" t="n"/>
+      <c r="I140" s="6" t="n"/>
+      <c r="J140" s="6" t="n"/>
+      <c r="K140" s="7" t="n"/>
+      <c r="L140" s="8" t="n"/>
+      <c r="M140" s="6" t="n"/>
+      <c r="N140" s="6" t="n"/>
+      <c r="O140" s="9" t="n"/>
+      <c r="P140" s="6" t="n"/>
+      <c r="Q140" s="6" t="n"/>
+      <c r="R140" s="6" t="n"/>
+      <c r="S140" s="6" t="n"/>
+      <c r="T140">
+        <f>IF(C140="","",IF(AND(K140&lt;&gt;"",L140=""),"Falta el costo",IF(AND(LEFT(I140,6)="Por ov",K140&lt;&gt;"",G140=""),"Falta el peso del ovillo",IF(AND(A140="",B140=""),"Falta la categoría",IF(AND(A140="",I140=""),"Falta cómo se vende",IF(AND(K140&lt;&gt;"",N140="",M140=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="11" t="n"/>
+      <c r="B141" s="6" t="n"/>
+      <c r="C141" s="6" t="n"/>
+      <c r="D141" s="6" t="n"/>
+      <c r="E141" s="6" t="n"/>
+      <c r="F141" s="6" t="n"/>
+      <c r="G141" s="6" t="n"/>
+      <c r="H141" s="6" t="n"/>
+      <c r="I141" s="6" t="n"/>
+      <c r="J141" s="6" t="n"/>
+      <c r="K141" s="7" t="n"/>
+      <c r="L141" s="8" t="n"/>
+      <c r="M141" s="6" t="n"/>
+      <c r="N141" s="6" t="n"/>
+      <c r="O141" s="9" t="n"/>
+      <c r="P141" s="6" t="n"/>
+      <c r="Q141" s="6" t="n"/>
+      <c r="R141" s="6" t="n"/>
+      <c r="S141" s="6" t="n"/>
+      <c r="T141">
+        <f>IF(C141="","",IF(AND(K141&lt;&gt;"",L141=""),"Falta el costo",IF(AND(LEFT(I141,6)="Por ov",K141&lt;&gt;"",G141=""),"Falta el peso del ovillo",IF(AND(A141="",B141=""),"Falta la categoría",IF(AND(A141="",I141=""),"Falta cómo se vende",IF(AND(K141&lt;&gt;"",N141="",M141=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="11" t="n"/>
+      <c r="B142" s="6" t="n"/>
+      <c r="C142" s="6" t="n"/>
+      <c r="D142" s="6" t="n"/>
+      <c r="E142" s="6" t="n"/>
+      <c r="F142" s="6" t="n"/>
+      <c r="G142" s="6" t="n"/>
+      <c r="H142" s="6" t="n"/>
+      <c r="I142" s="6" t="n"/>
+      <c r="J142" s="6" t="n"/>
+      <c r="K142" s="7" t="n"/>
+      <c r="L142" s="8" t="n"/>
+      <c r="M142" s="6" t="n"/>
+      <c r="N142" s="6" t="n"/>
+      <c r="O142" s="9" t="n"/>
+      <c r="P142" s="6" t="n"/>
+      <c r="Q142" s="6" t="n"/>
+      <c r="R142" s="6" t="n"/>
+      <c r="S142" s="6" t="n"/>
+      <c r="T142">
+        <f>IF(C142="","",IF(AND(K142&lt;&gt;"",L142=""),"Falta el costo",IF(AND(LEFT(I142,6)="Por ov",K142&lt;&gt;"",G142=""),"Falta el peso del ovillo",IF(AND(A142="",B142=""),"Falta la categoría",IF(AND(A142="",I142=""),"Falta cómo se vende",IF(AND(K142&lt;&gt;"",N142="",M142=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="11" t="n"/>
+      <c r="B143" s="6" t="n"/>
+      <c r="C143" s="6" t="n"/>
+      <c r="D143" s="6" t="n"/>
+      <c r="E143" s="6" t="n"/>
+      <c r="F143" s="6" t="n"/>
+      <c r="G143" s="6" t="n"/>
+      <c r="H143" s="6" t="n"/>
+      <c r="I143" s="6" t="n"/>
+      <c r="J143" s="6" t="n"/>
+      <c r="K143" s="7" t="n"/>
+      <c r="L143" s="8" t="n"/>
+      <c r="M143" s="6" t="n"/>
+      <c r="N143" s="6" t="n"/>
+      <c r="O143" s="9" t="n"/>
+      <c r="P143" s="6" t="n"/>
+      <c r="Q143" s="6" t="n"/>
+      <c r="R143" s="6" t="n"/>
+      <c r="S143" s="6" t="n"/>
+      <c r="T143">
+        <f>IF(C143="","",IF(AND(K143&lt;&gt;"",L143=""),"Falta el costo",IF(AND(LEFT(I143,6)="Por ov",K143&lt;&gt;"",G143=""),"Falta el peso del ovillo",IF(AND(A143="",B143=""),"Falta la categoría",IF(AND(A143="",I143=""),"Falta cómo se vende",IF(AND(K143&lt;&gt;"",N143="",M143=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="11" t="n"/>
+      <c r="B144" s="6" t="n"/>
+      <c r="C144" s="6" t="n"/>
+      <c r="D144" s="6" t="n"/>
+      <c r="E144" s="6" t="n"/>
+      <c r="F144" s="6" t="n"/>
+      <c r="G144" s="6" t="n"/>
+      <c r="H144" s="6" t="n"/>
+      <c r="I144" s="6" t="n"/>
+      <c r="J144" s="6" t="n"/>
+      <c r="K144" s="7" t="n"/>
+      <c r="L144" s="8" t="n"/>
+      <c r="M144" s="6" t="n"/>
+      <c r="N144" s="6" t="n"/>
+      <c r="O144" s="9" t="n"/>
+      <c r="P144" s="6" t="n"/>
+      <c r="Q144" s="6" t="n"/>
+      <c r="R144" s="6" t="n"/>
+      <c r="S144" s="6" t="n"/>
+      <c r="T144">
+        <f>IF(C144="","",IF(AND(K144&lt;&gt;"",L144=""),"Falta el costo",IF(AND(LEFT(I144,6)="Por ov",K144&lt;&gt;"",G144=""),"Falta el peso del ovillo",IF(AND(A144="",B144=""),"Falta la categoría",IF(AND(A144="",I144=""),"Falta cómo se vende",IF(AND(K144&lt;&gt;"",N144="",M144=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="11" t="n"/>
+      <c r="B145" s="6" t="n"/>
+      <c r="C145" s="6" t="n"/>
+      <c r="D145" s="6" t="n"/>
+      <c r="E145" s="6" t="n"/>
+      <c r="F145" s="6" t="n"/>
+      <c r="G145" s="6" t="n"/>
+      <c r="H145" s="6" t="n"/>
+      <c r="I145" s="6" t="n"/>
+      <c r="J145" s="6" t="n"/>
+      <c r="K145" s="7" t="n"/>
+      <c r="L145" s="8" t="n"/>
+      <c r="M145" s="6" t="n"/>
+      <c r="N145" s="6" t="n"/>
+      <c r="O145" s="9" t="n"/>
+      <c r="P145" s="6" t="n"/>
+      <c r="Q145" s="6" t="n"/>
+      <c r="R145" s="6" t="n"/>
+      <c r="S145" s="6" t="n"/>
+      <c r="T145">
+        <f>IF(C145="","",IF(AND(K145&lt;&gt;"",L145=""),"Falta el costo",IF(AND(LEFT(I145,6)="Por ov",K145&lt;&gt;"",G145=""),"Falta el peso del ovillo",IF(AND(A145="",B145=""),"Falta la categoría",IF(AND(A145="",I145=""),"Falta cómo se vende",IF(AND(K145&lt;&gt;"",N145="",M145=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="11" t="n"/>
+      <c r="B146" s="6" t="n"/>
+      <c r="C146" s="6" t="n"/>
+      <c r="D146" s="6" t="n"/>
+      <c r="E146" s="6" t="n"/>
+      <c r="F146" s="6" t="n"/>
+      <c r="G146" s="6" t="n"/>
+      <c r="H146" s="6" t="n"/>
+      <c r="I146" s="6" t="n"/>
+      <c r="J146" s="6" t="n"/>
+      <c r="K146" s="7" t="n"/>
+      <c r="L146" s="8" t="n"/>
+      <c r="M146" s="6" t="n"/>
+      <c r="N146" s="6" t="n"/>
+      <c r="O146" s="9" t="n"/>
+      <c r="P146" s="6" t="n"/>
+      <c r="Q146" s="6" t="n"/>
+      <c r="R146" s="6" t="n"/>
+      <c r="S146" s="6" t="n"/>
+      <c r="T146">
+        <f>IF(C146="","",IF(AND(K146&lt;&gt;"",L146=""),"Falta el costo",IF(AND(LEFT(I146,6)="Por ov",K146&lt;&gt;"",G146=""),"Falta el peso del ovillo",IF(AND(A146="",B146=""),"Falta la categoría",IF(AND(A146="",I146=""),"Falta cómo se vende",IF(AND(K146&lt;&gt;"",N146="",M146=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="11" t="n"/>
+      <c r="B147" s="6" t="n"/>
+      <c r="C147" s="6" t="n"/>
+      <c r="D147" s="6" t="n"/>
+      <c r="E147" s="6" t="n"/>
+      <c r="F147" s="6" t="n"/>
+      <c r="G147" s="6" t="n"/>
+      <c r="H147" s="6" t="n"/>
+      <c r="I147" s="6" t="n"/>
+      <c r="J147" s="6" t="n"/>
+      <c r="K147" s="7" t="n"/>
+      <c r="L147" s="8" t="n"/>
+      <c r="M147" s="6" t="n"/>
+      <c r="N147" s="6" t="n"/>
+      <c r="O147" s="9" t="n"/>
+      <c r="P147" s="6" t="n"/>
+      <c r="Q147" s="6" t="n"/>
+      <c r="R147" s="6" t="n"/>
+      <c r="S147" s="6" t="n"/>
+      <c r="T147">
+        <f>IF(C147="","",IF(AND(K147&lt;&gt;"",L147=""),"Falta el costo",IF(AND(LEFT(I147,6)="Por ov",K147&lt;&gt;"",G147=""),"Falta el peso del ovillo",IF(AND(A147="",B147=""),"Falta la categoría",IF(AND(A147="",I147=""),"Falta cómo se vende",IF(AND(K147&lt;&gt;"",N147="",M147=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="11" t="n"/>
+      <c r="B148" s="6" t="n"/>
+      <c r="C148" s="6" t="n"/>
+      <c r="D148" s="6" t="n"/>
+      <c r="E148" s="6" t="n"/>
+      <c r="F148" s="6" t="n"/>
+      <c r="G148" s="6" t="n"/>
+      <c r="H148" s="6" t="n"/>
+      <c r="I148" s="6" t="n"/>
+      <c r="J148" s="6" t="n"/>
+      <c r="K148" s="7" t="n"/>
+      <c r="L148" s="8" t="n"/>
+      <c r="M148" s="6" t="n"/>
+      <c r="N148" s="6" t="n"/>
+      <c r="O148" s="9" t="n"/>
+      <c r="P148" s="6" t="n"/>
+      <c r="Q148" s="6" t="n"/>
+      <c r="R148" s="6" t="n"/>
+      <c r="S148" s="6" t="n"/>
+      <c r="T148">
+        <f>IF(C148="","",IF(AND(K148&lt;&gt;"",L148=""),"Falta el costo",IF(AND(LEFT(I148,6)="Por ov",K148&lt;&gt;"",G148=""),"Falta el peso del ovillo",IF(AND(A148="",B148=""),"Falta la categoría",IF(AND(A148="",I148=""),"Falta cómo se vende",IF(AND(K148&lt;&gt;"",N148="",M148=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="11" t="n"/>
+      <c r="B149" s="6" t="n"/>
+      <c r="C149" s="6" t="n"/>
+      <c r="D149" s="6" t="n"/>
+      <c r="E149" s="6" t="n"/>
+      <c r="F149" s="6" t="n"/>
+      <c r="G149" s="6" t="n"/>
+      <c r="H149" s="6" t="n"/>
+      <c r="I149" s="6" t="n"/>
+      <c r="J149" s="6" t="n"/>
+      <c r="K149" s="7" t="n"/>
+      <c r="L149" s="8" t="n"/>
+      <c r="M149" s="6" t="n"/>
+      <c r="N149" s="6" t="n"/>
+      <c r="O149" s="9" t="n"/>
+      <c r="P149" s="6" t="n"/>
+      <c r="Q149" s="6" t="n"/>
+      <c r="R149" s="6" t="n"/>
+      <c r="S149" s="6" t="n"/>
+      <c r="T149">
+        <f>IF(C149="","",IF(AND(K149&lt;&gt;"",L149=""),"Falta el costo",IF(AND(LEFT(I149,6)="Por ov",K149&lt;&gt;"",G149=""),"Falta el peso del ovillo",IF(AND(A149="",B149=""),"Falta la categoría",IF(AND(A149="",I149=""),"Falta cómo se vende",IF(AND(K149&lt;&gt;"",N149="",M149=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="11" t="n"/>
+      <c r="B150" s="6" t="n"/>
+      <c r="C150" s="6" t="n"/>
+      <c r="D150" s="6" t="n"/>
+      <c r="E150" s="6" t="n"/>
+      <c r="F150" s="6" t="n"/>
+      <c r="G150" s="6" t="n"/>
+      <c r="H150" s="6" t="n"/>
+      <c r="I150" s="6" t="n"/>
+      <c r="J150" s="6" t="n"/>
+      <c r="K150" s="7" t="n"/>
+      <c r="L150" s="8" t="n"/>
+      <c r="M150" s="6" t="n"/>
+      <c r="N150" s="6" t="n"/>
+      <c r="O150" s="9" t="n"/>
+      <c r="P150" s="6" t="n"/>
+      <c r="Q150" s="6" t="n"/>
+      <c r="R150" s="6" t="n"/>
+      <c r="S150" s="6" t="n"/>
+      <c r="T150">
+        <f>IF(C150="","",IF(AND(K150&lt;&gt;"",L150=""),"Falta el costo",IF(AND(LEFT(I150,6)="Por ov",K150&lt;&gt;"",G150=""),"Falta el peso del ovillo",IF(AND(A150="",B150=""),"Falta la categoría",IF(AND(A150="",I150=""),"Falta cómo se vende",IF(AND(K150&lt;&gt;"",N150="",M150=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:S75"/>
+  <conditionalFormatting sqref="T2:T150">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(LEFT(T2,5)="Falta")</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>T2="OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="6">
-    <dataValidation sqref="B2:B75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B150" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>=Listas!$A$1:$A$10</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I150" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>=Listas!$C$1:$C$2</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J150" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>=Listas!$D$1:$D$2</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M150" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Listas!$B$1:$B$4</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:L75 Q2:Q75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Número" error="Escribe un número (sin puntos ni signos)." type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="K2:L150 Q2:Q150" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Número" error="Escribe un número (sin puntos ni signos)." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Escribe una fecha (DD/MM/AAAA)." type="date" operator="greaterThan">
+    <dataValidation sqref="O2:O150" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Escribe una fecha (DD/MM/AAAA)." type="date" operator="greaterThan">
       <formula1>45658</formula1>
     </dataValidation>
   </dataValidations>
@@ -3768,7 +6147,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Plantilla de carga de la Mercería: regla Taller/Tienda, hoja Resumen, revisión automática y más filas (#399)
Claude-Session: https://claude.ai/code/session_01U9SAsfVct6L94yoocG63si

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/herramientas/merceria-carga/plantilla_carga_merceria.xlsx
+++ b/herramientas/merceria-carga/plantilla_carga_merceria.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Productos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Listas" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Productos'!$A$1:$S$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Productos'!$A$1:$S$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,10 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="165" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +58,17 @@
     <font>
       <color rgb="008A8A8F"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00B00020"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="5">
@@ -98,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -119,10 +132,44 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00B00020"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FDE2E2"/>
+          <bgColor rgb="00FDE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="002E7D32"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -484,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -504,127 +551,176 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>IMPORTANTE: esta plantilla es SOLO para lo que se VENDE en la Mercería (el inventario de la TIENDA). Lo que usas para tejer (lanas, relleno, ojos… del inventario del TALLER) NO va aquí.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Si dudas de un producto, pregúntate: ¿lo va a comprar una clienta en la tienda? Si sí, va aquí; si es para tejer, no.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Cómo llenarla</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>1. Hoja "Productos": las primeras 34 filas son los productos que ya existen en el ERP. No cambies la columna ID.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>2. Para cada producto que vas a tener en la tienda, escribe la cantidad comprada (ovillos o unidades) y el costo de compra de cada ovillo o unidad (lo que pagaste, con IVA).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>3. Si un producto ya no lo vas a vender, escribe "No" en la columna "¿Se vende en la tienda?".</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>4. Los productos nuevos (agujas, herrajes, accesorios, relleno, tijeras, etc.) van en las filas vacías de abajo, sin ID.</t>
+          <t>1. Hoja "Productos": las primeras 34 filas son los productos que ya existen en el ERP. No cambies la columna ID.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>5. Proveedor, factura y fecha de compra: llénalos si los tienes; sirven para el Kardex y para la contabilidad.</t>
+          <t>2. Para cada producto que vas a tener en la tienda, escribe la cantidad comprada (ovillos o unidades) y el costo de compra de cada ovillo o unidad (lo que pagaste, con IVA).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>6. Código de barras: si el producto lo trae, escríbelo (o escanéalo con un lector); así se encuentra rápido en el POS.</t>
+          <t>3. Si un producto ya no lo vas a vender, escribe "No" en la columna "¿Se vende en la tienda?".</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>4. Los productos nuevos (agujas, herrajes, accesorios, relleno, tijeras, etc.) van en las filas vacías de abajo, sin ID.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Columna "¿Cómo se vende?"</t>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>5. Proveedor, factura y fecha de compra: llénalos si los tienes; sirven para el Kardex y para la contabilidad.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>6. Código de barras: si el producto lo trae, escríbelo (o escanéalo con un lector); así se encuentra rápido en el POS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Columna "¿Cómo se vende?"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>• Por ovillo y por gramo (lanas e hilos): en la caja se vende el ovillo completo o los gramos que pida el cliente. Escribe cuántos ovillos compraste y el costo de cada ovillo; el sistema guarda la existencia en gramos usando el peso del ovillo.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>• Por unidad: agujas, herrajes, tijeras, paquetes de relleno, etc. Se vende la pieza completa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Para las lanas y los hilos es obligatorio el peso por ovillo (columna "Peso por unidad (g)").</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>El precio de venta no hace falta</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>Para las lanas y los hilos es obligatorio el peso por ovillo (columna "Peso por unidad (g)").</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>El precio de venta no hace falta</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>Claude lo calcula con la regla de la Mercería del ERP: costo × (1 + carga de costos fijos) ÷ (1 − 40 % de utilidad), redondeado a los $100.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>La columna "Precio de venta hoy" es solo de referencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Cuando termines</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>La columna "Precio de venta hoy" es solo de referencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Cuando termines</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t>Envía el archivo a Claude. Claude crea los productos nuevos, registra las entradas con su costo (como "Entrada de nueva mercancía" del ERP), calcula los precios y te muestra un resumen antes de dejarlo listo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>Para no equivocarte (ayudas nuevas, 22-oct-2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>• La columna T de "Productos" ("Revisión") te avisa en rojo si a una fila le falta el costo, el peso del ovillo o la categoría. Déjala vacía antes de enviar el archivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>• La hoja "Resumen" cuenta cuántos productos llevan cantidad, cuántos ovillos/unidades y cuánto vale la mercancía (cantidad × costo). Ese valor es el que necesita el contador para el saldo de apertura.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>• Ejemplo de una lana: Cantidad comprada = 10 (ovillos), Costo por ovillo = 7.500, Peso por unidad = 160. El sistema guarda 1.600 g a $46,88 el gramo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>• Ejemplo de una aguja: Cantidad = 24, Costo por unidad = 1.800, "¿Cómo se vende?" = Por unidad.</t>
         </is>
       </c>
     </row>
@@ -639,7 +735,105 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S75"/>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Resumen de la carga (se calcula solo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Productos con cantidad comprada</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>COUNTIFS(Productos!K2:K150,"&gt;0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ovillos o unidades compradas (suma)</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>SUM(Productos!K2:K150)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Valor de la mercancía a costo (COP)</t>
+        </is>
+      </c>
+      <c r="B5" s="16">
+        <f>SUMPRODUCT(Productos!K2:K150,Productos!L2:L150)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Productos nuevos (sin ID) por crear</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>COUNTIFS(Productos!A2:A150,"",Productos!C2:C150,"&lt;&gt;")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Filas con algo por corregir</t>
+        </is>
+      </c>
+      <c r="B7" s="17">
+        <f>COUNTIF(Productos!T2:T150,"Falta*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Productos marcados "No se vende"</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>COUNTIF(Productos!J2:J150,"No")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Si "Filas con algo por corregir" no es 0, revisa la columna T de la hoja Productos antes de enviar el archivo.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -661,6 +855,7 @@
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
     <col width="30" customWidth="1" min="19" max="19"/>
+    <col width="34" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1">
@@ -757,6 +952,11 @@
       <c r="S1" s="4" t="inlineStr">
         <is>
           <t>Notas</t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>Revisión (automática, no tocar)</t>
         </is>
       </c>
     </row>
@@ -822,6 +1022,10 @@
         </is>
       </c>
       <c r="S2" s="6" t="n"/>
+      <c r="T2">
+        <f>IF(C2="","",IF(AND(K2&lt;&gt;"",L2=""),"Falta el costo",IF(AND(LEFT(I2,6)="Por ov",K2&lt;&gt;"",G2=""),"Falta el peso del ovillo",IF(AND(A2="",B2=""),"Falta la categoría",IF(AND(A2="",I2=""),"Falta cómo se vende",IF(AND(K2&lt;&gt;"",N2="",M2=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -885,6 +1089,10 @@
         </is>
       </c>
       <c r="S3" s="6" t="n"/>
+      <c r="T3">
+        <f>IF(C3="","",IF(AND(K3&lt;&gt;"",L3=""),"Falta el costo",IF(AND(LEFT(I3,6)="Por ov",K3&lt;&gt;"",G3=""),"Falta el peso del ovillo",IF(AND(A3="",B3=""),"Falta la categoría",IF(AND(A3="",I3=""),"Falta cómo se vende",IF(AND(K3&lt;&gt;"",N3="",M3=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -948,6 +1156,10 @@
         </is>
       </c>
       <c r="S4" s="6" t="n"/>
+      <c r="T4">
+        <f>IF(C4="","",IF(AND(K4&lt;&gt;"",L4=""),"Falta el costo",IF(AND(LEFT(I4,6)="Por ov",K4&lt;&gt;"",G4=""),"Falta el peso del ovillo",IF(AND(A4="",B4=""),"Falta la categoría",IF(AND(A4="",I4=""),"Falta cómo se vende",IF(AND(K4&lt;&gt;"",N4="",M4=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -1011,6 +1223,10 @@
         </is>
       </c>
       <c r="S5" s="6" t="n"/>
+      <c r="T5">
+        <f>IF(C5="","",IF(AND(K5&lt;&gt;"",L5=""),"Falta el costo",IF(AND(LEFT(I5,6)="Por ov",K5&lt;&gt;"",G5=""),"Falta el peso del ovillo",IF(AND(A5="",B5=""),"Falta la categoría",IF(AND(A5="",I5=""),"Falta cómo se vende",IF(AND(K5&lt;&gt;"",N5="",M5=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1074,6 +1290,10 @@
         </is>
       </c>
       <c r="S6" s="6" t="n"/>
+      <c r="T6">
+        <f>IF(C6="","",IF(AND(K6&lt;&gt;"",L6=""),"Falta el costo",IF(AND(LEFT(I6,6)="Por ov",K6&lt;&gt;"",G6=""),"Falta el peso del ovillo",IF(AND(A6="",B6=""),"Falta la categoría",IF(AND(A6="",I6=""),"Falta cómo se vende",IF(AND(K6&lt;&gt;"",N6="",M6=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1137,6 +1357,10 @@
         </is>
       </c>
       <c r="S7" s="6" t="n"/>
+      <c r="T7">
+        <f>IF(C7="","",IF(AND(K7&lt;&gt;"",L7=""),"Falta el costo",IF(AND(LEFT(I7,6)="Por ov",K7&lt;&gt;"",G7=""),"Falta el peso del ovillo",IF(AND(A7="",B7=""),"Falta la categoría",IF(AND(A7="",I7=""),"Falta cómo se vende",IF(AND(K7&lt;&gt;"",N7="",M7=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1200,6 +1424,10 @@
         </is>
       </c>
       <c r="S8" s="6" t="n"/>
+      <c r="T8">
+        <f>IF(C8="","",IF(AND(K8&lt;&gt;"",L8=""),"Falta el costo",IF(AND(LEFT(I8,6)="Por ov",K8&lt;&gt;"",G8=""),"Falta el peso del ovillo",IF(AND(A8="",B8=""),"Falta la categoría",IF(AND(A8="",I8=""),"Falta cómo se vende",IF(AND(K8&lt;&gt;"",N8="",M8=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1263,6 +1491,10 @@
         </is>
       </c>
       <c r="S9" s="6" t="n"/>
+      <c r="T9">
+        <f>IF(C9="","",IF(AND(K9&lt;&gt;"",L9=""),"Falta el costo",IF(AND(LEFT(I9,6)="Por ov",K9&lt;&gt;"",G9=""),"Falta el peso del ovillo",IF(AND(A9="",B9=""),"Falta la categoría",IF(AND(A9="",I9=""),"Falta cómo se vende",IF(AND(K9&lt;&gt;"",N9="",M9=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1326,6 +1558,10 @@
         </is>
       </c>
       <c r="S10" s="6" t="n"/>
+      <c r="T10">
+        <f>IF(C10="","",IF(AND(K10&lt;&gt;"",L10=""),"Falta el costo",IF(AND(LEFT(I10,6)="Por ov",K10&lt;&gt;"",G10=""),"Falta el peso del ovillo",IF(AND(A10="",B10=""),"Falta la categoría",IF(AND(A10="",I10=""),"Falta cómo se vende",IF(AND(K10&lt;&gt;"",N10="",M10=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1389,6 +1625,10 @@
         </is>
       </c>
       <c r="S11" s="6" t="n"/>
+      <c r="T11">
+        <f>IF(C11="","",IF(AND(K11&lt;&gt;"",L11=""),"Falta el costo",IF(AND(LEFT(I11,6)="Por ov",K11&lt;&gt;"",G11=""),"Falta el peso del ovillo",IF(AND(A11="",B11=""),"Falta la categoría",IF(AND(A11="",I11=""),"Falta cómo se vende",IF(AND(K11&lt;&gt;"",N11="",M11=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1452,6 +1692,10 @@
         </is>
       </c>
       <c r="S12" s="6" t="n"/>
+      <c r="T12">
+        <f>IF(C12="","",IF(AND(K12&lt;&gt;"",L12=""),"Falta el costo",IF(AND(LEFT(I12,6)="Por ov",K12&lt;&gt;"",G12=""),"Falta el peso del ovillo",IF(AND(A12="",B12=""),"Falta la categoría",IF(AND(A12="",I12=""),"Falta cómo se vende",IF(AND(K12&lt;&gt;"",N12="",M12=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1515,6 +1759,10 @@
         </is>
       </c>
       <c r="S13" s="6" t="n"/>
+      <c r="T13">
+        <f>IF(C13="","",IF(AND(K13&lt;&gt;"",L13=""),"Falta el costo",IF(AND(LEFT(I13,6)="Por ov",K13&lt;&gt;"",G13=""),"Falta el peso del ovillo",IF(AND(A13="",B13=""),"Falta la categoría",IF(AND(A13="",I13=""),"Falta cómo se vende",IF(AND(K13&lt;&gt;"",N13="",M13=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1578,6 +1826,10 @@
         </is>
       </c>
       <c r="S14" s="6" t="n"/>
+      <c r="T14">
+        <f>IF(C14="","",IF(AND(K14&lt;&gt;"",L14=""),"Falta el costo",IF(AND(LEFT(I14,6)="Por ov",K14&lt;&gt;"",G14=""),"Falta el peso del ovillo",IF(AND(A14="",B14=""),"Falta la categoría",IF(AND(A14="",I14=""),"Falta cómo se vende",IF(AND(K14&lt;&gt;"",N14="",M14=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1641,6 +1893,10 @@
         </is>
       </c>
       <c r="S15" s="6" t="n"/>
+      <c r="T15">
+        <f>IF(C15="","",IF(AND(K15&lt;&gt;"",L15=""),"Falta el costo",IF(AND(LEFT(I15,6)="Por ov",K15&lt;&gt;"",G15=""),"Falta el peso del ovillo",IF(AND(A15="",B15=""),"Falta la categoría",IF(AND(A15="",I15=""),"Falta cómo se vende",IF(AND(K15&lt;&gt;"",N15="",M15=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1704,6 +1960,10 @@
         </is>
       </c>
       <c r="S16" s="6" t="n"/>
+      <c r="T16">
+        <f>IF(C16="","",IF(AND(K16&lt;&gt;"",L16=""),"Falta el costo",IF(AND(LEFT(I16,6)="Por ov",K16&lt;&gt;"",G16=""),"Falta el peso del ovillo",IF(AND(A16="",B16=""),"Falta la categoría",IF(AND(A16="",I16=""),"Falta cómo se vende",IF(AND(K16&lt;&gt;"",N16="",M16=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1767,6 +2027,10 @@
         </is>
       </c>
       <c r="S17" s="6" t="n"/>
+      <c r="T17">
+        <f>IF(C17="","",IF(AND(K17&lt;&gt;"",L17=""),"Falta el costo",IF(AND(LEFT(I17,6)="Por ov",K17&lt;&gt;"",G17=""),"Falta el peso del ovillo",IF(AND(A17="",B17=""),"Falta la categoría",IF(AND(A17="",I17=""),"Falta cómo se vende",IF(AND(K17&lt;&gt;"",N17="",M17=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1830,6 +2094,10 @@
         </is>
       </c>
       <c r="S18" s="6" t="n"/>
+      <c r="T18">
+        <f>IF(C18="","",IF(AND(K18&lt;&gt;"",L18=""),"Falta el costo",IF(AND(LEFT(I18,6)="Por ov",K18&lt;&gt;"",G18=""),"Falta el peso del ovillo",IF(AND(A18="",B18=""),"Falta la categoría",IF(AND(A18="",I18=""),"Falta cómo se vende",IF(AND(K18&lt;&gt;"",N18="",M18=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1893,6 +2161,10 @@
         </is>
       </c>
       <c r="S19" s="6" t="n"/>
+      <c r="T19">
+        <f>IF(C19="","",IF(AND(K19&lt;&gt;"",L19=""),"Falta el costo",IF(AND(LEFT(I19,6)="Por ov",K19&lt;&gt;"",G19=""),"Falta el peso del ovillo",IF(AND(A19="",B19=""),"Falta la categoría",IF(AND(A19="",I19=""),"Falta cómo se vende",IF(AND(K19&lt;&gt;"",N19="",M19=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1956,6 +2228,10 @@
         </is>
       </c>
       <c r="S20" s="6" t="n"/>
+      <c r="T20">
+        <f>IF(C20="","",IF(AND(K20&lt;&gt;"",L20=""),"Falta el costo",IF(AND(LEFT(I20,6)="Por ov",K20&lt;&gt;"",G20=""),"Falta el peso del ovillo",IF(AND(A20="",B20=""),"Falta la categoría",IF(AND(A20="",I20=""),"Falta cómo se vende",IF(AND(K20&lt;&gt;"",N20="",M20=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -2019,6 +2295,10 @@
         </is>
       </c>
       <c r="S21" s="6" t="n"/>
+      <c r="T21">
+        <f>IF(C21="","",IF(AND(K21&lt;&gt;"",L21=""),"Falta el costo",IF(AND(LEFT(I21,6)="Por ov",K21&lt;&gt;"",G21=""),"Falta el peso del ovillo",IF(AND(A21="",B21=""),"Falta la categoría",IF(AND(A21="",I21=""),"Falta cómo se vende",IF(AND(K21&lt;&gt;"",N21="",M21=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -2082,6 +2362,10 @@
         </is>
       </c>
       <c r="S22" s="6" t="n"/>
+      <c r="T22">
+        <f>IF(C22="","",IF(AND(K22&lt;&gt;"",L22=""),"Falta el costo",IF(AND(LEFT(I22,6)="Por ov",K22&lt;&gt;"",G22=""),"Falta el peso del ovillo",IF(AND(A22="",B22=""),"Falta la categoría",IF(AND(A22="",I22=""),"Falta cómo se vende",IF(AND(K22&lt;&gt;"",N22="",M22=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -2145,6 +2429,10 @@
         </is>
       </c>
       <c r="S23" s="6" t="n"/>
+      <c r="T23">
+        <f>IF(C23="","",IF(AND(K23&lt;&gt;"",L23=""),"Falta el costo",IF(AND(LEFT(I23,6)="Por ov",K23&lt;&gt;"",G23=""),"Falta el peso del ovillo",IF(AND(A23="",B23=""),"Falta la categoría",IF(AND(A23="",I23=""),"Falta cómo se vende",IF(AND(K23&lt;&gt;"",N23="",M23=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -2208,6 +2496,10 @@
         </is>
       </c>
       <c r="S24" s="6" t="n"/>
+      <c r="T24">
+        <f>IF(C24="","",IF(AND(K24&lt;&gt;"",L24=""),"Falta el costo",IF(AND(LEFT(I24,6)="Por ov",K24&lt;&gt;"",G24=""),"Falta el peso del ovillo",IF(AND(A24="",B24=""),"Falta la categoría",IF(AND(A24="",I24=""),"Falta cómo se vende",IF(AND(K24&lt;&gt;"",N24="",M24=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -2271,6 +2563,10 @@
         </is>
       </c>
       <c r="S25" s="6" t="n"/>
+      <c r="T25">
+        <f>IF(C25="","",IF(AND(K25&lt;&gt;"",L25=""),"Falta el costo",IF(AND(LEFT(I25,6)="Por ov",K25&lt;&gt;"",G25=""),"Falta el peso del ovillo",IF(AND(A25="",B25=""),"Falta la categoría",IF(AND(A25="",I25=""),"Falta cómo se vende",IF(AND(K25&lt;&gt;"",N25="",M25=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -2334,6 +2630,10 @@
         </is>
       </c>
       <c r="S26" s="6" t="n"/>
+      <c r="T26">
+        <f>IF(C26="","",IF(AND(K26&lt;&gt;"",L26=""),"Falta el costo",IF(AND(LEFT(I26,6)="Por ov",K26&lt;&gt;"",G26=""),"Falta el peso del ovillo",IF(AND(A26="",B26=""),"Falta la categoría",IF(AND(A26="",I26=""),"Falta cómo se vende",IF(AND(K26&lt;&gt;"",N26="",M26=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -2397,6 +2697,10 @@
         </is>
       </c>
       <c r="S27" s="6" t="n"/>
+      <c r="T27">
+        <f>IF(C27="","",IF(AND(K27&lt;&gt;"",L27=""),"Falta el costo",IF(AND(LEFT(I27,6)="Por ov",K27&lt;&gt;"",G27=""),"Falta el peso del ovillo",IF(AND(A27="",B27=""),"Falta la categoría",IF(AND(A27="",I27=""),"Falta cómo se vende",IF(AND(K27&lt;&gt;"",N27="",M27=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -2460,6 +2764,10 @@
         </is>
       </c>
       <c r="S28" s="6" t="n"/>
+      <c r="T28">
+        <f>IF(C28="","",IF(AND(K28&lt;&gt;"",L28=""),"Falta el costo",IF(AND(LEFT(I28,6)="Por ov",K28&lt;&gt;"",G28=""),"Falta el peso del ovillo",IF(AND(A28="",B28=""),"Falta la categoría",IF(AND(A28="",I28=""),"Falta cómo se vende",IF(AND(K28&lt;&gt;"",N28="",M28=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -2523,6 +2831,10 @@
         </is>
       </c>
       <c r="S29" s="6" t="n"/>
+      <c r="T29">
+        <f>IF(C29="","",IF(AND(K29&lt;&gt;"",L29=""),"Falta el costo",IF(AND(LEFT(I29,6)="Por ov",K29&lt;&gt;"",G29=""),"Falta el peso del ovillo",IF(AND(A29="",B29=""),"Falta la categoría",IF(AND(A29="",I29=""),"Falta cómo se vende",IF(AND(K29&lt;&gt;"",N29="",M29=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -2586,6 +2898,10 @@
         </is>
       </c>
       <c r="S30" s="6" t="n"/>
+      <c r="T30">
+        <f>IF(C30="","",IF(AND(K30&lt;&gt;"",L30=""),"Falta el costo",IF(AND(LEFT(I30,6)="Por ov",K30&lt;&gt;"",G30=""),"Falta el peso del ovillo",IF(AND(A30="",B30=""),"Falta la categoría",IF(AND(A30="",I30=""),"Falta cómo se vende",IF(AND(K30&lt;&gt;"",N30="",M30=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -2649,6 +2965,10 @@
         </is>
       </c>
       <c r="S31" s="6" t="n"/>
+      <c r="T31">
+        <f>IF(C31="","",IF(AND(K31&lt;&gt;"",L31=""),"Falta el costo",IF(AND(LEFT(I31,6)="Por ov",K31&lt;&gt;"",G31=""),"Falta el peso del ovillo",IF(AND(A31="",B31=""),"Falta la categoría",IF(AND(A31="",I31=""),"Falta cómo se vende",IF(AND(K31&lt;&gt;"",N31="",M31=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -2712,6 +3032,10 @@
         </is>
       </c>
       <c r="S32" s="6" t="n"/>
+      <c r="T32">
+        <f>IF(C32="","",IF(AND(K32&lt;&gt;"",L32=""),"Falta el costo",IF(AND(LEFT(I32,6)="Por ov",K32&lt;&gt;"",G32=""),"Falta el peso del ovillo",IF(AND(A32="",B32=""),"Falta la categoría",IF(AND(A32="",I32=""),"Falta cómo se vende",IF(AND(K32&lt;&gt;"",N32="",M32=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -2775,6 +3099,10 @@
         </is>
       </c>
       <c r="S33" s="6" t="n"/>
+      <c r="T33">
+        <f>IF(C33="","",IF(AND(K33&lt;&gt;"",L33=""),"Falta el costo",IF(AND(LEFT(I33,6)="Por ov",K33&lt;&gt;"",G33=""),"Falta el peso del ovillo",IF(AND(A33="",B33=""),"Falta la categoría",IF(AND(A33="",I33=""),"Falta cómo se vende",IF(AND(K33&lt;&gt;"",N33="",M33=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -2838,6 +3166,10 @@
         </is>
       </c>
       <c r="S34" s="6" t="n"/>
+      <c r="T34">
+        <f>IF(C34="","",IF(AND(K34&lt;&gt;"",L34=""),"Falta el costo",IF(AND(LEFT(I34,6)="Por ov",K34&lt;&gt;"",G34=""),"Falta el peso del ovillo",IF(AND(A34="",B34=""),"Falta la categoría",IF(AND(A34="",I34=""),"Falta cómo se vende",IF(AND(K34&lt;&gt;"",N34="",M34=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -2901,6 +3233,10 @@
         </is>
       </c>
       <c r="S35" s="6" t="n"/>
+      <c r="T35">
+        <f>IF(C35="","",IF(AND(K35&lt;&gt;"",L35=""),"Falta el costo",IF(AND(LEFT(I35,6)="Por ov",K35&lt;&gt;"",G35=""),"Falta el peso del ovillo",IF(AND(A35="",B35=""),"Falta la categoría",IF(AND(A35="",I35=""),"Falta cómo se vende",IF(AND(K35&lt;&gt;"",N35="",M35=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n"/>
@@ -2922,6 +3258,10 @@
       <c r="Q36" s="6" t="n"/>
       <c r="R36" s="6" t="n"/>
       <c r="S36" s="6" t="n"/>
+      <c r="T36">
+        <f>IF(C36="","",IF(AND(K36&lt;&gt;"",L36=""),"Falta el costo",IF(AND(LEFT(I36,6)="Por ov",K36&lt;&gt;"",G36=""),"Falta el peso del ovillo",IF(AND(A36="",B36=""),"Falta la categoría",IF(AND(A36="",I36=""),"Falta cómo se vende",IF(AND(K36&lt;&gt;"",N36="",M36=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n"/>
@@ -2943,6 +3283,10 @@
       <c r="Q37" s="6" t="n"/>
       <c r="R37" s="6" t="n"/>
       <c r="S37" s="6" t="n"/>
+      <c r="T37">
+        <f>IF(C37="","",IF(AND(K37&lt;&gt;"",L37=""),"Falta el costo",IF(AND(LEFT(I37,6)="Por ov",K37&lt;&gt;"",G37=""),"Falta el peso del ovillo",IF(AND(A37="",B37=""),"Falta la categoría",IF(AND(A37="",I37=""),"Falta cómo se vende",IF(AND(K37&lt;&gt;"",N37="",M37=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="n"/>
@@ -2964,6 +3308,10 @@
       <c r="Q38" s="6" t="n"/>
       <c r="R38" s="6" t="n"/>
       <c r="S38" s="6" t="n"/>
+      <c r="T38">
+        <f>IF(C38="","",IF(AND(K38&lt;&gt;"",L38=""),"Falta el costo",IF(AND(LEFT(I38,6)="Por ov",K38&lt;&gt;"",G38=""),"Falta el peso del ovillo",IF(AND(A38="",B38=""),"Falta la categoría",IF(AND(A38="",I38=""),"Falta cómo se vende",IF(AND(K38&lt;&gt;"",N38="",M38=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="11" t="n"/>
@@ -2985,6 +3333,10 @@
       <c r="Q39" s="6" t="n"/>
       <c r="R39" s="6" t="n"/>
       <c r="S39" s="6" t="n"/>
+      <c r="T39">
+        <f>IF(C39="","",IF(AND(K39&lt;&gt;"",L39=""),"Falta el costo",IF(AND(LEFT(I39,6)="Por ov",K39&lt;&gt;"",G39=""),"Falta el peso del ovillo",IF(AND(A39="",B39=""),"Falta la categoría",IF(AND(A39="",I39=""),"Falta cómo se vende",IF(AND(K39&lt;&gt;"",N39="",M39=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="11" t="n"/>
@@ -3006,6 +3358,10 @@
       <c r="Q40" s="6" t="n"/>
       <c r="R40" s="6" t="n"/>
       <c r="S40" s="6" t="n"/>
+      <c r="T40">
+        <f>IF(C40="","",IF(AND(K40&lt;&gt;"",L40=""),"Falta el costo",IF(AND(LEFT(I40,6)="Por ov",K40&lt;&gt;"",G40=""),"Falta el peso del ovillo",IF(AND(A40="",B40=""),"Falta la categoría",IF(AND(A40="",I40=""),"Falta cómo se vende",IF(AND(K40&lt;&gt;"",N40="",M40=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="11" t="n"/>
@@ -3027,6 +3383,10 @@
       <c r="Q41" s="6" t="n"/>
       <c r="R41" s="6" t="n"/>
       <c r="S41" s="6" t="n"/>
+      <c r="T41">
+        <f>IF(C41="","",IF(AND(K41&lt;&gt;"",L41=""),"Falta el costo",IF(AND(LEFT(I41,6)="Por ov",K41&lt;&gt;"",G41=""),"Falta el peso del ovillo",IF(AND(A41="",B41=""),"Falta la categoría",IF(AND(A41="",I41=""),"Falta cómo se vende",IF(AND(K41&lt;&gt;"",N41="",M41=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="11" t="n"/>
@@ -3048,6 +3408,10 @@
       <c r="Q42" s="6" t="n"/>
       <c r="R42" s="6" t="n"/>
       <c r="S42" s="6" t="n"/>
+      <c r="T42">
+        <f>IF(C42="","",IF(AND(K42&lt;&gt;"",L42=""),"Falta el costo",IF(AND(LEFT(I42,6)="Por ov",K42&lt;&gt;"",G42=""),"Falta el peso del ovillo",IF(AND(A42="",B42=""),"Falta la categoría",IF(AND(A42="",I42=""),"Falta cómo se vende",IF(AND(K42&lt;&gt;"",N42="",M42=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="11" t="n"/>
@@ -3069,6 +3433,10 @@
       <c r="Q43" s="6" t="n"/>
       <c r="R43" s="6" t="n"/>
       <c r="S43" s="6" t="n"/>
+      <c r="T43">
+        <f>IF(C43="","",IF(AND(K43&lt;&gt;"",L43=""),"Falta el costo",IF(AND(LEFT(I43,6)="Por ov",K43&lt;&gt;"",G43=""),"Falta el peso del ovillo",IF(AND(A43="",B43=""),"Falta la categoría",IF(AND(A43="",I43=""),"Falta cómo se vende",IF(AND(K43&lt;&gt;"",N43="",M43=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="11" t="n"/>
@@ -3090,6 +3458,10 @@
       <c r="Q44" s="6" t="n"/>
       <c r="R44" s="6" t="n"/>
       <c r="S44" s="6" t="n"/>
+      <c r="T44">
+        <f>IF(C44="","",IF(AND(K44&lt;&gt;"",L44=""),"Falta el costo",IF(AND(LEFT(I44,6)="Por ov",K44&lt;&gt;"",G44=""),"Falta el peso del ovillo",IF(AND(A44="",B44=""),"Falta la categoría",IF(AND(A44="",I44=""),"Falta cómo se vende",IF(AND(K44&lt;&gt;"",N44="",M44=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="11" t="n"/>
@@ -3111,6 +3483,10 @@
       <c r="Q45" s="6" t="n"/>
       <c r="R45" s="6" t="n"/>
       <c r="S45" s="6" t="n"/>
+      <c r="T45">
+        <f>IF(C45="","",IF(AND(K45&lt;&gt;"",L45=""),"Falta el costo",IF(AND(LEFT(I45,6)="Por ov",K45&lt;&gt;"",G45=""),"Falta el peso del ovillo",IF(AND(A45="",B45=""),"Falta la categoría",IF(AND(A45="",I45=""),"Falta cómo se vende",IF(AND(K45&lt;&gt;"",N45="",M45=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="11" t="n"/>
@@ -3132,6 +3508,10 @@
       <c r="Q46" s="6" t="n"/>
       <c r="R46" s="6" t="n"/>
       <c r="S46" s="6" t="n"/>
+      <c r="T46">
+        <f>IF(C46="","",IF(AND(K46&lt;&gt;"",L46=""),"Falta el costo",IF(AND(LEFT(I46,6)="Por ov",K46&lt;&gt;"",G46=""),"Falta el peso del ovillo",IF(AND(A46="",B46=""),"Falta la categoría",IF(AND(A46="",I46=""),"Falta cómo se vende",IF(AND(K46&lt;&gt;"",N46="",M46=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="11" t="n"/>
@@ -3153,6 +3533,10 @@
       <c r="Q47" s="6" t="n"/>
       <c r="R47" s="6" t="n"/>
       <c r="S47" s="6" t="n"/>
+      <c r="T47">
+        <f>IF(C47="","",IF(AND(K47&lt;&gt;"",L47=""),"Falta el costo",IF(AND(LEFT(I47,6)="Por ov",K47&lt;&gt;"",G47=""),"Falta el peso del ovillo",IF(AND(A47="",B47=""),"Falta la categoría",IF(AND(A47="",I47=""),"Falta cómo se vende",IF(AND(K47&lt;&gt;"",N47="",M47=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="11" t="n"/>
@@ -3174,6 +3558,10 @@
       <c r="Q48" s="6" t="n"/>
       <c r="R48" s="6" t="n"/>
       <c r="S48" s="6" t="n"/>
+      <c r="T48">
+        <f>IF(C48="","",IF(AND(K48&lt;&gt;"",L48=""),"Falta el costo",IF(AND(LEFT(I48,6)="Por ov",K48&lt;&gt;"",G48=""),"Falta el peso del ovillo",IF(AND(A48="",B48=""),"Falta la categoría",IF(AND(A48="",I48=""),"Falta cómo se vende",IF(AND(K48&lt;&gt;"",N48="",M48=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="11" t="n"/>
@@ -3195,6 +3583,10 @@
       <c r="Q49" s="6" t="n"/>
       <c r="R49" s="6" t="n"/>
       <c r="S49" s="6" t="n"/>
+      <c r="T49">
+        <f>IF(C49="","",IF(AND(K49&lt;&gt;"",L49=""),"Falta el costo",IF(AND(LEFT(I49,6)="Por ov",K49&lt;&gt;"",G49=""),"Falta el peso del ovillo",IF(AND(A49="",B49=""),"Falta la categoría",IF(AND(A49="",I49=""),"Falta cómo se vende",IF(AND(K49&lt;&gt;"",N49="",M49=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="11" t="n"/>
@@ -3216,6 +3608,10 @@
       <c r="Q50" s="6" t="n"/>
       <c r="R50" s="6" t="n"/>
       <c r="S50" s="6" t="n"/>
+      <c r="T50">
+        <f>IF(C50="","",IF(AND(K50&lt;&gt;"",L50=""),"Falta el costo",IF(AND(LEFT(I50,6)="Por ov",K50&lt;&gt;"",G50=""),"Falta el peso del ovillo",IF(AND(A50="",B50=""),"Falta la categoría",IF(AND(A50="",I50=""),"Falta cómo se vende",IF(AND(K50&lt;&gt;"",N50="",M50=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="11" t="n"/>
@@ -3237,6 +3633,10 @@
       <c r="Q51" s="6" t="n"/>
       <c r="R51" s="6" t="n"/>
       <c r="S51" s="6" t="n"/>
+      <c r="T51">
+        <f>IF(C51="","",IF(AND(K51&lt;&gt;"",L51=""),"Falta el costo",IF(AND(LEFT(I51,6)="Por ov",K51&lt;&gt;"",G51=""),"Falta el peso del ovillo",IF(AND(A51="",B51=""),"Falta la categoría",IF(AND(A51="",I51=""),"Falta cómo se vende",IF(AND(K51&lt;&gt;"",N51="",M51=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="11" t="n"/>
@@ -3258,6 +3658,10 @@
       <c r="Q52" s="6" t="n"/>
       <c r="R52" s="6" t="n"/>
       <c r="S52" s="6" t="n"/>
+      <c r="T52">
+        <f>IF(C52="","",IF(AND(K52&lt;&gt;"",L52=""),"Falta el costo",IF(AND(LEFT(I52,6)="Por ov",K52&lt;&gt;"",G52=""),"Falta el peso del ovillo",IF(AND(A52="",B52=""),"Falta la categoría",IF(AND(A52="",I52=""),"Falta cómo se vende",IF(AND(K52&lt;&gt;"",N52="",M52=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n"/>
@@ -3279,6 +3683,10 @@
       <c r="Q53" s="6" t="n"/>
       <c r="R53" s="6" t="n"/>
       <c r="S53" s="6" t="n"/>
+      <c r="T53">
+        <f>IF(C53="","",IF(AND(K53&lt;&gt;"",L53=""),"Falta el costo",IF(AND(LEFT(I53,6)="Por ov",K53&lt;&gt;"",G53=""),"Falta el peso del ovillo",IF(AND(A53="",B53=""),"Falta la categoría",IF(AND(A53="",I53=""),"Falta cómo se vende",IF(AND(K53&lt;&gt;"",N53="",M53=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="11" t="n"/>
@@ -3300,6 +3708,10 @@
       <c r="Q54" s="6" t="n"/>
       <c r="R54" s="6" t="n"/>
       <c r="S54" s="6" t="n"/>
+      <c r="T54">
+        <f>IF(C54="","",IF(AND(K54&lt;&gt;"",L54=""),"Falta el costo",IF(AND(LEFT(I54,6)="Por ov",K54&lt;&gt;"",G54=""),"Falta el peso del ovillo",IF(AND(A54="",B54=""),"Falta la categoría",IF(AND(A54="",I54=""),"Falta cómo se vende",IF(AND(K54&lt;&gt;"",N54="",M54=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n"/>
@@ -3321,6 +3733,10 @@
       <c r="Q55" s="6" t="n"/>
       <c r="R55" s="6" t="n"/>
       <c r="S55" s="6" t="n"/>
+      <c r="T55">
+        <f>IF(C55="","",IF(AND(K55&lt;&gt;"",L55=""),"Falta el costo",IF(AND(LEFT(I55,6)="Por ov",K55&lt;&gt;"",G55=""),"Falta el peso del ovillo",IF(AND(A55="",B55=""),"Falta la categoría",IF(AND(A55="",I55=""),"Falta cómo se vende",IF(AND(K55&lt;&gt;"",N55="",M55=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n"/>
@@ -3342,6 +3758,10 @@
       <c r="Q56" s="6" t="n"/>
       <c r="R56" s="6" t="n"/>
       <c r="S56" s="6" t="n"/>
+      <c r="T56">
+        <f>IF(C56="","",IF(AND(K56&lt;&gt;"",L56=""),"Falta el costo",IF(AND(LEFT(I56,6)="Por ov",K56&lt;&gt;"",G56=""),"Falta el peso del ovillo",IF(AND(A56="",B56=""),"Falta la categoría",IF(AND(A56="",I56=""),"Falta cómo se vende",IF(AND(K56&lt;&gt;"",N56="",M56=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n"/>
@@ -3363,6 +3783,10 @@
       <c r="Q57" s="6" t="n"/>
       <c r="R57" s="6" t="n"/>
       <c r="S57" s="6" t="n"/>
+      <c r="T57">
+        <f>IF(C57="","",IF(AND(K57&lt;&gt;"",L57=""),"Falta el costo",IF(AND(LEFT(I57,6)="Por ov",K57&lt;&gt;"",G57=""),"Falta el peso del ovillo",IF(AND(A57="",B57=""),"Falta la categoría",IF(AND(A57="",I57=""),"Falta cómo se vende",IF(AND(K57&lt;&gt;"",N57="",M57=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n"/>
@@ -3384,6 +3808,10 @@
       <c r="Q58" s="6" t="n"/>
       <c r="R58" s="6" t="n"/>
       <c r="S58" s="6" t="n"/>
+      <c r="T58">
+        <f>IF(C58="","",IF(AND(K58&lt;&gt;"",L58=""),"Falta el costo",IF(AND(LEFT(I58,6)="Por ov",K58&lt;&gt;"",G58=""),"Falta el peso del ovillo",IF(AND(A58="",B58=""),"Falta la categoría",IF(AND(A58="",I58=""),"Falta cómo se vende",IF(AND(K58&lt;&gt;"",N58="",M58=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="11" t="n"/>
@@ -3405,6 +3833,10 @@
       <c r="Q59" s="6" t="n"/>
       <c r="R59" s="6" t="n"/>
       <c r="S59" s="6" t="n"/>
+      <c r="T59">
+        <f>IF(C59="","",IF(AND(K59&lt;&gt;"",L59=""),"Falta el costo",IF(AND(LEFT(I59,6)="Por ov",K59&lt;&gt;"",G59=""),"Falta el peso del ovillo",IF(AND(A59="",B59=""),"Falta la categoría",IF(AND(A59="",I59=""),"Falta cómo se vende",IF(AND(K59&lt;&gt;"",N59="",M59=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n"/>
@@ -3426,6 +3858,10 @@
       <c r="Q60" s="6" t="n"/>
       <c r="R60" s="6" t="n"/>
       <c r="S60" s="6" t="n"/>
+      <c r="T60">
+        <f>IF(C60="","",IF(AND(K60&lt;&gt;"",L60=""),"Falta el costo",IF(AND(LEFT(I60,6)="Por ov",K60&lt;&gt;"",G60=""),"Falta el peso del ovillo",IF(AND(A60="",B60=""),"Falta la categoría",IF(AND(A60="",I60=""),"Falta cómo se vende",IF(AND(K60&lt;&gt;"",N60="",M60=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n"/>
@@ -3447,6 +3883,10 @@
       <c r="Q61" s="6" t="n"/>
       <c r="R61" s="6" t="n"/>
       <c r="S61" s="6" t="n"/>
+      <c r="T61">
+        <f>IF(C61="","",IF(AND(K61&lt;&gt;"",L61=""),"Falta el costo",IF(AND(LEFT(I61,6)="Por ov",K61&lt;&gt;"",G61=""),"Falta el peso del ovillo",IF(AND(A61="",B61=""),"Falta la categoría",IF(AND(A61="",I61=""),"Falta cómo se vende",IF(AND(K61&lt;&gt;"",N61="",M61=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n"/>
@@ -3468,6 +3908,10 @@
       <c r="Q62" s="6" t="n"/>
       <c r="R62" s="6" t="n"/>
       <c r="S62" s="6" t="n"/>
+      <c r="T62">
+        <f>IF(C62="","",IF(AND(K62&lt;&gt;"",L62=""),"Falta el costo",IF(AND(LEFT(I62,6)="Por ov",K62&lt;&gt;"",G62=""),"Falta el peso del ovillo",IF(AND(A62="",B62=""),"Falta la categoría",IF(AND(A62="",I62=""),"Falta cómo se vende",IF(AND(K62&lt;&gt;"",N62="",M62=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n"/>
@@ -3489,6 +3933,10 @@
       <c r="Q63" s="6" t="n"/>
       <c r="R63" s="6" t="n"/>
       <c r="S63" s="6" t="n"/>
+      <c r="T63">
+        <f>IF(C63="","",IF(AND(K63&lt;&gt;"",L63=""),"Falta el costo",IF(AND(LEFT(I63,6)="Por ov",K63&lt;&gt;"",G63=""),"Falta el peso del ovillo",IF(AND(A63="",B63=""),"Falta la categoría",IF(AND(A63="",I63=""),"Falta cómo se vende",IF(AND(K63&lt;&gt;"",N63="",M63=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="11" t="n"/>
@@ -3510,6 +3958,10 @@
       <c r="Q64" s="6" t="n"/>
       <c r="R64" s="6" t="n"/>
       <c r="S64" s="6" t="n"/>
+      <c r="T64">
+        <f>IF(C64="","",IF(AND(K64&lt;&gt;"",L64=""),"Falta el costo",IF(AND(LEFT(I64,6)="Por ov",K64&lt;&gt;"",G64=""),"Falta el peso del ovillo",IF(AND(A64="",B64=""),"Falta la categoría",IF(AND(A64="",I64=""),"Falta cómo se vende",IF(AND(K64&lt;&gt;"",N64="",M64=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="11" t="n"/>
@@ -3531,6 +3983,10 @@
       <c r="Q65" s="6" t="n"/>
       <c r="R65" s="6" t="n"/>
       <c r="S65" s="6" t="n"/>
+      <c r="T65">
+        <f>IF(C65="","",IF(AND(K65&lt;&gt;"",L65=""),"Falta el costo",IF(AND(LEFT(I65,6)="Por ov",K65&lt;&gt;"",G65=""),"Falta el peso del ovillo",IF(AND(A65="",B65=""),"Falta la categoría",IF(AND(A65="",I65=""),"Falta cómo se vende",IF(AND(K65&lt;&gt;"",N65="",M65=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="11" t="n"/>
@@ -3552,6 +4008,10 @@
       <c r="Q66" s="6" t="n"/>
       <c r="R66" s="6" t="n"/>
       <c r="S66" s="6" t="n"/>
+      <c r="T66">
+        <f>IF(C66="","",IF(AND(K66&lt;&gt;"",L66=""),"Falta el costo",IF(AND(LEFT(I66,6)="Por ov",K66&lt;&gt;"",G66=""),"Falta el peso del ovillo",IF(AND(A66="",B66=""),"Falta la categoría",IF(AND(A66="",I66=""),"Falta cómo se vende",IF(AND(K66&lt;&gt;"",N66="",M66=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="11" t="n"/>
@@ -3573,6 +4033,10 @@
       <c r="Q67" s="6" t="n"/>
       <c r="R67" s="6" t="n"/>
       <c r="S67" s="6" t="n"/>
+      <c r="T67">
+        <f>IF(C67="","",IF(AND(K67&lt;&gt;"",L67=""),"Falta el costo",IF(AND(LEFT(I67,6)="Por ov",K67&lt;&gt;"",G67=""),"Falta el peso del ovillo",IF(AND(A67="",B67=""),"Falta la categoría",IF(AND(A67="",I67=""),"Falta cómo se vende",IF(AND(K67&lt;&gt;"",N67="",M67=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="11" t="n"/>
@@ -3594,6 +4058,10 @@
       <c r="Q68" s="6" t="n"/>
       <c r="R68" s="6" t="n"/>
       <c r="S68" s="6" t="n"/>
+      <c r="T68">
+        <f>IF(C68="","",IF(AND(K68&lt;&gt;"",L68=""),"Falta el costo",IF(AND(LEFT(I68,6)="Por ov",K68&lt;&gt;"",G68=""),"Falta el peso del ovillo",IF(AND(A68="",B68=""),"Falta la categoría",IF(AND(A68="",I68=""),"Falta cómo se vende",IF(AND(K68&lt;&gt;"",N68="",M68=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="11" t="n"/>
@@ -3615,6 +4083,10 @@
       <c r="Q69" s="6" t="n"/>
       <c r="R69" s="6" t="n"/>
       <c r="S69" s="6" t="n"/>
+      <c r="T69">
+        <f>IF(C69="","",IF(AND(K69&lt;&gt;"",L69=""),"Falta el costo",IF(AND(LEFT(I69,6)="Por ov",K69&lt;&gt;"",G69=""),"Falta el peso del ovillo",IF(AND(A69="",B69=""),"Falta la categoría",IF(AND(A69="",I69=""),"Falta cómo se vende",IF(AND(K69&lt;&gt;"",N69="",M69=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="11" t="n"/>
@@ -3636,6 +4108,10 @@
       <c r="Q70" s="6" t="n"/>
       <c r="R70" s="6" t="n"/>
       <c r="S70" s="6" t="n"/>
+      <c r="T70">
+        <f>IF(C70="","",IF(AND(K70&lt;&gt;"",L70=""),"Falta el costo",IF(AND(LEFT(I70,6)="Por ov",K70&lt;&gt;"",G70=""),"Falta el peso del ovillo",IF(AND(A70="",B70=""),"Falta la categoría",IF(AND(A70="",I70=""),"Falta cómo se vende",IF(AND(K70&lt;&gt;"",N70="",M70=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="11" t="n"/>
@@ -3657,6 +4133,10 @@
       <c r="Q71" s="6" t="n"/>
       <c r="R71" s="6" t="n"/>
       <c r="S71" s="6" t="n"/>
+      <c r="T71">
+        <f>IF(C71="","",IF(AND(K71&lt;&gt;"",L71=""),"Falta el costo",IF(AND(LEFT(I71,6)="Por ov",K71&lt;&gt;"",G71=""),"Falta el peso del ovillo",IF(AND(A71="",B71=""),"Falta la categoría",IF(AND(A71="",I71=""),"Falta cómo se vende",IF(AND(K71&lt;&gt;"",N71="",M71=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="11" t="n"/>
@@ -3678,6 +4158,10 @@
       <c r="Q72" s="6" t="n"/>
       <c r="R72" s="6" t="n"/>
       <c r="S72" s="6" t="n"/>
+      <c r="T72">
+        <f>IF(C72="","",IF(AND(K72&lt;&gt;"",L72=""),"Falta el costo",IF(AND(LEFT(I72,6)="Por ov",K72&lt;&gt;"",G72=""),"Falta el peso del ovillo",IF(AND(A72="",B72=""),"Falta la categoría",IF(AND(A72="",I72=""),"Falta cómo se vende",IF(AND(K72&lt;&gt;"",N72="",M72=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="11" t="n"/>
@@ -3699,6 +4183,10 @@
       <c r="Q73" s="6" t="n"/>
       <c r="R73" s="6" t="n"/>
       <c r="S73" s="6" t="n"/>
+      <c r="T73">
+        <f>IF(C73="","",IF(AND(K73&lt;&gt;"",L73=""),"Falta el costo",IF(AND(LEFT(I73,6)="Por ov",K73&lt;&gt;"",G73=""),"Falta el peso del ovillo",IF(AND(A73="",B73=""),"Falta la categoría",IF(AND(A73="",I73=""),"Falta cómo se vende",IF(AND(K73&lt;&gt;"",N73="",M73=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="11" t="n"/>
@@ -3720,6 +4208,10 @@
       <c r="Q74" s="6" t="n"/>
       <c r="R74" s="6" t="n"/>
       <c r="S74" s="6" t="n"/>
+      <c r="T74">
+        <f>IF(C74="","",IF(AND(K74&lt;&gt;"",L74=""),"Falta el costo",IF(AND(LEFT(I74,6)="Por ov",K74&lt;&gt;"",G74=""),"Falta el peso del ovillo",IF(AND(A74="",B74=""),"Falta la categoría",IF(AND(A74="",I74=""),"Falta cómo se vende",IF(AND(K74&lt;&gt;"",N74="",M74=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="11" t="n"/>
@@ -3741,26 +4233,1913 @@
       <c r="Q75" s="6" t="n"/>
       <c r="R75" s="6" t="n"/>
       <c r="S75" s="6" t="n"/>
+      <c r="T75">
+        <f>IF(C75="","",IF(AND(K75&lt;&gt;"",L75=""),"Falta el costo",IF(AND(LEFT(I75,6)="Por ov",K75&lt;&gt;"",G75=""),"Falta el peso del ovillo",IF(AND(A75="",B75=""),"Falta la categoría",IF(AND(A75="",I75=""),"Falta cómo se vende",IF(AND(K75&lt;&gt;"",N75="",M75=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="n"/>
+      <c r="B76" s="6" t="n"/>
+      <c r="C76" s="6" t="n"/>
+      <c r="D76" s="6" t="n"/>
+      <c r="E76" s="6" t="n"/>
+      <c r="F76" s="6" t="n"/>
+      <c r="G76" s="6" t="n"/>
+      <c r="H76" s="6" t="n"/>
+      <c r="I76" s="6" t="n"/>
+      <c r="J76" s="6" t="n"/>
+      <c r="K76" s="7" t="n"/>
+      <c r="L76" s="8" t="n"/>
+      <c r="M76" s="6" t="n"/>
+      <c r="N76" s="6" t="n"/>
+      <c r="O76" s="9" t="n"/>
+      <c r="P76" s="6" t="n"/>
+      <c r="Q76" s="6" t="n"/>
+      <c r="R76" s="6" t="n"/>
+      <c r="S76" s="6" t="n"/>
+      <c r="T76">
+        <f>IF(C76="","",IF(AND(K76&lt;&gt;"",L76=""),"Falta el costo",IF(AND(LEFT(I76,6)="Por ov",K76&lt;&gt;"",G76=""),"Falta el peso del ovillo",IF(AND(A76="",B76=""),"Falta la categoría",IF(AND(A76="",I76=""),"Falta cómo se vende",IF(AND(K76&lt;&gt;"",N76="",M76=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="11" t="n"/>
+      <c r="B77" s="6" t="n"/>
+      <c r="C77" s="6" t="n"/>
+      <c r="D77" s="6" t="n"/>
+      <c r="E77" s="6" t="n"/>
+      <c r="F77" s="6" t="n"/>
+      <c r="G77" s="6" t="n"/>
+      <c r="H77" s="6" t="n"/>
+      <c r="I77" s="6" t="n"/>
+      <c r="J77" s="6" t="n"/>
+      <c r="K77" s="7" t="n"/>
+      <c r="L77" s="8" t="n"/>
+      <c r="M77" s="6" t="n"/>
+      <c r="N77" s="6" t="n"/>
+      <c r="O77" s="9" t="n"/>
+      <c r="P77" s="6" t="n"/>
+      <c r="Q77" s="6" t="n"/>
+      <c r="R77" s="6" t="n"/>
+      <c r="S77" s="6" t="n"/>
+      <c r="T77">
+        <f>IF(C77="","",IF(AND(K77&lt;&gt;"",L77=""),"Falta el costo",IF(AND(LEFT(I77,6)="Por ov",K77&lt;&gt;"",G77=""),"Falta el peso del ovillo",IF(AND(A77="",B77=""),"Falta la categoría",IF(AND(A77="",I77=""),"Falta cómo se vende",IF(AND(K77&lt;&gt;"",N77="",M77=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="n"/>
+      <c r="B78" s="6" t="n"/>
+      <c r="C78" s="6" t="n"/>
+      <c r="D78" s="6" t="n"/>
+      <c r="E78" s="6" t="n"/>
+      <c r="F78" s="6" t="n"/>
+      <c r="G78" s="6" t="n"/>
+      <c r="H78" s="6" t="n"/>
+      <c r="I78" s="6" t="n"/>
+      <c r="J78" s="6" t="n"/>
+      <c r="K78" s="7" t="n"/>
+      <c r="L78" s="8" t="n"/>
+      <c r="M78" s="6" t="n"/>
+      <c r="N78" s="6" t="n"/>
+      <c r="O78" s="9" t="n"/>
+      <c r="P78" s="6" t="n"/>
+      <c r="Q78" s="6" t="n"/>
+      <c r="R78" s="6" t="n"/>
+      <c r="S78" s="6" t="n"/>
+      <c r="T78">
+        <f>IF(C78="","",IF(AND(K78&lt;&gt;"",L78=""),"Falta el costo",IF(AND(LEFT(I78,6)="Por ov",K78&lt;&gt;"",G78=""),"Falta el peso del ovillo",IF(AND(A78="",B78=""),"Falta la categoría",IF(AND(A78="",I78=""),"Falta cómo se vende",IF(AND(K78&lt;&gt;"",N78="",M78=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="11" t="n"/>
+      <c r="B79" s="6" t="n"/>
+      <c r="C79" s="6" t="n"/>
+      <c r="D79" s="6" t="n"/>
+      <c r="E79" s="6" t="n"/>
+      <c r="F79" s="6" t="n"/>
+      <c r="G79" s="6" t="n"/>
+      <c r="H79" s="6" t="n"/>
+      <c r="I79" s="6" t="n"/>
+      <c r="J79" s="6" t="n"/>
+      <c r="K79" s="7" t="n"/>
+      <c r="L79" s="8" t="n"/>
+      <c r="M79" s="6" t="n"/>
+      <c r="N79" s="6" t="n"/>
+      <c r="O79" s="9" t="n"/>
+      <c r="P79" s="6" t="n"/>
+      <c r="Q79" s="6" t="n"/>
+      <c r="R79" s="6" t="n"/>
+      <c r="S79" s="6" t="n"/>
+      <c r="T79">
+        <f>IF(C79="","",IF(AND(K79&lt;&gt;"",L79=""),"Falta el costo",IF(AND(LEFT(I79,6)="Por ov",K79&lt;&gt;"",G79=""),"Falta el peso del ovillo",IF(AND(A79="",B79=""),"Falta la categoría",IF(AND(A79="",I79=""),"Falta cómo se vende",IF(AND(K79&lt;&gt;"",N79="",M79=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="n"/>
+      <c r="B80" s="6" t="n"/>
+      <c r="C80" s="6" t="n"/>
+      <c r="D80" s="6" t="n"/>
+      <c r="E80" s="6" t="n"/>
+      <c r="F80" s="6" t="n"/>
+      <c r="G80" s="6" t="n"/>
+      <c r="H80" s="6" t="n"/>
+      <c r="I80" s="6" t="n"/>
+      <c r="J80" s="6" t="n"/>
+      <c r="K80" s="7" t="n"/>
+      <c r="L80" s="8" t="n"/>
+      <c r="M80" s="6" t="n"/>
+      <c r="N80" s="6" t="n"/>
+      <c r="O80" s="9" t="n"/>
+      <c r="P80" s="6" t="n"/>
+      <c r="Q80" s="6" t="n"/>
+      <c r="R80" s="6" t="n"/>
+      <c r="S80" s="6" t="n"/>
+      <c r="T80">
+        <f>IF(C80="","",IF(AND(K80&lt;&gt;"",L80=""),"Falta el costo",IF(AND(LEFT(I80,6)="Por ov",K80&lt;&gt;"",G80=""),"Falta el peso del ovillo",IF(AND(A80="",B80=""),"Falta la categoría",IF(AND(A80="",I80=""),"Falta cómo se vende",IF(AND(K80&lt;&gt;"",N80="",M80=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="11" t="n"/>
+      <c r="B81" s="6" t="n"/>
+      <c r="C81" s="6" t="n"/>
+      <c r="D81" s="6" t="n"/>
+      <c r="E81" s="6" t="n"/>
+      <c r="F81" s="6" t="n"/>
+      <c r="G81" s="6" t="n"/>
+      <c r="H81" s="6" t="n"/>
+      <c r="I81" s="6" t="n"/>
+      <c r="J81" s="6" t="n"/>
+      <c r="K81" s="7" t="n"/>
+      <c r="L81" s="8" t="n"/>
+      <c r="M81" s="6" t="n"/>
+      <c r="N81" s="6" t="n"/>
+      <c r="O81" s="9" t="n"/>
+      <c r="P81" s="6" t="n"/>
+      <c r="Q81" s="6" t="n"/>
+      <c r="R81" s="6" t="n"/>
+      <c r="S81" s="6" t="n"/>
+      <c r="T81">
+        <f>IF(C81="","",IF(AND(K81&lt;&gt;"",L81=""),"Falta el costo",IF(AND(LEFT(I81,6)="Por ov",K81&lt;&gt;"",G81=""),"Falta el peso del ovillo",IF(AND(A81="",B81=""),"Falta la categoría",IF(AND(A81="",I81=""),"Falta cómo se vende",IF(AND(K81&lt;&gt;"",N81="",M81=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="n"/>
+      <c r="B82" s="6" t="n"/>
+      <c r="C82" s="6" t="n"/>
+      <c r="D82" s="6" t="n"/>
+      <c r="E82" s="6" t="n"/>
+      <c r="F82" s="6" t="n"/>
+      <c r="G82" s="6" t="n"/>
+      <c r="H82" s="6" t="n"/>
+      <c r="I82" s="6" t="n"/>
+      <c r="J82" s="6" t="n"/>
+      <c r="K82" s="7" t="n"/>
+      <c r="L82" s="8" t="n"/>
+      <c r="M82" s="6" t="n"/>
+      <c r="N82" s="6" t="n"/>
+      <c r="O82" s="9" t="n"/>
+      <c r="P82" s="6" t="n"/>
+      <c r="Q82" s="6" t="n"/>
+      <c r="R82" s="6" t="n"/>
+      <c r="S82" s="6" t="n"/>
+      <c r="T82">
+        <f>IF(C82="","",IF(AND(K82&lt;&gt;"",L82=""),"Falta el costo",IF(AND(LEFT(I82,6)="Por ov",K82&lt;&gt;"",G82=""),"Falta el peso del ovillo",IF(AND(A82="",B82=""),"Falta la categoría",IF(AND(A82="",I82=""),"Falta cómo se vende",IF(AND(K82&lt;&gt;"",N82="",M82=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="11" t="n"/>
+      <c r="B83" s="6" t="n"/>
+      <c r="C83" s="6" t="n"/>
+      <c r="D83" s="6" t="n"/>
+      <c r="E83" s="6" t="n"/>
+      <c r="F83" s="6" t="n"/>
+      <c r="G83" s="6" t="n"/>
+      <c r="H83" s="6" t="n"/>
+      <c r="I83" s="6" t="n"/>
+      <c r="J83" s="6" t="n"/>
+      <c r="K83" s="7" t="n"/>
+      <c r="L83" s="8" t="n"/>
+      <c r="M83" s="6" t="n"/>
+      <c r="N83" s="6" t="n"/>
+      <c r="O83" s="9" t="n"/>
+      <c r="P83" s="6" t="n"/>
+      <c r="Q83" s="6" t="n"/>
+      <c r="R83" s="6" t="n"/>
+      <c r="S83" s="6" t="n"/>
+      <c r="T83">
+        <f>IF(C83="","",IF(AND(K83&lt;&gt;"",L83=""),"Falta el costo",IF(AND(LEFT(I83,6)="Por ov",K83&lt;&gt;"",G83=""),"Falta el peso del ovillo",IF(AND(A83="",B83=""),"Falta la categoría",IF(AND(A83="",I83=""),"Falta cómo se vende",IF(AND(K83&lt;&gt;"",N83="",M83=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="n"/>
+      <c r="B84" s="6" t="n"/>
+      <c r="C84" s="6" t="n"/>
+      <c r="D84" s="6" t="n"/>
+      <c r="E84" s="6" t="n"/>
+      <c r="F84" s="6" t="n"/>
+      <c r="G84" s="6" t="n"/>
+      <c r="H84" s="6" t="n"/>
+      <c r="I84" s="6" t="n"/>
+      <c r="J84" s="6" t="n"/>
+      <c r="K84" s="7" t="n"/>
+      <c r="L84" s="8" t="n"/>
+      <c r="M84" s="6" t="n"/>
+      <c r="N84" s="6" t="n"/>
+      <c r="O84" s="9" t="n"/>
+      <c r="P84" s="6" t="n"/>
+      <c r="Q84" s="6" t="n"/>
+      <c r="R84" s="6" t="n"/>
+      <c r="S84" s="6" t="n"/>
+      <c r="T84">
+        <f>IF(C84="","",IF(AND(K84&lt;&gt;"",L84=""),"Falta el costo",IF(AND(LEFT(I84,6)="Por ov",K84&lt;&gt;"",G84=""),"Falta el peso del ovillo",IF(AND(A84="",B84=""),"Falta la categoría",IF(AND(A84="",I84=""),"Falta cómo se vende",IF(AND(K84&lt;&gt;"",N84="",M84=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="11" t="n"/>
+      <c r="B85" s="6" t="n"/>
+      <c r="C85" s="6" t="n"/>
+      <c r="D85" s="6" t="n"/>
+      <c r="E85" s="6" t="n"/>
+      <c r="F85" s="6" t="n"/>
+      <c r="G85" s="6" t="n"/>
+      <c r="H85" s="6" t="n"/>
+      <c r="I85" s="6" t="n"/>
+      <c r="J85" s="6" t="n"/>
+      <c r="K85" s="7" t="n"/>
+      <c r="L85" s="8" t="n"/>
+      <c r="M85" s="6" t="n"/>
+      <c r="N85" s="6" t="n"/>
+      <c r="O85" s="9" t="n"/>
+      <c r="P85" s="6" t="n"/>
+      <c r="Q85" s="6" t="n"/>
+      <c r="R85" s="6" t="n"/>
+      <c r="S85" s="6" t="n"/>
+      <c r="T85">
+        <f>IF(C85="","",IF(AND(K85&lt;&gt;"",L85=""),"Falta el costo",IF(AND(LEFT(I85,6)="Por ov",K85&lt;&gt;"",G85=""),"Falta el peso del ovillo",IF(AND(A85="",B85=""),"Falta la categoría",IF(AND(A85="",I85=""),"Falta cómo se vende",IF(AND(K85&lt;&gt;"",N85="",M85=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="11" t="n"/>
+      <c r="B86" s="6" t="n"/>
+      <c r="C86" s="6" t="n"/>
+      <c r="D86" s="6" t="n"/>
+      <c r="E86" s="6" t="n"/>
+      <c r="F86" s="6" t="n"/>
+      <c r="G86" s="6" t="n"/>
+      <c r="H86" s="6" t="n"/>
+      <c r="I86" s="6" t="n"/>
+      <c r="J86" s="6" t="n"/>
+      <c r="K86" s="7" t="n"/>
+      <c r="L86" s="8" t="n"/>
+      <c r="M86" s="6" t="n"/>
+      <c r="N86" s="6" t="n"/>
+      <c r="O86" s="9" t="n"/>
+      <c r="P86" s="6" t="n"/>
+      <c r="Q86" s="6" t="n"/>
+      <c r="R86" s="6" t="n"/>
+      <c r="S86" s="6" t="n"/>
+      <c r="T86">
+        <f>IF(C86="","",IF(AND(K86&lt;&gt;"",L86=""),"Falta el costo",IF(AND(LEFT(I86,6)="Por ov",K86&lt;&gt;"",G86=""),"Falta el peso del ovillo",IF(AND(A86="",B86=""),"Falta la categoría",IF(AND(A86="",I86=""),"Falta cómo se vende",IF(AND(K86&lt;&gt;"",N86="",M86=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="11" t="n"/>
+      <c r="B87" s="6" t="n"/>
+      <c r="C87" s="6" t="n"/>
+      <c r="D87" s="6" t="n"/>
+      <c r="E87" s="6" t="n"/>
+      <c r="F87" s="6" t="n"/>
+      <c r="G87" s="6" t="n"/>
+      <c r="H87" s="6" t="n"/>
+      <c r="I87" s="6" t="n"/>
+      <c r="J87" s="6" t="n"/>
+      <c r="K87" s="7" t="n"/>
+      <c r="L87" s="8" t="n"/>
+      <c r="M87" s="6" t="n"/>
+      <c r="N87" s="6" t="n"/>
+      <c r="O87" s="9" t="n"/>
+      <c r="P87" s="6" t="n"/>
+      <c r="Q87" s="6" t="n"/>
+      <c r="R87" s="6" t="n"/>
+      <c r="S87" s="6" t="n"/>
+      <c r="T87">
+        <f>IF(C87="","",IF(AND(K87&lt;&gt;"",L87=""),"Falta el costo",IF(AND(LEFT(I87,6)="Por ov",K87&lt;&gt;"",G87=""),"Falta el peso del ovillo",IF(AND(A87="",B87=""),"Falta la categoría",IF(AND(A87="",I87=""),"Falta cómo se vende",IF(AND(K87&lt;&gt;"",N87="",M87=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="11" t="n"/>
+      <c r="B88" s="6" t="n"/>
+      <c r="C88" s="6" t="n"/>
+      <c r="D88" s="6" t="n"/>
+      <c r="E88" s="6" t="n"/>
+      <c r="F88" s="6" t="n"/>
+      <c r="G88" s="6" t="n"/>
+      <c r="H88" s="6" t="n"/>
+      <c r="I88" s="6" t="n"/>
+      <c r="J88" s="6" t="n"/>
+      <c r="K88" s="7" t="n"/>
+      <c r="L88" s="8" t="n"/>
+      <c r="M88" s="6" t="n"/>
+      <c r="N88" s="6" t="n"/>
+      <c r="O88" s="9" t="n"/>
+      <c r="P88" s="6" t="n"/>
+      <c r="Q88" s="6" t="n"/>
+      <c r="R88" s="6" t="n"/>
+      <c r="S88" s="6" t="n"/>
+      <c r="T88">
+        <f>IF(C88="","",IF(AND(K88&lt;&gt;"",L88=""),"Falta el costo",IF(AND(LEFT(I88,6)="Por ov",K88&lt;&gt;"",G88=""),"Falta el peso del ovillo",IF(AND(A88="",B88=""),"Falta la categoría",IF(AND(A88="",I88=""),"Falta cómo se vende",IF(AND(K88&lt;&gt;"",N88="",M88=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="11" t="n"/>
+      <c r="B89" s="6" t="n"/>
+      <c r="C89" s="6" t="n"/>
+      <c r="D89" s="6" t="n"/>
+      <c r="E89" s="6" t="n"/>
+      <c r="F89" s="6" t="n"/>
+      <c r="G89" s="6" t="n"/>
+      <c r="H89" s="6" t="n"/>
+      <c r="I89" s="6" t="n"/>
+      <c r="J89" s="6" t="n"/>
+      <c r="K89" s="7" t="n"/>
+      <c r="L89" s="8" t="n"/>
+      <c r="M89" s="6" t="n"/>
+      <c r="N89" s="6" t="n"/>
+      <c r="O89" s="9" t="n"/>
+      <c r="P89" s="6" t="n"/>
+      <c r="Q89" s="6" t="n"/>
+      <c r="R89" s="6" t="n"/>
+      <c r="S89" s="6" t="n"/>
+      <c r="T89">
+        <f>IF(C89="","",IF(AND(K89&lt;&gt;"",L89=""),"Falta el costo",IF(AND(LEFT(I89,6)="Por ov",K89&lt;&gt;"",G89=""),"Falta el peso del ovillo",IF(AND(A89="",B89=""),"Falta la categoría",IF(AND(A89="",I89=""),"Falta cómo se vende",IF(AND(K89&lt;&gt;"",N89="",M89=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="11" t="n"/>
+      <c r="B90" s="6" t="n"/>
+      <c r="C90" s="6" t="n"/>
+      <c r="D90" s="6" t="n"/>
+      <c r="E90" s="6" t="n"/>
+      <c r="F90" s="6" t="n"/>
+      <c r="G90" s="6" t="n"/>
+      <c r="H90" s="6" t="n"/>
+      <c r="I90" s="6" t="n"/>
+      <c r="J90" s="6" t="n"/>
+      <c r="K90" s="7" t="n"/>
+      <c r="L90" s="8" t="n"/>
+      <c r="M90" s="6" t="n"/>
+      <c r="N90" s="6" t="n"/>
+      <c r="O90" s="9" t="n"/>
+      <c r="P90" s="6" t="n"/>
+      <c r="Q90" s="6" t="n"/>
+      <c r="R90" s="6" t="n"/>
+      <c r="S90" s="6" t="n"/>
+      <c r="T90">
+        <f>IF(C90="","",IF(AND(K90&lt;&gt;"",L90=""),"Falta el costo",IF(AND(LEFT(I90,6)="Por ov",K90&lt;&gt;"",G90=""),"Falta el peso del ovillo",IF(AND(A90="",B90=""),"Falta la categoría",IF(AND(A90="",I90=""),"Falta cómo se vende",IF(AND(K90&lt;&gt;"",N90="",M90=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="11" t="n"/>
+      <c r="B91" s="6" t="n"/>
+      <c r="C91" s="6" t="n"/>
+      <c r="D91" s="6" t="n"/>
+      <c r="E91" s="6" t="n"/>
+      <c r="F91" s="6" t="n"/>
+      <c r="G91" s="6" t="n"/>
+      <c r="H91" s="6" t="n"/>
+      <c r="I91" s="6" t="n"/>
+      <c r="J91" s="6" t="n"/>
+      <c r="K91" s="7" t="n"/>
+      <c r="L91" s="8" t="n"/>
+      <c r="M91" s="6" t="n"/>
+      <c r="N91" s="6" t="n"/>
+      <c r="O91" s="9" t="n"/>
+      <c r="P91" s="6" t="n"/>
+      <c r="Q91" s="6" t="n"/>
+      <c r="R91" s="6" t="n"/>
+      <c r="S91" s="6" t="n"/>
+      <c r="T91">
+        <f>IF(C91="","",IF(AND(K91&lt;&gt;"",L91=""),"Falta el costo",IF(AND(LEFT(I91,6)="Por ov",K91&lt;&gt;"",G91=""),"Falta el peso del ovillo",IF(AND(A91="",B91=""),"Falta la categoría",IF(AND(A91="",I91=""),"Falta cómo se vende",IF(AND(K91&lt;&gt;"",N91="",M91=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="11" t="n"/>
+      <c r="B92" s="6" t="n"/>
+      <c r="C92" s="6" t="n"/>
+      <c r="D92" s="6" t="n"/>
+      <c r="E92" s="6" t="n"/>
+      <c r="F92" s="6" t="n"/>
+      <c r="G92" s="6" t="n"/>
+      <c r="H92" s="6" t="n"/>
+      <c r="I92" s="6" t="n"/>
+      <c r="J92" s="6" t="n"/>
+      <c r="K92" s="7" t="n"/>
+      <c r="L92" s="8" t="n"/>
+      <c r="M92" s="6" t="n"/>
+      <c r="N92" s="6" t="n"/>
+      <c r="O92" s="9" t="n"/>
+      <c r="P92" s="6" t="n"/>
+      <c r="Q92" s="6" t="n"/>
+      <c r="R92" s="6" t="n"/>
+      <c r="S92" s="6" t="n"/>
+      <c r="T92">
+        <f>IF(C92="","",IF(AND(K92&lt;&gt;"",L92=""),"Falta el costo",IF(AND(LEFT(I92,6)="Por ov",K92&lt;&gt;"",G92=""),"Falta el peso del ovillo",IF(AND(A92="",B92=""),"Falta la categoría",IF(AND(A92="",I92=""),"Falta cómo se vende",IF(AND(K92&lt;&gt;"",N92="",M92=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="11" t="n"/>
+      <c r="B93" s="6" t="n"/>
+      <c r="C93" s="6" t="n"/>
+      <c r="D93" s="6" t="n"/>
+      <c r="E93" s="6" t="n"/>
+      <c r="F93" s="6" t="n"/>
+      <c r="G93" s="6" t="n"/>
+      <c r="H93" s="6" t="n"/>
+      <c r="I93" s="6" t="n"/>
+      <c r="J93" s="6" t="n"/>
+      <c r="K93" s="7" t="n"/>
+      <c r="L93" s="8" t="n"/>
+      <c r="M93" s="6" t="n"/>
+      <c r="N93" s="6" t="n"/>
+      <c r="O93" s="9" t="n"/>
+      <c r="P93" s="6" t="n"/>
+      <c r="Q93" s="6" t="n"/>
+      <c r="R93" s="6" t="n"/>
+      <c r="S93" s="6" t="n"/>
+      <c r="T93">
+        <f>IF(C93="","",IF(AND(K93&lt;&gt;"",L93=""),"Falta el costo",IF(AND(LEFT(I93,6)="Por ov",K93&lt;&gt;"",G93=""),"Falta el peso del ovillo",IF(AND(A93="",B93=""),"Falta la categoría",IF(AND(A93="",I93=""),"Falta cómo se vende",IF(AND(K93&lt;&gt;"",N93="",M93=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="11" t="n"/>
+      <c r="B94" s="6" t="n"/>
+      <c r="C94" s="6" t="n"/>
+      <c r="D94" s="6" t="n"/>
+      <c r="E94" s="6" t="n"/>
+      <c r="F94" s="6" t="n"/>
+      <c r="G94" s="6" t="n"/>
+      <c r="H94" s="6" t="n"/>
+      <c r="I94" s="6" t="n"/>
+      <c r="J94" s="6" t="n"/>
+      <c r="K94" s="7" t="n"/>
+      <c r="L94" s="8" t="n"/>
+      <c r="M94" s="6" t="n"/>
+      <c r="N94" s="6" t="n"/>
+      <c r="O94" s="9" t="n"/>
+      <c r="P94" s="6" t="n"/>
+      <c r="Q94" s="6" t="n"/>
+      <c r="R94" s="6" t="n"/>
+      <c r="S94" s="6" t="n"/>
+      <c r="T94">
+        <f>IF(C94="","",IF(AND(K94&lt;&gt;"",L94=""),"Falta el costo",IF(AND(LEFT(I94,6)="Por ov",K94&lt;&gt;"",G94=""),"Falta el peso del ovillo",IF(AND(A94="",B94=""),"Falta la categoría",IF(AND(A94="",I94=""),"Falta cómo se vende",IF(AND(K94&lt;&gt;"",N94="",M94=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="11" t="n"/>
+      <c r="B95" s="6" t="n"/>
+      <c r="C95" s="6" t="n"/>
+      <c r="D95" s="6" t="n"/>
+      <c r="E95" s="6" t="n"/>
+      <c r="F95" s="6" t="n"/>
+      <c r="G95" s="6" t="n"/>
+      <c r="H95" s="6" t="n"/>
+      <c r="I95" s="6" t="n"/>
+      <c r="J95" s="6" t="n"/>
+      <c r="K95" s="7" t="n"/>
+      <c r="L95" s="8" t="n"/>
+      <c r="M95" s="6" t="n"/>
+      <c r="N95" s="6" t="n"/>
+      <c r="O95" s="9" t="n"/>
+      <c r="P95" s="6" t="n"/>
+      <c r="Q95" s="6" t="n"/>
+      <c r="R95" s="6" t="n"/>
+      <c r="S95" s="6" t="n"/>
+      <c r="T95">
+        <f>IF(C95="","",IF(AND(K95&lt;&gt;"",L95=""),"Falta el costo",IF(AND(LEFT(I95,6)="Por ov",K95&lt;&gt;"",G95=""),"Falta el peso del ovillo",IF(AND(A95="",B95=""),"Falta la categoría",IF(AND(A95="",I95=""),"Falta cómo se vende",IF(AND(K95&lt;&gt;"",N95="",M95=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="11" t="n"/>
+      <c r="B96" s="6" t="n"/>
+      <c r="C96" s="6" t="n"/>
+      <c r="D96" s="6" t="n"/>
+      <c r="E96" s="6" t="n"/>
+      <c r="F96" s="6" t="n"/>
+      <c r="G96" s="6" t="n"/>
+      <c r="H96" s="6" t="n"/>
+      <c r="I96" s="6" t="n"/>
+      <c r="J96" s="6" t="n"/>
+      <c r="K96" s="7" t="n"/>
+      <c r="L96" s="8" t="n"/>
+      <c r="M96" s="6" t="n"/>
+      <c r="N96" s="6" t="n"/>
+      <c r="O96" s="9" t="n"/>
+      <c r="P96" s="6" t="n"/>
+      <c r="Q96" s="6" t="n"/>
+      <c r="R96" s="6" t="n"/>
+      <c r="S96" s="6" t="n"/>
+      <c r="T96">
+        <f>IF(C96="","",IF(AND(K96&lt;&gt;"",L96=""),"Falta el costo",IF(AND(LEFT(I96,6)="Por ov",K96&lt;&gt;"",G96=""),"Falta el peso del ovillo",IF(AND(A96="",B96=""),"Falta la categoría",IF(AND(A96="",I96=""),"Falta cómo se vende",IF(AND(K96&lt;&gt;"",N96="",M96=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="11" t="n"/>
+      <c r="B97" s="6" t="n"/>
+      <c r="C97" s="6" t="n"/>
+      <c r="D97" s="6" t="n"/>
+      <c r="E97" s="6" t="n"/>
+      <c r="F97" s="6" t="n"/>
+      <c r="G97" s="6" t="n"/>
+      <c r="H97" s="6" t="n"/>
+      <c r="I97" s="6" t="n"/>
+      <c r="J97" s="6" t="n"/>
+      <c r="K97" s="7" t="n"/>
+      <c r="L97" s="8" t="n"/>
+      <c r="M97" s="6" t="n"/>
+      <c r="N97" s="6" t="n"/>
+      <c r="O97" s="9" t="n"/>
+      <c r="P97" s="6" t="n"/>
+      <c r="Q97" s="6" t="n"/>
+      <c r="R97" s="6" t="n"/>
+      <c r="S97" s="6" t="n"/>
+      <c r="T97">
+        <f>IF(C97="","",IF(AND(K97&lt;&gt;"",L97=""),"Falta el costo",IF(AND(LEFT(I97,6)="Por ov",K97&lt;&gt;"",G97=""),"Falta el peso del ovillo",IF(AND(A97="",B97=""),"Falta la categoría",IF(AND(A97="",I97=""),"Falta cómo se vende",IF(AND(K97&lt;&gt;"",N97="",M97=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="11" t="n"/>
+      <c r="B98" s="6" t="n"/>
+      <c r="C98" s="6" t="n"/>
+      <c r="D98" s="6" t="n"/>
+      <c r="E98" s="6" t="n"/>
+      <c r="F98" s="6" t="n"/>
+      <c r="G98" s="6" t="n"/>
+      <c r="H98" s="6" t="n"/>
+      <c r="I98" s="6" t="n"/>
+      <c r="J98" s="6" t="n"/>
+      <c r="K98" s="7" t="n"/>
+      <c r="L98" s="8" t="n"/>
+      <c r="M98" s="6" t="n"/>
+      <c r="N98" s="6" t="n"/>
+      <c r="O98" s="9" t="n"/>
+      <c r="P98" s="6" t="n"/>
+      <c r="Q98" s="6" t="n"/>
+      <c r="R98" s="6" t="n"/>
+      <c r="S98" s="6" t="n"/>
+      <c r="T98">
+        <f>IF(C98="","",IF(AND(K98&lt;&gt;"",L98=""),"Falta el costo",IF(AND(LEFT(I98,6)="Por ov",K98&lt;&gt;"",G98=""),"Falta el peso del ovillo",IF(AND(A98="",B98=""),"Falta la categoría",IF(AND(A98="",I98=""),"Falta cómo se vende",IF(AND(K98&lt;&gt;"",N98="",M98=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="11" t="n"/>
+      <c r="B99" s="6" t="n"/>
+      <c r="C99" s="6" t="n"/>
+      <c r="D99" s="6" t="n"/>
+      <c r="E99" s="6" t="n"/>
+      <c r="F99" s="6" t="n"/>
+      <c r="G99" s="6" t="n"/>
+      <c r="H99" s="6" t="n"/>
+      <c r="I99" s="6" t="n"/>
+      <c r="J99" s="6" t="n"/>
+      <c r="K99" s="7" t="n"/>
+      <c r="L99" s="8" t="n"/>
+      <c r="M99" s="6" t="n"/>
+      <c r="N99" s="6" t="n"/>
+      <c r="O99" s="9" t="n"/>
+      <c r="P99" s="6" t="n"/>
+      <c r="Q99" s="6" t="n"/>
+      <c r="R99" s="6" t="n"/>
+      <c r="S99" s="6" t="n"/>
+      <c r="T99">
+        <f>IF(C99="","",IF(AND(K99&lt;&gt;"",L99=""),"Falta el costo",IF(AND(LEFT(I99,6)="Por ov",K99&lt;&gt;"",G99=""),"Falta el peso del ovillo",IF(AND(A99="",B99=""),"Falta la categoría",IF(AND(A99="",I99=""),"Falta cómo se vende",IF(AND(K99&lt;&gt;"",N99="",M99=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="11" t="n"/>
+      <c r="B100" s="6" t="n"/>
+      <c r="C100" s="6" t="n"/>
+      <c r="D100" s="6" t="n"/>
+      <c r="E100" s="6" t="n"/>
+      <c r="F100" s="6" t="n"/>
+      <c r="G100" s="6" t="n"/>
+      <c r="H100" s="6" t="n"/>
+      <c r="I100" s="6" t="n"/>
+      <c r="J100" s="6" t="n"/>
+      <c r="K100" s="7" t="n"/>
+      <c r="L100" s="8" t="n"/>
+      <c r="M100" s="6" t="n"/>
+      <c r="N100" s="6" t="n"/>
+      <c r="O100" s="9" t="n"/>
+      <c r="P100" s="6" t="n"/>
+      <c r="Q100" s="6" t="n"/>
+      <c r="R100" s="6" t="n"/>
+      <c r="S100" s="6" t="n"/>
+      <c r="T100">
+        <f>IF(C100="","",IF(AND(K100&lt;&gt;"",L100=""),"Falta el costo",IF(AND(LEFT(I100,6)="Por ov",K100&lt;&gt;"",G100=""),"Falta el peso del ovillo",IF(AND(A100="",B100=""),"Falta la categoría",IF(AND(A100="",I100=""),"Falta cómo se vende",IF(AND(K100&lt;&gt;"",N100="",M100=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="11" t="n"/>
+      <c r="B101" s="6" t="n"/>
+      <c r="C101" s="6" t="n"/>
+      <c r="D101" s="6" t="n"/>
+      <c r="E101" s="6" t="n"/>
+      <c r="F101" s="6" t="n"/>
+      <c r="G101" s="6" t="n"/>
+      <c r="H101" s="6" t="n"/>
+      <c r="I101" s="6" t="n"/>
+      <c r="J101" s="6" t="n"/>
+      <c r="K101" s="7" t="n"/>
+      <c r="L101" s="8" t="n"/>
+      <c r="M101" s="6" t="n"/>
+      <c r="N101" s="6" t="n"/>
+      <c r="O101" s="9" t="n"/>
+      <c r="P101" s="6" t="n"/>
+      <c r="Q101" s="6" t="n"/>
+      <c r="R101" s="6" t="n"/>
+      <c r="S101" s="6" t="n"/>
+      <c r="T101">
+        <f>IF(C101="","",IF(AND(K101&lt;&gt;"",L101=""),"Falta el costo",IF(AND(LEFT(I101,6)="Por ov",K101&lt;&gt;"",G101=""),"Falta el peso del ovillo",IF(AND(A101="",B101=""),"Falta la categoría",IF(AND(A101="",I101=""),"Falta cómo se vende",IF(AND(K101&lt;&gt;"",N101="",M101=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="11" t="n"/>
+      <c r="B102" s="6" t="n"/>
+      <c r="C102" s="6" t="n"/>
+      <c r="D102" s="6" t="n"/>
+      <c r="E102" s="6" t="n"/>
+      <c r="F102" s="6" t="n"/>
+      <c r="G102" s="6" t="n"/>
+      <c r="H102" s="6" t="n"/>
+      <c r="I102" s="6" t="n"/>
+      <c r="J102" s="6" t="n"/>
+      <c r="K102" s="7" t="n"/>
+      <c r="L102" s="8" t="n"/>
+      <c r="M102" s="6" t="n"/>
+      <c r="N102" s="6" t="n"/>
+      <c r="O102" s="9" t="n"/>
+      <c r="P102" s="6" t="n"/>
+      <c r="Q102" s="6" t="n"/>
+      <c r="R102" s="6" t="n"/>
+      <c r="S102" s="6" t="n"/>
+      <c r="T102">
+        <f>IF(C102="","",IF(AND(K102&lt;&gt;"",L102=""),"Falta el costo",IF(AND(LEFT(I102,6)="Por ov",K102&lt;&gt;"",G102=""),"Falta el peso del ovillo",IF(AND(A102="",B102=""),"Falta la categoría",IF(AND(A102="",I102=""),"Falta cómo se vende",IF(AND(K102&lt;&gt;"",N102="",M102=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="11" t="n"/>
+      <c r="B103" s="6" t="n"/>
+      <c r="C103" s="6" t="n"/>
+      <c r="D103" s="6" t="n"/>
+      <c r="E103" s="6" t="n"/>
+      <c r="F103" s="6" t="n"/>
+      <c r="G103" s="6" t="n"/>
+      <c r="H103" s="6" t="n"/>
+      <c r="I103" s="6" t="n"/>
+      <c r="J103" s="6" t="n"/>
+      <c r="K103" s="7" t="n"/>
+      <c r="L103" s="8" t="n"/>
+      <c r="M103" s="6" t="n"/>
+      <c r="N103" s="6" t="n"/>
+      <c r="O103" s="9" t="n"/>
+      <c r="P103" s="6" t="n"/>
+      <c r="Q103" s="6" t="n"/>
+      <c r="R103" s="6" t="n"/>
+      <c r="S103" s="6" t="n"/>
+      <c r="T103">
+        <f>IF(C103="","",IF(AND(K103&lt;&gt;"",L103=""),"Falta el costo",IF(AND(LEFT(I103,6)="Por ov",K103&lt;&gt;"",G103=""),"Falta el peso del ovillo",IF(AND(A103="",B103=""),"Falta la categoría",IF(AND(A103="",I103=""),"Falta cómo se vende",IF(AND(K103&lt;&gt;"",N103="",M103=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="11" t="n"/>
+      <c r="B104" s="6" t="n"/>
+      <c r="C104" s="6" t="n"/>
+      <c r="D104" s="6" t="n"/>
+      <c r="E104" s="6" t="n"/>
+      <c r="F104" s="6" t="n"/>
+      <c r="G104" s="6" t="n"/>
+      <c r="H104" s="6" t="n"/>
+      <c r="I104" s="6" t="n"/>
+      <c r="J104" s="6" t="n"/>
+      <c r="K104" s="7" t="n"/>
+      <c r="L104" s="8" t="n"/>
+      <c r="M104" s="6" t="n"/>
+      <c r="N104" s="6" t="n"/>
+      <c r="O104" s="9" t="n"/>
+      <c r="P104" s="6" t="n"/>
+      <c r="Q104" s="6" t="n"/>
+      <c r="R104" s="6" t="n"/>
+      <c r="S104" s="6" t="n"/>
+      <c r="T104">
+        <f>IF(C104="","",IF(AND(K104&lt;&gt;"",L104=""),"Falta el costo",IF(AND(LEFT(I104,6)="Por ov",K104&lt;&gt;"",G104=""),"Falta el peso del ovillo",IF(AND(A104="",B104=""),"Falta la categoría",IF(AND(A104="",I104=""),"Falta cómo se vende",IF(AND(K104&lt;&gt;"",N104="",M104=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="11" t="n"/>
+      <c r="B105" s="6" t="n"/>
+      <c r="C105" s="6" t="n"/>
+      <c r="D105" s="6" t="n"/>
+      <c r="E105" s="6" t="n"/>
+      <c r="F105" s="6" t="n"/>
+      <c r="G105" s="6" t="n"/>
+      <c r="H105" s="6" t="n"/>
+      <c r="I105" s="6" t="n"/>
+      <c r="J105" s="6" t="n"/>
+      <c r="K105" s="7" t="n"/>
+      <c r="L105" s="8" t="n"/>
+      <c r="M105" s="6" t="n"/>
+      <c r="N105" s="6" t="n"/>
+      <c r="O105" s="9" t="n"/>
+      <c r="P105" s="6" t="n"/>
+      <c r="Q105" s="6" t="n"/>
+      <c r="R105" s="6" t="n"/>
+      <c r="S105" s="6" t="n"/>
+      <c r="T105">
+        <f>IF(C105="","",IF(AND(K105&lt;&gt;"",L105=""),"Falta el costo",IF(AND(LEFT(I105,6)="Por ov",K105&lt;&gt;"",G105=""),"Falta el peso del ovillo",IF(AND(A105="",B105=""),"Falta la categoría",IF(AND(A105="",I105=""),"Falta cómo se vende",IF(AND(K105&lt;&gt;"",N105="",M105=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="11" t="n"/>
+      <c r="B106" s="6" t="n"/>
+      <c r="C106" s="6" t="n"/>
+      <c r="D106" s="6" t="n"/>
+      <c r="E106" s="6" t="n"/>
+      <c r="F106" s="6" t="n"/>
+      <c r="G106" s="6" t="n"/>
+      <c r="H106" s="6" t="n"/>
+      <c r="I106" s="6" t="n"/>
+      <c r="J106" s="6" t="n"/>
+      <c r="K106" s="7" t="n"/>
+      <c r="L106" s="8" t="n"/>
+      <c r="M106" s="6" t="n"/>
+      <c r="N106" s="6" t="n"/>
+      <c r="O106" s="9" t="n"/>
+      <c r="P106" s="6" t="n"/>
+      <c r="Q106" s="6" t="n"/>
+      <c r="R106" s="6" t="n"/>
+      <c r="S106" s="6" t="n"/>
+      <c r="T106">
+        <f>IF(C106="","",IF(AND(K106&lt;&gt;"",L106=""),"Falta el costo",IF(AND(LEFT(I106,6)="Por ov",K106&lt;&gt;"",G106=""),"Falta el peso del ovillo",IF(AND(A106="",B106=""),"Falta la categoría",IF(AND(A106="",I106=""),"Falta cómo se vende",IF(AND(K106&lt;&gt;"",N106="",M106=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="11" t="n"/>
+      <c r="B107" s="6" t="n"/>
+      <c r="C107" s="6" t="n"/>
+      <c r="D107" s="6" t="n"/>
+      <c r="E107" s="6" t="n"/>
+      <c r="F107" s="6" t="n"/>
+      <c r="G107" s="6" t="n"/>
+      <c r="H107" s="6" t="n"/>
+      <c r="I107" s="6" t="n"/>
+      <c r="J107" s="6" t="n"/>
+      <c r="K107" s="7" t="n"/>
+      <c r="L107" s="8" t="n"/>
+      <c r="M107" s="6" t="n"/>
+      <c r="N107" s="6" t="n"/>
+      <c r="O107" s="9" t="n"/>
+      <c r="P107" s="6" t="n"/>
+      <c r="Q107" s="6" t="n"/>
+      <c r="R107" s="6" t="n"/>
+      <c r="S107" s="6" t="n"/>
+      <c r="T107">
+        <f>IF(C107="","",IF(AND(K107&lt;&gt;"",L107=""),"Falta el costo",IF(AND(LEFT(I107,6)="Por ov",K107&lt;&gt;"",G107=""),"Falta el peso del ovillo",IF(AND(A107="",B107=""),"Falta la categoría",IF(AND(A107="",I107=""),"Falta cómo se vende",IF(AND(K107&lt;&gt;"",N107="",M107=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="11" t="n"/>
+      <c r="B108" s="6" t="n"/>
+      <c r="C108" s="6" t="n"/>
+      <c r="D108" s="6" t="n"/>
+      <c r="E108" s="6" t="n"/>
+      <c r="F108" s="6" t="n"/>
+      <c r="G108" s="6" t="n"/>
+      <c r="H108" s="6" t="n"/>
+      <c r="I108" s="6" t="n"/>
+      <c r="J108" s="6" t="n"/>
+      <c r="K108" s="7" t="n"/>
+      <c r="L108" s="8" t="n"/>
+      <c r="M108" s="6" t="n"/>
+      <c r="N108" s="6" t="n"/>
+      <c r="O108" s="9" t="n"/>
+      <c r="P108" s="6" t="n"/>
+      <c r="Q108" s="6" t="n"/>
+      <c r="R108" s="6" t="n"/>
+      <c r="S108" s="6" t="n"/>
+      <c r="T108">
+        <f>IF(C108="","",IF(AND(K108&lt;&gt;"",L108=""),"Falta el costo",IF(AND(LEFT(I108,6)="Por ov",K108&lt;&gt;"",G108=""),"Falta el peso del ovillo",IF(AND(A108="",B108=""),"Falta la categoría",IF(AND(A108="",I108=""),"Falta cómo se vende",IF(AND(K108&lt;&gt;"",N108="",M108=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="11" t="n"/>
+      <c r="B109" s="6" t="n"/>
+      <c r="C109" s="6" t="n"/>
+      <c r="D109" s="6" t="n"/>
+      <c r="E109" s="6" t="n"/>
+      <c r="F109" s="6" t="n"/>
+      <c r="G109" s="6" t="n"/>
+      <c r="H109" s="6" t="n"/>
+      <c r="I109" s="6" t="n"/>
+      <c r="J109" s="6" t="n"/>
+      <c r="K109" s="7" t="n"/>
+      <c r="L109" s="8" t="n"/>
+      <c r="M109" s="6" t="n"/>
+      <c r="N109" s="6" t="n"/>
+      <c r="O109" s="9" t="n"/>
+      <c r="P109" s="6" t="n"/>
+      <c r="Q109" s="6" t="n"/>
+      <c r="R109" s="6" t="n"/>
+      <c r="S109" s="6" t="n"/>
+      <c r="T109">
+        <f>IF(C109="","",IF(AND(K109&lt;&gt;"",L109=""),"Falta el costo",IF(AND(LEFT(I109,6)="Por ov",K109&lt;&gt;"",G109=""),"Falta el peso del ovillo",IF(AND(A109="",B109=""),"Falta la categoría",IF(AND(A109="",I109=""),"Falta cómo se vende",IF(AND(K109&lt;&gt;"",N109="",M109=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="11" t="n"/>
+      <c r="B110" s="6" t="n"/>
+      <c r="C110" s="6" t="n"/>
+      <c r="D110" s="6" t="n"/>
+      <c r="E110" s="6" t="n"/>
+      <c r="F110" s="6" t="n"/>
+      <c r="G110" s="6" t="n"/>
+      <c r="H110" s="6" t="n"/>
+      <c r="I110" s="6" t="n"/>
+      <c r="J110" s="6" t="n"/>
+      <c r="K110" s="7" t="n"/>
+      <c r="L110" s="8" t="n"/>
+      <c r="M110" s="6" t="n"/>
+      <c r="N110" s="6" t="n"/>
+      <c r="O110" s="9" t="n"/>
+      <c r="P110" s="6" t="n"/>
+      <c r="Q110" s="6" t="n"/>
+      <c r="R110" s="6" t="n"/>
+      <c r="S110" s="6" t="n"/>
+      <c r="T110">
+        <f>IF(C110="","",IF(AND(K110&lt;&gt;"",L110=""),"Falta el costo",IF(AND(LEFT(I110,6)="Por ov",K110&lt;&gt;"",G110=""),"Falta el peso del ovillo",IF(AND(A110="",B110=""),"Falta la categoría",IF(AND(A110="",I110=""),"Falta cómo se vende",IF(AND(K110&lt;&gt;"",N110="",M110=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="11" t="n"/>
+      <c r="B111" s="6" t="n"/>
+      <c r="C111" s="6" t="n"/>
+      <c r="D111" s="6" t="n"/>
+      <c r="E111" s="6" t="n"/>
+      <c r="F111" s="6" t="n"/>
+      <c r="G111" s="6" t="n"/>
+      <c r="H111" s="6" t="n"/>
+      <c r="I111" s="6" t="n"/>
+      <c r="J111" s="6" t="n"/>
+      <c r="K111" s="7" t="n"/>
+      <c r="L111" s="8" t="n"/>
+      <c r="M111" s="6" t="n"/>
+      <c r="N111" s="6" t="n"/>
+      <c r="O111" s="9" t="n"/>
+      <c r="P111" s="6" t="n"/>
+      <c r="Q111" s="6" t="n"/>
+      <c r="R111" s="6" t="n"/>
+      <c r="S111" s="6" t="n"/>
+      <c r="T111">
+        <f>IF(C111="","",IF(AND(K111&lt;&gt;"",L111=""),"Falta el costo",IF(AND(LEFT(I111,6)="Por ov",K111&lt;&gt;"",G111=""),"Falta el peso del ovillo",IF(AND(A111="",B111=""),"Falta la categoría",IF(AND(A111="",I111=""),"Falta cómo se vende",IF(AND(K111&lt;&gt;"",N111="",M111=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="11" t="n"/>
+      <c r="B112" s="6" t="n"/>
+      <c r="C112" s="6" t="n"/>
+      <c r="D112" s="6" t="n"/>
+      <c r="E112" s="6" t="n"/>
+      <c r="F112" s="6" t="n"/>
+      <c r="G112" s="6" t="n"/>
+      <c r="H112" s="6" t="n"/>
+      <c r="I112" s="6" t="n"/>
+      <c r="J112" s="6" t="n"/>
+      <c r="K112" s="7" t="n"/>
+      <c r="L112" s="8" t="n"/>
+      <c r="M112" s="6" t="n"/>
+      <c r="N112" s="6" t="n"/>
+      <c r="O112" s="9" t="n"/>
+      <c r="P112" s="6" t="n"/>
+      <c r="Q112" s="6" t="n"/>
+      <c r="R112" s="6" t="n"/>
+      <c r="S112" s="6" t="n"/>
+      <c r="T112">
+        <f>IF(C112="","",IF(AND(K112&lt;&gt;"",L112=""),"Falta el costo",IF(AND(LEFT(I112,6)="Por ov",K112&lt;&gt;"",G112=""),"Falta el peso del ovillo",IF(AND(A112="",B112=""),"Falta la categoría",IF(AND(A112="",I112=""),"Falta cómo se vende",IF(AND(K112&lt;&gt;"",N112="",M112=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="11" t="n"/>
+      <c r="B113" s="6" t="n"/>
+      <c r="C113" s="6" t="n"/>
+      <c r="D113" s="6" t="n"/>
+      <c r="E113" s="6" t="n"/>
+      <c r="F113" s="6" t="n"/>
+      <c r="G113" s="6" t="n"/>
+      <c r="H113" s="6" t="n"/>
+      <c r="I113" s="6" t="n"/>
+      <c r="J113" s="6" t="n"/>
+      <c r="K113" s="7" t="n"/>
+      <c r="L113" s="8" t="n"/>
+      <c r="M113" s="6" t="n"/>
+      <c r="N113" s="6" t="n"/>
+      <c r="O113" s="9" t="n"/>
+      <c r="P113" s="6" t="n"/>
+      <c r="Q113" s="6" t="n"/>
+      <c r="R113" s="6" t="n"/>
+      <c r="S113" s="6" t="n"/>
+      <c r="T113">
+        <f>IF(C113="","",IF(AND(K113&lt;&gt;"",L113=""),"Falta el costo",IF(AND(LEFT(I113,6)="Por ov",K113&lt;&gt;"",G113=""),"Falta el peso del ovillo",IF(AND(A113="",B113=""),"Falta la categoría",IF(AND(A113="",I113=""),"Falta cómo se vende",IF(AND(K113&lt;&gt;"",N113="",M113=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="11" t="n"/>
+      <c r="B114" s="6" t="n"/>
+      <c r="C114" s="6" t="n"/>
+      <c r="D114" s="6" t="n"/>
+      <c r="E114" s="6" t="n"/>
+      <c r="F114" s="6" t="n"/>
+      <c r="G114" s="6" t="n"/>
+      <c r="H114" s="6" t="n"/>
+      <c r="I114" s="6" t="n"/>
+      <c r="J114" s="6" t="n"/>
+      <c r="K114" s="7" t="n"/>
+      <c r="L114" s="8" t="n"/>
+      <c r="M114" s="6" t="n"/>
+      <c r="N114" s="6" t="n"/>
+      <c r="O114" s="9" t="n"/>
+      <c r="P114" s="6" t="n"/>
+      <c r="Q114" s="6" t="n"/>
+      <c r="R114" s="6" t="n"/>
+      <c r="S114" s="6" t="n"/>
+      <c r="T114">
+        <f>IF(C114="","",IF(AND(K114&lt;&gt;"",L114=""),"Falta el costo",IF(AND(LEFT(I114,6)="Por ov",K114&lt;&gt;"",G114=""),"Falta el peso del ovillo",IF(AND(A114="",B114=""),"Falta la categoría",IF(AND(A114="",I114=""),"Falta cómo se vende",IF(AND(K114&lt;&gt;"",N114="",M114=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="11" t="n"/>
+      <c r="B115" s="6" t="n"/>
+      <c r="C115" s="6" t="n"/>
+      <c r="D115" s="6" t="n"/>
+      <c r="E115" s="6" t="n"/>
+      <c r="F115" s="6" t="n"/>
+      <c r="G115" s="6" t="n"/>
+      <c r="H115" s="6" t="n"/>
+      <c r="I115" s="6" t="n"/>
+      <c r="J115" s="6" t="n"/>
+      <c r="K115" s="7" t="n"/>
+      <c r="L115" s="8" t="n"/>
+      <c r="M115" s="6" t="n"/>
+      <c r="N115" s="6" t="n"/>
+      <c r="O115" s="9" t="n"/>
+      <c r="P115" s="6" t="n"/>
+      <c r="Q115" s="6" t="n"/>
+      <c r="R115" s="6" t="n"/>
+      <c r="S115" s="6" t="n"/>
+      <c r="T115">
+        <f>IF(C115="","",IF(AND(K115&lt;&gt;"",L115=""),"Falta el costo",IF(AND(LEFT(I115,6)="Por ov",K115&lt;&gt;"",G115=""),"Falta el peso del ovillo",IF(AND(A115="",B115=""),"Falta la categoría",IF(AND(A115="",I115=""),"Falta cómo se vende",IF(AND(K115&lt;&gt;"",N115="",M115=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="11" t="n"/>
+      <c r="B116" s="6" t="n"/>
+      <c r="C116" s="6" t="n"/>
+      <c r="D116" s="6" t="n"/>
+      <c r="E116" s="6" t="n"/>
+      <c r="F116" s="6" t="n"/>
+      <c r="G116" s="6" t="n"/>
+      <c r="H116" s="6" t="n"/>
+      <c r="I116" s="6" t="n"/>
+      <c r="J116" s="6" t="n"/>
+      <c r="K116" s="7" t="n"/>
+      <c r="L116" s="8" t="n"/>
+      <c r="M116" s="6" t="n"/>
+      <c r="N116" s="6" t="n"/>
+      <c r="O116" s="9" t="n"/>
+      <c r="P116" s="6" t="n"/>
+      <c r="Q116" s="6" t="n"/>
+      <c r="R116" s="6" t="n"/>
+      <c r="S116" s="6" t="n"/>
+      <c r="T116">
+        <f>IF(C116="","",IF(AND(K116&lt;&gt;"",L116=""),"Falta el costo",IF(AND(LEFT(I116,6)="Por ov",K116&lt;&gt;"",G116=""),"Falta el peso del ovillo",IF(AND(A116="",B116=""),"Falta la categoría",IF(AND(A116="",I116=""),"Falta cómo se vende",IF(AND(K116&lt;&gt;"",N116="",M116=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="11" t="n"/>
+      <c r="B117" s="6" t="n"/>
+      <c r="C117" s="6" t="n"/>
+      <c r="D117" s="6" t="n"/>
+      <c r="E117" s="6" t="n"/>
+      <c r="F117" s="6" t="n"/>
+      <c r="G117" s="6" t="n"/>
+      <c r="H117" s="6" t="n"/>
+      <c r="I117" s="6" t="n"/>
+      <c r="J117" s="6" t="n"/>
+      <c r="K117" s="7" t="n"/>
+      <c r="L117" s="8" t="n"/>
+      <c r="M117" s="6" t="n"/>
+      <c r="N117" s="6" t="n"/>
+      <c r="O117" s="9" t="n"/>
+      <c r="P117" s="6" t="n"/>
+      <c r="Q117" s="6" t="n"/>
+      <c r="R117" s="6" t="n"/>
+      <c r="S117" s="6" t="n"/>
+      <c r="T117">
+        <f>IF(C117="","",IF(AND(K117&lt;&gt;"",L117=""),"Falta el costo",IF(AND(LEFT(I117,6)="Por ov",K117&lt;&gt;"",G117=""),"Falta el peso del ovillo",IF(AND(A117="",B117=""),"Falta la categoría",IF(AND(A117="",I117=""),"Falta cómo se vende",IF(AND(K117&lt;&gt;"",N117="",M117=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="11" t="n"/>
+      <c r="B118" s="6" t="n"/>
+      <c r="C118" s="6" t="n"/>
+      <c r="D118" s="6" t="n"/>
+      <c r="E118" s="6" t="n"/>
+      <c r="F118" s="6" t="n"/>
+      <c r="G118" s="6" t="n"/>
+      <c r="H118" s="6" t="n"/>
+      <c r="I118" s="6" t="n"/>
+      <c r="J118" s="6" t="n"/>
+      <c r="K118" s="7" t="n"/>
+      <c r="L118" s="8" t="n"/>
+      <c r="M118" s="6" t="n"/>
+      <c r="N118" s="6" t="n"/>
+      <c r="O118" s="9" t="n"/>
+      <c r="P118" s="6" t="n"/>
+      <c r="Q118" s="6" t="n"/>
+      <c r="R118" s="6" t="n"/>
+      <c r="S118" s="6" t="n"/>
+      <c r="T118">
+        <f>IF(C118="","",IF(AND(K118&lt;&gt;"",L118=""),"Falta el costo",IF(AND(LEFT(I118,6)="Por ov",K118&lt;&gt;"",G118=""),"Falta el peso del ovillo",IF(AND(A118="",B118=""),"Falta la categoría",IF(AND(A118="",I118=""),"Falta cómo se vende",IF(AND(K118&lt;&gt;"",N118="",M118=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="11" t="n"/>
+      <c r="B119" s="6" t="n"/>
+      <c r="C119" s="6" t="n"/>
+      <c r="D119" s="6" t="n"/>
+      <c r="E119" s="6" t="n"/>
+      <c r="F119" s="6" t="n"/>
+      <c r="G119" s="6" t="n"/>
+      <c r="H119" s="6" t="n"/>
+      <c r="I119" s="6" t="n"/>
+      <c r="J119" s="6" t="n"/>
+      <c r="K119" s="7" t="n"/>
+      <c r="L119" s="8" t="n"/>
+      <c r="M119" s="6" t="n"/>
+      <c r="N119" s="6" t="n"/>
+      <c r="O119" s="9" t="n"/>
+      <c r="P119" s="6" t="n"/>
+      <c r="Q119" s="6" t="n"/>
+      <c r="R119" s="6" t="n"/>
+      <c r="S119" s="6" t="n"/>
+      <c r="T119">
+        <f>IF(C119="","",IF(AND(K119&lt;&gt;"",L119=""),"Falta el costo",IF(AND(LEFT(I119,6)="Por ov",K119&lt;&gt;"",G119=""),"Falta el peso del ovillo",IF(AND(A119="",B119=""),"Falta la categoría",IF(AND(A119="",I119=""),"Falta cómo se vende",IF(AND(K119&lt;&gt;"",N119="",M119=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="11" t="n"/>
+      <c r="B120" s="6" t="n"/>
+      <c r="C120" s="6" t="n"/>
+      <c r="D120" s="6" t="n"/>
+      <c r="E120" s="6" t="n"/>
+      <c r="F120" s="6" t="n"/>
+      <c r="G120" s="6" t="n"/>
+      <c r="H120" s="6" t="n"/>
+      <c r="I120" s="6" t="n"/>
+      <c r="J120" s="6" t="n"/>
+      <c r="K120" s="7" t="n"/>
+      <c r="L120" s="8" t="n"/>
+      <c r="M120" s="6" t="n"/>
+      <c r="N120" s="6" t="n"/>
+      <c r="O120" s="9" t="n"/>
+      <c r="P120" s="6" t="n"/>
+      <c r="Q120" s="6" t="n"/>
+      <c r="R120" s="6" t="n"/>
+      <c r="S120" s="6" t="n"/>
+      <c r="T120">
+        <f>IF(C120="","",IF(AND(K120&lt;&gt;"",L120=""),"Falta el costo",IF(AND(LEFT(I120,6)="Por ov",K120&lt;&gt;"",G120=""),"Falta el peso del ovillo",IF(AND(A120="",B120=""),"Falta la categoría",IF(AND(A120="",I120=""),"Falta cómo se vende",IF(AND(K120&lt;&gt;"",N120="",M120=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="11" t="n"/>
+      <c r="B121" s="6" t="n"/>
+      <c r="C121" s="6" t="n"/>
+      <c r="D121" s="6" t="n"/>
+      <c r="E121" s="6" t="n"/>
+      <c r="F121" s="6" t="n"/>
+      <c r="G121" s="6" t="n"/>
+      <c r="H121" s="6" t="n"/>
+      <c r="I121" s="6" t="n"/>
+      <c r="J121" s="6" t="n"/>
+      <c r="K121" s="7" t="n"/>
+      <c r="L121" s="8" t="n"/>
+      <c r="M121" s="6" t="n"/>
+      <c r="N121" s="6" t="n"/>
+      <c r="O121" s="9" t="n"/>
+      <c r="P121" s="6" t="n"/>
+      <c r="Q121" s="6" t="n"/>
+      <c r="R121" s="6" t="n"/>
+      <c r="S121" s="6" t="n"/>
+      <c r="T121">
+        <f>IF(C121="","",IF(AND(K121&lt;&gt;"",L121=""),"Falta el costo",IF(AND(LEFT(I121,6)="Por ov",K121&lt;&gt;"",G121=""),"Falta el peso del ovillo",IF(AND(A121="",B121=""),"Falta la categoría",IF(AND(A121="",I121=""),"Falta cómo se vende",IF(AND(K121&lt;&gt;"",N121="",M121=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="11" t="n"/>
+      <c r="B122" s="6" t="n"/>
+      <c r="C122" s="6" t="n"/>
+      <c r="D122" s="6" t="n"/>
+      <c r="E122" s="6" t="n"/>
+      <c r="F122" s="6" t="n"/>
+      <c r="G122" s="6" t="n"/>
+      <c r="H122" s="6" t="n"/>
+      <c r="I122" s="6" t="n"/>
+      <c r="J122" s="6" t="n"/>
+      <c r="K122" s="7" t="n"/>
+      <c r="L122" s="8" t="n"/>
+      <c r="M122" s="6" t="n"/>
+      <c r="N122" s="6" t="n"/>
+      <c r="O122" s="9" t="n"/>
+      <c r="P122" s="6" t="n"/>
+      <c r="Q122" s="6" t="n"/>
+      <c r="R122" s="6" t="n"/>
+      <c r="S122" s="6" t="n"/>
+      <c r="T122">
+        <f>IF(C122="","",IF(AND(K122&lt;&gt;"",L122=""),"Falta el costo",IF(AND(LEFT(I122,6)="Por ov",K122&lt;&gt;"",G122=""),"Falta el peso del ovillo",IF(AND(A122="",B122=""),"Falta la categoría",IF(AND(A122="",I122=""),"Falta cómo se vende",IF(AND(K122&lt;&gt;"",N122="",M122=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="11" t="n"/>
+      <c r="B123" s="6" t="n"/>
+      <c r="C123" s="6" t="n"/>
+      <c r="D123" s="6" t="n"/>
+      <c r="E123" s="6" t="n"/>
+      <c r="F123" s="6" t="n"/>
+      <c r="G123" s="6" t="n"/>
+      <c r="H123" s="6" t="n"/>
+      <c r="I123" s="6" t="n"/>
+      <c r="J123" s="6" t="n"/>
+      <c r="K123" s="7" t="n"/>
+      <c r="L123" s="8" t="n"/>
+      <c r="M123" s="6" t="n"/>
+      <c r="N123" s="6" t="n"/>
+      <c r="O123" s="9" t="n"/>
+      <c r="P123" s="6" t="n"/>
+      <c r="Q123" s="6" t="n"/>
+      <c r="R123" s="6" t="n"/>
+      <c r="S123" s="6" t="n"/>
+      <c r="T123">
+        <f>IF(C123="","",IF(AND(K123&lt;&gt;"",L123=""),"Falta el costo",IF(AND(LEFT(I123,6)="Por ov",K123&lt;&gt;"",G123=""),"Falta el peso del ovillo",IF(AND(A123="",B123=""),"Falta la categoría",IF(AND(A123="",I123=""),"Falta cómo se vende",IF(AND(K123&lt;&gt;"",N123="",M123=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="11" t="n"/>
+      <c r="B124" s="6" t="n"/>
+      <c r="C124" s="6" t="n"/>
+      <c r="D124" s="6" t="n"/>
+      <c r="E124" s="6" t="n"/>
+      <c r="F124" s="6" t="n"/>
+      <c r="G124" s="6" t="n"/>
+      <c r="H124" s="6" t="n"/>
+      <c r="I124" s="6" t="n"/>
+      <c r="J124" s="6" t="n"/>
+      <c r="K124" s="7" t="n"/>
+      <c r="L124" s="8" t="n"/>
+      <c r="M124" s="6" t="n"/>
+      <c r="N124" s="6" t="n"/>
+      <c r="O124" s="9" t="n"/>
+      <c r="P124" s="6" t="n"/>
+      <c r="Q124" s="6" t="n"/>
+      <c r="R124" s="6" t="n"/>
+      <c r="S124" s="6" t="n"/>
+      <c r="T124">
+        <f>IF(C124="","",IF(AND(K124&lt;&gt;"",L124=""),"Falta el costo",IF(AND(LEFT(I124,6)="Por ov",K124&lt;&gt;"",G124=""),"Falta el peso del ovillo",IF(AND(A124="",B124=""),"Falta la categoría",IF(AND(A124="",I124=""),"Falta cómo se vende",IF(AND(K124&lt;&gt;"",N124="",M124=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="11" t="n"/>
+      <c r="B125" s="6" t="n"/>
+      <c r="C125" s="6" t="n"/>
+      <c r="D125" s="6" t="n"/>
+      <c r="E125" s="6" t="n"/>
+      <c r="F125" s="6" t="n"/>
+      <c r="G125" s="6" t="n"/>
+      <c r="H125" s="6" t="n"/>
+      <c r="I125" s="6" t="n"/>
+      <c r="J125" s="6" t="n"/>
+      <c r="K125" s="7" t="n"/>
+      <c r="L125" s="8" t="n"/>
+      <c r="M125" s="6" t="n"/>
+      <c r="N125" s="6" t="n"/>
+      <c r="O125" s="9" t="n"/>
+      <c r="P125" s="6" t="n"/>
+      <c r="Q125" s="6" t="n"/>
+      <c r="R125" s="6" t="n"/>
+      <c r="S125" s="6" t="n"/>
+      <c r="T125">
+        <f>IF(C125="","",IF(AND(K125&lt;&gt;"",L125=""),"Falta el costo",IF(AND(LEFT(I125,6)="Por ov",K125&lt;&gt;"",G125=""),"Falta el peso del ovillo",IF(AND(A125="",B125=""),"Falta la categoría",IF(AND(A125="",I125=""),"Falta cómo se vende",IF(AND(K125&lt;&gt;"",N125="",M125=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="11" t="n"/>
+      <c r="B126" s="6" t="n"/>
+      <c r="C126" s="6" t="n"/>
+      <c r="D126" s="6" t="n"/>
+      <c r="E126" s="6" t="n"/>
+      <c r="F126" s="6" t="n"/>
+      <c r="G126" s="6" t="n"/>
+      <c r="H126" s="6" t="n"/>
+      <c r="I126" s="6" t="n"/>
+      <c r="J126" s="6" t="n"/>
+      <c r="K126" s="7" t="n"/>
+      <c r="L126" s="8" t="n"/>
+      <c r="M126" s="6" t="n"/>
+      <c r="N126" s="6" t="n"/>
+      <c r="O126" s="9" t="n"/>
+      <c r="P126" s="6" t="n"/>
+      <c r="Q126" s="6" t="n"/>
+      <c r="R126" s="6" t="n"/>
+      <c r="S126" s="6" t="n"/>
+      <c r="T126">
+        <f>IF(C126="","",IF(AND(K126&lt;&gt;"",L126=""),"Falta el costo",IF(AND(LEFT(I126,6)="Por ov",K126&lt;&gt;"",G126=""),"Falta el peso del ovillo",IF(AND(A126="",B126=""),"Falta la categoría",IF(AND(A126="",I126=""),"Falta cómo se vende",IF(AND(K126&lt;&gt;"",N126="",M126=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="11" t="n"/>
+      <c r="B127" s="6" t="n"/>
+      <c r="C127" s="6" t="n"/>
+      <c r="D127" s="6" t="n"/>
+      <c r="E127" s="6" t="n"/>
+      <c r="F127" s="6" t="n"/>
+      <c r="G127" s="6" t="n"/>
+      <c r="H127" s="6" t="n"/>
+      <c r="I127" s="6" t="n"/>
+      <c r="J127" s="6" t="n"/>
+      <c r="K127" s="7" t="n"/>
+      <c r="L127" s="8" t="n"/>
+      <c r="M127" s="6" t="n"/>
+      <c r="N127" s="6" t="n"/>
+      <c r="O127" s="9" t="n"/>
+      <c r="P127" s="6" t="n"/>
+      <c r="Q127" s="6" t="n"/>
+      <c r="R127" s="6" t="n"/>
+      <c r="S127" s="6" t="n"/>
+      <c r="T127">
+        <f>IF(C127="","",IF(AND(K127&lt;&gt;"",L127=""),"Falta el costo",IF(AND(LEFT(I127,6)="Por ov",K127&lt;&gt;"",G127=""),"Falta el peso del ovillo",IF(AND(A127="",B127=""),"Falta la categoría",IF(AND(A127="",I127=""),"Falta cómo se vende",IF(AND(K127&lt;&gt;"",N127="",M127=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="11" t="n"/>
+      <c r="B128" s="6" t="n"/>
+      <c r="C128" s="6" t="n"/>
+      <c r="D128" s="6" t="n"/>
+      <c r="E128" s="6" t="n"/>
+      <c r="F128" s="6" t="n"/>
+      <c r="G128" s="6" t="n"/>
+      <c r="H128" s="6" t="n"/>
+      <c r="I128" s="6" t="n"/>
+      <c r="J128" s="6" t="n"/>
+      <c r="K128" s="7" t="n"/>
+      <c r="L128" s="8" t="n"/>
+      <c r="M128" s="6" t="n"/>
+      <c r="N128" s="6" t="n"/>
+      <c r="O128" s="9" t="n"/>
+      <c r="P128" s="6" t="n"/>
+      <c r="Q128" s="6" t="n"/>
+      <c r="R128" s="6" t="n"/>
+      <c r="S128" s="6" t="n"/>
+      <c r="T128">
+        <f>IF(C128="","",IF(AND(K128&lt;&gt;"",L128=""),"Falta el costo",IF(AND(LEFT(I128,6)="Por ov",K128&lt;&gt;"",G128=""),"Falta el peso del ovillo",IF(AND(A128="",B128=""),"Falta la categoría",IF(AND(A128="",I128=""),"Falta cómo se vende",IF(AND(K128&lt;&gt;"",N128="",M128=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="11" t="n"/>
+      <c r="B129" s="6" t="n"/>
+      <c r="C129" s="6" t="n"/>
+      <c r="D129" s="6" t="n"/>
+      <c r="E129" s="6" t="n"/>
+      <c r="F129" s="6" t="n"/>
+      <c r="G129" s="6" t="n"/>
+      <c r="H129" s="6" t="n"/>
+      <c r="I129" s="6" t="n"/>
+      <c r="J129" s="6" t="n"/>
+      <c r="K129" s="7" t="n"/>
+      <c r="L129" s="8" t="n"/>
+      <c r="M129" s="6" t="n"/>
+      <c r="N129" s="6" t="n"/>
+      <c r="O129" s="9" t="n"/>
+      <c r="P129" s="6" t="n"/>
+      <c r="Q129" s="6" t="n"/>
+      <c r="R129" s="6" t="n"/>
+      <c r="S129" s="6" t="n"/>
+      <c r="T129">
+        <f>IF(C129="","",IF(AND(K129&lt;&gt;"",L129=""),"Falta el costo",IF(AND(LEFT(I129,6)="Por ov",K129&lt;&gt;"",G129=""),"Falta el peso del ovillo",IF(AND(A129="",B129=""),"Falta la categoría",IF(AND(A129="",I129=""),"Falta cómo se vende",IF(AND(K129&lt;&gt;"",N129="",M129=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="11" t="n"/>
+      <c r="B130" s="6" t="n"/>
+      <c r="C130" s="6" t="n"/>
+      <c r="D130" s="6" t="n"/>
+      <c r="E130" s="6" t="n"/>
+      <c r="F130" s="6" t="n"/>
+      <c r="G130" s="6" t="n"/>
+      <c r="H130" s="6" t="n"/>
+      <c r="I130" s="6" t="n"/>
+      <c r="J130" s="6" t="n"/>
+      <c r="K130" s="7" t="n"/>
+      <c r="L130" s="8" t="n"/>
+      <c r="M130" s="6" t="n"/>
+      <c r="N130" s="6" t="n"/>
+      <c r="O130" s="9" t="n"/>
+      <c r="P130" s="6" t="n"/>
+      <c r="Q130" s="6" t="n"/>
+      <c r="R130" s="6" t="n"/>
+      <c r="S130" s="6" t="n"/>
+      <c r="T130">
+        <f>IF(C130="","",IF(AND(K130&lt;&gt;"",L130=""),"Falta el costo",IF(AND(LEFT(I130,6)="Por ov",K130&lt;&gt;"",G130=""),"Falta el peso del ovillo",IF(AND(A130="",B130=""),"Falta la categoría",IF(AND(A130="",I130=""),"Falta cómo se vende",IF(AND(K130&lt;&gt;"",N130="",M130=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="11" t="n"/>
+      <c r="B131" s="6" t="n"/>
+      <c r="C131" s="6" t="n"/>
+      <c r="D131" s="6" t="n"/>
+      <c r="E131" s="6" t="n"/>
+      <c r="F131" s="6" t="n"/>
+      <c r="G131" s="6" t="n"/>
+      <c r="H131" s="6" t="n"/>
+      <c r="I131" s="6" t="n"/>
+      <c r="J131" s="6" t="n"/>
+      <c r="K131" s="7" t="n"/>
+      <c r="L131" s="8" t="n"/>
+      <c r="M131" s="6" t="n"/>
+      <c r="N131" s="6" t="n"/>
+      <c r="O131" s="9" t="n"/>
+      <c r="P131" s="6" t="n"/>
+      <c r="Q131" s="6" t="n"/>
+      <c r="R131" s="6" t="n"/>
+      <c r="S131" s="6" t="n"/>
+      <c r="T131">
+        <f>IF(C131="","",IF(AND(K131&lt;&gt;"",L131=""),"Falta el costo",IF(AND(LEFT(I131,6)="Por ov",K131&lt;&gt;"",G131=""),"Falta el peso del ovillo",IF(AND(A131="",B131=""),"Falta la categoría",IF(AND(A131="",I131=""),"Falta cómo se vende",IF(AND(K131&lt;&gt;"",N131="",M131=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="11" t="n"/>
+      <c r="B132" s="6" t="n"/>
+      <c r="C132" s="6" t="n"/>
+      <c r="D132" s="6" t="n"/>
+      <c r="E132" s="6" t="n"/>
+      <c r="F132" s="6" t="n"/>
+      <c r="G132" s="6" t="n"/>
+      <c r="H132" s="6" t="n"/>
+      <c r="I132" s="6" t="n"/>
+      <c r="J132" s="6" t="n"/>
+      <c r="K132" s="7" t="n"/>
+      <c r="L132" s="8" t="n"/>
+      <c r="M132" s="6" t="n"/>
+      <c r="N132" s="6" t="n"/>
+      <c r="O132" s="9" t="n"/>
+      <c r="P132" s="6" t="n"/>
+      <c r="Q132" s="6" t="n"/>
+      <c r="R132" s="6" t="n"/>
+      <c r="S132" s="6" t="n"/>
+      <c r="T132">
+        <f>IF(C132="","",IF(AND(K132&lt;&gt;"",L132=""),"Falta el costo",IF(AND(LEFT(I132,6)="Por ov",K132&lt;&gt;"",G132=""),"Falta el peso del ovillo",IF(AND(A132="",B132=""),"Falta la categoría",IF(AND(A132="",I132=""),"Falta cómo se vende",IF(AND(K132&lt;&gt;"",N132="",M132=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="11" t="n"/>
+      <c r="B133" s="6" t="n"/>
+      <c r="C133" s="6" t="n"/>
+      <c r="D133" s="6" t="n"/>
+      <c r="E133" s="6" t="n"/>
+      <c r="F133" s="6" t="n"/>
+      <c r="G133" s="6" t="n"/>
+      <c r="H133" s="6" t="n"/>
+      <c r="I133" s="6" t="n"/>
+      <c r="J133" s="6" t="n"/>
+      <c r="K133" s="7" t="n"/>
+      <c r="L133" s="8" t="n"/>
+      <c r="M133" s="6" t="n"/>
+      <c r="N133" s="6" t="n"/>
+      <c r="O133" s="9" t="n"/>
+      <c r="P133" s="6" t="n"/>
+      <c r="Q133" s="6" t="n"/>
+      <c r="R133" s="6" t="n"/>
+      <c r="S133" s="6" t="n"/>
+      <c r="T133">
+        <f>IF(C133="","",IF(AND(K133&lt;&gt;"",L133=""),"Falta el costo",IF(AND(LEFT(I133,6)="Por ov",K133&lt;&gt;"",G133=""),"Falta el peso del ovillo",IF(AND(A133="",B133=""),"Falta la categoría",IF(AND(A133="",I133=""),"Falta cómo se vende",IF(AND(K133&lt;&gt;"",N133="",M133=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="11" t="n"/>
+      <c r="B134" s="6" t="n"/>
+      <c r="C134" s="6" t="n"/>
+      <c r="D134" s="6" t="n"/>
+      <c r="E134" s="6" t="n"/>
+      <c r="F134" s="6" t="n"/>
+      <c r="G134" s="6" t="n"/>
+      <c r="H134" s="6" t="n"/>
+      <c r="I134" s="6" t="n"/>
+      <c r="J134" s="6" t="n"/>
+      <c r="K134" s="7" t="n"/>
+      <c r="L134" s="8" t="n"/>
+      <c r="M134" s="6" t="n"/>
+      <c r="N134" s="6" t="n"/>
+      <c r="O134" s="9" t="n"/>
+      <c r="P134" s="6" t="n"/>
+      <c r="Q134" s="6" t="n"/>
+      <c r="R134" s="6" t="n"/>
+      <c r="S134" s="6" t="n"/>
+      <c r="T134">
+        <f>IF(C134="","",IF(AND(K134&lt;&gt;"",L134=""),"Falta el costo",IF(AND(LEFT(I134,6)="Por ov",K134&lt;&gt;"",G134=""),"Falta el peso del ovillo",IF(AND(A134="",B134=""),"Falta la categoría",IF(AND(A134="",I134=""),"Falta cómo se vende",IF(AND(K134&lt;&gt;"",N134="",M134=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="11" t="n"/>
+      <c r="B135" s="6" t="n"/>
+      <c r="C135" s="6" t="n"/>
+      <c r="D135" s="6" t="n"/>
+      <c r="E135" s="6" t="n"/>
+      <c r="F135" s="6" t="n"/>
+      <c r="G135" s="6" t="n"/>
+      <c r="H135" s="6" t="n"/>
+      <c r="I135" s="6" t="n"/>
+      <c r="J135" s="6" t="n"/>
+      <c r="K135" s="7" t="n"/>
+      <c r="L135" s="8" t="n"/>
+      <c r="M135" s="6" t="n"/>
+      <c r="N135" s="6" t="n"/>
+      <c r="O135" s="9" t="n"/>
+      <c r="P135" s="6" t="n"/>
+      <c r="Q135" s="6" t="n"/>
+      <c r="R135" s="6" t="n"/>
+      <c r="S135" s="6" t="n"/>
+      <c r="T135">
+        <f>IF(C135="","",IF(AND(K135&lt;&gt;"",L135=""),"Falta el costo",IF(AND(LEFT(I135,6)="Por ov",K135&lt;&gt;"",G135=""),"Falta el peso del ovillo",IF(AND(A135="",B135=""),"Falta la categoría",IF(AND(A135="",I135=""),"Falta cómo se vende",IF(AND(K135&lt;&gt;"",N135="",M135=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="11" t="n"/>
+      <c r="B136" s="6" t="n"/>
+      <c r="C136" s="6" t="n"/>
+      <c r="D136" s="6" t="n"/>
+      <c r="E136" s="6" t="n"/>
+      <c r="F136" s="6" t="n"/>
+      <c r="G136" s="6" t="n"/>
+      <c r="H136" s="6" t="n"/>
+      <c r="I136" s="6" t="n"/>
+      <c r="J136" s="6" t="n"/>
+      <c r="K136" s="7" t="n"/>
+      <c r="L136" s="8" t="n"/>
+      <c r="M136" s="6" t="n"/>
+      <c r="N136" s="6" t="n"/>
+      <c r="O136" s="9" t="n"/>
+      <c r="P136" s="6" t="n"/>
+      <c r="Q136" s="6" t="n"/>
+      <c r="R136" s="6" t="n"/>
+      <c r="S136" s="6" t="n"/>
+      <c r="T136">
+        <f>IF(C136="","",IF(AND(K136&lt;&gt;"",L136=""),"Falta el costo",IF(AND(LEFT(I136,6)="Por ov",K136&lt;&gt;"",G136=""),"Falta el peso del ovillo",IF(AND(A136="",B136=""),"Falta la categoría",IF(AND(A136="",I136=""),"Falta cómo se vende",IF(AND(K136&lt;&gt;"",N136="",M136=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="11" t="n"/>
+      <c r="B137" s="6" t="n"/>
+      <c r="C137" s="6" t="n"/>
+      <c r="D137" s="6" t="n"/>
+      <c r="E137" s="6" t="n"/>
+      <c r="F137" s="6" t="n"/>
+      <c r="G137" s="6" t="n"/>
+      <c r="H137" s="6" t="n"/>
+      <c r="I137" s="6" t="n"/>
+      <c r="J137" s="6" t="n"/>
+      <c r="K137" s="7" t="n"/>
+      <c r="L137" s="8" t="n"/>
+      <c r="M137" s="6" t="n"/>
+      <c r="N137" s="6" t="n"/>
+      <c r="O137" s="9" t="n"/>
+      <c r="P137" s="6" t="n"/>
+      <c r="Q137" s="6" t="n"/>
+      <c r="R137" s="6" t="n"/>
+      <c r="S137" s="6" t="n"/>
+      <c r="T137">
+        <f>IF(C137="","",IF(AND(K137&lt;&gt;"",L137=""),"Falta el costo",IF(AND(LEFT(I137,6)="Por ov",K137&lt;&gt;"",G137=""),"Falta el peso del ovillo",IF(AND(A137="",B137=""),"Falta la categoría",IF(AND(A137="",I137=""),"Falta cómo se vende",IF(AND(K137&lt;&gt;"",N137="",M137=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="11" t="n"/>
+      <c r="B138" s="6" t="n"/>
+      <c r="C138" s="6" t="n"/>
+      <c r="D138" s="6" t="n"/>
+      <c r="E138" s="6" t="n"/>
+      <c r="F138" s="6" t="n"/>
+      <c r="G138" s="6" t="n"/>
+      <c r="H138" s="6" t="n"/>
+      <c r="I138" s="6" t="n"/>
+      <c r="J138" s="6" t="n"/>
+      <c r="K138" s="7" t="n"/>
+      <c r="L138" s="8" t="n"/>
+      <c r="M138" s="6" t="n"/>
+      <c r="N138" s="6" t="n"/>
+      <c r="O138" s="9" t="n"/>
+      <c r="P138" s="6" t="n"/>
+      <c r="Q138" s="6" t="n"/>
+      <c r="R138" s="6" t="n"/>
+      <c r="S138" s="6" t="n"/>
+      <c r="T138">
+        <f>IF(C138="","",IF(AND(K138&lt;&gt;"",L138=""),"Falta el costo",IF(AND(LEFT(I138,6)="Por ov",K138&lt;&gt;"",G138=""),"Falta el peso del ovillo",IF(AND(A138="",B138=""),"Falta la categoría",IF(AND(A138="",I138=""),"Falta cómo se vende",IF(AND(K138&lt;&gt;"",N138="",M138=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="11" t="n"/>
+      <c r="B139" s="6" t="n"/>
+      <c r="C139" s="6" t="n"/>
+      <c r="D139" s="6" t="n"/>
+      <c r="E139" s="6" t="n"/>
+      <c r="F139" s="6" t="n"/>
+      <c r="G139" s="6" t="n"/>
+      <c r="H139" s="6" t="n"/>
+      <c r="I139" s="6" t="n"/>
+      <c r="J139" s="6" t="n"/>
+      <c r="K139" s="7" t="n"/>
+      <c r="L139" s="8" t="n"/>
+      <c r="M139" s="6" t="n"/>
+      <c r="N139" s="6" t="n"/>
+      <c r="O139" s="9" t="n"/>
+      <c r="P139" s="6" t="n"/>
+      <c r="Q139" s="6" t="n"/>
+      <c r="R139" s="6" t="n"/>
+      <c r="S139" s="6" t="n"/>
+      <c r="T139">
+        <f>IF(C139="","",IF(AND(K139&lt;&gt;"",L139=""),"Falta el costo",IF(AND(LEFT(I139,6)="Por ov",K139&lt;&gt;"",G139=""),"Falta el peso del ovillo",IF(AND(A139="",B139=""),"Falta la categoría",IF(AND(A139="",I139=""),"Falta cómo se vende",IF(AND(K139&lt;&gt;"",N139="",M139=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="11" t="n"/>
+      <c r="B140" s="6" t="n"/>
+      <c r="C140" s="6" t="n"/>
+      <c r="D140" s="6" t="n"/>
+      <c r="E140" s="6" t="n"/>
+      <c r="F140" s="6" t="n"/>
+      <c r="G140" s="6" t="n"/>
+      <c r="H140" s="6" t="n"/>
+      <c r="I140" s="6" t="n"/>
+      <c r="J140" s="6" t="n"/>
+      <c r="K140" s="7" t="n"/>
+      <c r="L140" s="8" t="n"/>
+      <c r="M140" s="6" t="n"/>
+      <c r="N140" s="6" t="n"/>
+      <c r="O140" s="9" t="n"/>
+      <c r="P140" s="6" t="n"/>
+      <c r="Q140" s="6" t="n"/>
+      <c r="R140" s="6" t="n"/>
+      <c r="S140" s="6" t="n"/>
+      <c r="T140">
+        <f>IF(C140="","",IF(AND(K140&lt;&gt;"",L140=""),"Falta el costo",IF(AND(LEFT(I140,6)="Por ov",K140&lt;&gt;"",G140=""),"Falta el peso del ovillo",IF(AND(A140="",B140=""),"Falta la categoría",IF(AND(A140="",I140=""),"Falta cómo se vende",IF(AND(K140&lt;&gt;"",N140="",M140=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="11" t="n"/>
+      <c r="B141" s="6" t="n"/>
+      <c r="C141" s="6" t="n"/>
+      <c r="D141" s="6" t="n"/>
+      <c r="E141" s="6" t="n"/>
+      <c r="F141" s="6" t="n"/>
+      <c r="G141" s="6" t="n"/>
+      <c r="H141" s="6" t="n"/>
+      <c r="I141" s="6" t="n"/>
+      <c r="J141" s="6" t="n"/>
+      <c r="K141" s="7" t="n"/>
+      <c r="L141" s="8" t="n"/>
+      <c r="M141" s="6" t="n"/>
+      <c r="N141" s="6" t="n"/>
+      <c r="O141" s="9" t="n"/>
+      <c r="P141" s="6" t="n"/>
+      <c r="Q141" s="6" t="n"/>
+      <c r="R141" s="6" t="n"/>
+      <c r="S141" s="6" t="n"/>
+      <c r="T141">
+        <f>IF(C141="","",IF(AND(K141&lt;&gt;"",L141=""),"Falta el costo",IF(AND(LEFT(I141,6)="Por ov",K141&lt;&gt;"",G141=""),"Falta el peso del ovillo",IF(AND(A141="",B141=""),"Falta la categoría",IF(AND(A141="",I141=""),"Falta cómo se vende",IF(AND(K141&lt;&gt;"",N141="",M141=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="11" t="n"/>
+      <c r="B142" s="6" t="n"/>
+      <c r="C142" s="6" t="n"/>
+      <c r="D142" s="6" t="n"/>
+      <c r="E142" s="6" t="n"/>
+      <c r="F142" s="6" t="n"/>
+      <c r="G142" s="6" t="n"/>
+      <c r="H142" s="6" t="n"/>
+      <c r="I142" s="6" t="n"/>
+      <c r="J142" s="6" t="n"/>
+      <c r="K142" s="7" t="n"/>
+      <c r="L142" s="8" t="n"/>
+      <c r="M142" s="6" t="n"/>
+      <c r="N142" s="6" t="n"/>
+      <c r="O142" s="9" t="n"/>
+      <c r="P142" s="6" t="n"/>
+      <c r="Q142" s="6" t="n"/>
+      <c r="R142" s="6" t="n"/>
+      <c r="S142" s="6" t="n"/>
+      <c r="T142">
+        <f>IF(C142="","",IF(AND(K142&lt;&gt;"",L142=""),"Falta el costo",IF(AND(LEFT(I142,6)="Por ov",K142&lt;&gt;"",G142=""),"Falta el peso del ovillo",IF(AND(A142="",B142=""),"Falta la categoría",IF(AND(A142="",I142=""),"Falta cómo se vende",IF(AND(K142&lt;&gt;"",N142="",M142=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="11" t="n"/>
+      <c r="B143" s="6" t="n"/>
+      <c r="C143" s="6" t="n"/>
+      <c r="D143" s="6" t="n"/>
+      <c r="E143" s="6" t="n"/>
+      <c r="F143" s="6" t="n"/>
+      <c r="G143" s="6" t="n"/>
+      <c r="H143" s="6" t="n"/>
+      <c r="I143" s="6" t="n"/>
+      <c r="J143" s="6" t="n"/>
+      <c r="K143" s="7" t="n"/>
+      <c r="L143" s="8" t="n"/>
+      <c r="M143" s="6" t="n"/>
+      <c r="N143" s="6" t="n"/>
+      <c r="O143" s="9" t="n"/>
+      <c r="P143" s="6" t="n"/>
+      <c r="Q143" s="6" t="n"/>
+      <c r="R143" s="6" t="n"/>
+      <c r="S143" s="6" t="n"/>
+      <c r="T143">
+        <f>IF(C143="","",IF(AND(K143&lt;&gt;"",L143=""),"Falta el costo",IF(AND(LEFT(I143,6)="Por ov",K143&lt;&gt;"",G143=""),"Falta el peso del ovillo",IF(AND(A143="",B143=""),"Falta la categoría",IF(AND(A143="",I143=""),"Falta cómo se vende",IF(AND(K143&lt;&gt;"",N143="",M143=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="11" t="n"/>
+      <c r="B144" s="6" t="n"/>
+      <c r="C144" s="6" t="n"/>
+      <c r="D144" s="6" t="n"/>
+      <c r="E144" s="6" t="n"/>
+      <c r="F144" s="6" t="n"/>
+      <c r="G144" s="6" t="n"/>
+      <c r="H144" s="6" t="n"/>
+      <c r="I144" s="6" t="n"/>
+      <c r="J144" s="6" t="n"/>
+      <c r="K144" s="7" t="n"/>
+      <c r="L144" s="8" t="n"/>
+      <c r="M144" s="6" t="n"/>
+      <c r="N144" s="6" t="n"/>
+      <c r="O144" s="9" t="n"/>
+      <c r="P144" s="6" t="n"/>
+      <c r="Q144" s="6" t="n"/>
+      <c r="R144" s="6" t="n"/>
+      <c r="S144" s="6" t="n"/>
+      <c r="T144">
+        <f>IF(C144="","",IF(AND(K144&lt;&gt;"",L144=""),"Falta el costo",IF(AND(LEFT(I144,6)="Por ov",K144&lt;&gt;"",G144=""),"Falta el peso del ovillo",IF(AND(A144="",B144=""),"Falta la categoría",IF(AND(A144="",I144=""),"Falta cómo se vende",IF(AND(K144&lt;&gt;"",N144="",M144=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="11" t="n"/>
+      <c r="B145" s="6" t="n"/>
+      <c r="C145" s="6" t="n"/>
+      <c r="D145" s="6" t="n"/>
+      <c r="E145" s="6" t="n"/>
+      <c r="F145" s="6" t="n"/>
+      <c r="G145" s="6" t="n"/>
+      <c r="H145" s="6" t="n"/>
+      <c r="I145" s="6" t="n"/>
+      <c r="J145" s="6" t="n"/>
+      <c r="K145" s="7" t="n"/>
+      <c r="L145" s="8" t="n"/>
+      <c r="M145" s="6" t="n"/>
+      <c r="N145" s="6" t="n"/>
+      <c r="O145" s="9" t="n"/>
+      <c r="P145" s="6" t="n"/>
+      <c r="Q145" s="6" t="n"/>
+      <c r="R145" s="6" t="n"/>
+      <c r="S145" s="6" t="n"/>
+      <c r="T145">
+        <f>IF(C145="","",IF(AND(K145&lt;&gt;"",L145=""),"Falta el costo",IF(AND(LEFT(I145,6)="Por ov",K145&lt;&gt;"",G145=""),"Falta el peso del ovillo",IF(AND(A145="",B145=""),"Falta la categoría",IF(AND(A145="",I145=""),"Falta cómo se vende",IF(AND(K145&lt;&gt;"",N145="",M145=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="11" t="n"/>
+      <c r="B146" s="6" t="n"/>
+      <c r="C146" s="6" t="n"/>
+      <c r="D146" s="6" t="n"/>
+      <c r="E146" s="6" t="n"/>
+      <c r="F146" s="6" t="n"/>
+      <c r="G146" s="6" t="n"/>
+      <c r="H146" s="6" t="n"/>
+      <c r="I146" s="6" t="n"/>
+      <c r="J146" s="6" t="n"/>
+      <c r="K146" s="7" t="n"/>
+      <c r="L146" s="8" t="n"/>
+      <c r="M146" s="6" t="n"/>
+      <c r="N146" s="6" t="n"/>
+      <c r="O146" s="9" t="n"/>
+      <c r="P146" s="6" t="n"/>
+      <c r="Q146" s="6" t="n"/>
+      <c r="R146" s="6" t="n"/>
+      <c r="S146" s="6" t="n"/>
+      <c r="T146">
+        <f>IF(C146="","",IF(AND(K146&lt;&gt;"",L146=""),"Falta el costo",IF(AND(LEFT(I146,6)="Por ov",K146&lt;&gt;"",G146=""),"Falta el peso del ovillo",IF(AND(A146="",B146=""),"Falta la categoría",IF(AND(A146="",I146=""),"Falta cómo se vende",IF(AND(K146&lt;&gt;"",N146="",M146=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="11" t="n"/>
+      <c r="B147" s="6" t="n"/>
+      <c r="C147" s="6" t="n"/>
+      <c r="D147" s="6" t="n"/>
+      <c r="E147" s="6" t="n"/>
+      <c r="F147" s="6" t="n"/>
+      <c r="G147" s="6" t="n"/>
+      <c r="H147" s="6" t="n"/>
+      <c r="I147" s="6" t="n"/>
+      <c r="J147" s="6" t="n"/>
+      <c r="K147" s="7" t="n"/>
+      <c r="L147" s="8" t="n"/>
+      <c r="M147" s="6" t="n"/>
+      <c r="N147" s="6" t="n"/>
+      <c r="O147" s="9" t="n"/>
+      <c r="P147" s="6" t="n"/>
+      <c r="Q147" s="6" t="n"/>
+      <c r="R147" s="6" t="n"/>
+      <c r="S147" s="6" t="n"/>
+      <c r="T147">
+        <f>IF(C147="","",IF(AND(K147&lt;&gt;"",L147=""),"Falta el costo",IF(AND(LEFT(I147,6)="Por ov",K147&lt;&gt;"",G147=""),"Falta el peso del ovillo",IF(AND(A147="",B147=""),"Falta la categoría",IF(AND(A147="",I147=""),"Falta cómo se vende",IF(AND(K147&lt;&gt;"",N147="",M147=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="11" t="n"/>
+      <c r="B148" s="6" t="n"/>
+      <c r="C148" s="6" t="n"/>
+      <c r="D148" s="6" t="n"/>
+      <c r="E148" s="6" t="n"/>
+      <c r="F148" s="6" t="n"/>
+      <c r="G148" s="6" t="n"/>
+      <c r="H148" s="6" t="n"/>
+      <c r="I148" s="6" t="n"/>
+      <c r="J148" s="6" t="n"/>
+      <c r="K148" s="7" t="n"/>
+      <c r="L148" s="8" t="n"/>
+      <c r="M148" s="6" t="n"/>
+      <c r="N148" s="6" t="n"/>
+      <c r="O148" s="9" t="n"/>
+      <c r="P148" s="6" t="n"/>
+      <c r="Q148" s="6" t="n"/>
+      <c r="R148" s="6" t="n"/>
+      <c r="S148" s="6" t="n"/>
+      <c r="T148">
+        <f>IF(C148="","",IF(AND(K148&lt;&gt;"",L148=""),"Falta el costo",IF(AND(LEFT(I148,6)="Por ov",K148&lt;&gt;"",G148=""),"Falta el peso del ovillo",IF(AND(A148="",B148=""),"Falta la categoría",IF(AND(A148="",I148=""),"Falta cómo se vende",IF(AND(K148&lt;&gt;"",N148="",M148=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="11" t="n"/>
+      <c r="B149" s="6" t="n"/>
+      <c r="C149" s="6" t="n"/>
+      <c r="D149" s="6" t="n"/>
+      <c r="E149" s="6" t="n"/>
+      <c r="F149" s="6" t="n"/>
+      <c r="G149" s="6" t="n"/>
+      <c r="H149" s="6" t="n"/>
+      <c r="I149" s="6" t="n"/>
+      <c r="J149" s="6" t="n"/>
+      <c r="K149" s="7" t="n"/>
+      <c r="L149" s="8" t="n"/>
+      <c r="M149" s="6" t="n"/>
+      <c r="N149" s="6" t="n"/>
+      <c r="O149" s="9" t="n"/>
+      <c r="P149" s="6" t="n"/>
+      <c r="Q149" s="6" t="n"/>
+      <c r="R149" s="6" t="n"/>
+      <c r="S149" s="6" t="n"/>
+      <c r="T149">
+        <f>IF(C149="","",IF(AND(K149&lt;&gt;"",L149=""),"Falta el costo",IF(AND(LEFT(I149,6)="Por ov",K149&lt;&gt;"",G149=""),"Falta el peso del ovillo",IF(AND(A149="",B149=""),"Falta la categoría",IF(AND(A149="",I149=""),"Falta cómo se vende",IF(AND(K149&lt;&gt;"",N149="",M149=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="11" t="n"/>
+      <c r="B150" s="6" t="n"/>
+      <c r="C150" s="6" t="n"/>
+      <c r="D150" s="6" t="n"/>
+      <c r="E150" s="6" t="n"/>
+      <c r="F150" s="6" t="n"/>
+      <c r="G150" s="6" t="n"/>
+      <c r="H150" s="6" t="n"/>
+      <c r="I150" s="6" t="n"/>
+      <c r="J150" s="6" t="n"/>
+      <c r="K150" s="7" t="n"/>
+      <c r="L150" s="8" t="n"/>
+      <c r="M150" s="6" t="n"/>
+      <c r="N150" s="6" t="n"/>
+      <c r="O150" s="9" t="n"/>
+      <c r="P150" s="6" t="n"/>
+      <c r="Q150" s="6" t="n"/>
+      <c r="R150" s="6" t="n"/>
+      <c r="S150" s="6" t="n"/>
+      <c r="T150">
+        <f>IF(C150="","",IF(AND(K150&lt;&gt;"",L150=""),"Falta el costo",IF(AND(LEFT(I150,6)="Por ov",K150&lt;&gt;"",G150=""),"Falta el peso del ovillo",IF(AND(A150="",B150=""),"Falta la categoría",IF(AND(A150="",I150=""),"Falta cómo se vende",IF(AND(K150&lt;&gt;"",N150="",M150=""),"(opcional) sin proveedor","OK"))))))</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:S75"/>
+  <conditionalFormatting sqref="T2:T150">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(LEFT(T2,5)="Falta")</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>T2="OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="6">
-    <dataValidation sqref="B2:B75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B150" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>=Listas!$A$1:$A$10</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I150" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>=Listas!$C$1:$C$2</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J150" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>=Listas!$D$1:$D$2</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M150" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Listas!$B$1:$B$4</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:L75 Q2:Q75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Número" error="Escribe un número (sin puntos ni signos)." type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="K2:L150 Q2:Q150" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Número" error="Escribe un número (sin puntos ni signos)." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Escribe una fecha (DD/MM/AAAA)." type="date" operator="greaterThan">
+    <dataValidation sqref="O2:O150" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Escribe una fecha (DD/MM/AAAA)." type="date" operator="greaterThan">
       <formula1>45658</formula1>
     </dataValidation>
   </dataValidations>
@@ -3768,7 +6147,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>